<commit_message>
Excel of the whole site: final stories and reviewed Hebrew
All 14 stories (12 products, Home, Catalog) passed the marketing and
fact critics; the 30 new strings passed a translator and two Hebrew
reviewers. Unresolved keys: 0. The status column is dropped now that no
page is in review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/MITODERM-3D-story.xlsx
+++ b/mitoderm-catalog/site/MITODERM-3D-story.xlsx
@@ -438,22 +438,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -464,60 +463,55 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Статус</t>
+          <t>Slug</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Slug</t>
+          <t>Линейка</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Линейка</t>
+          <t>Назначение</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Назначение</t>
+          <t>Цветовое окружение</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Цветовое окружение</t>
+          <t>Экран с оттенком серии</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Экран с оттенком серии</t>
+          <t>Герой-объект</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Герой-объект</t>
+          <t>Сюжет одной строкой</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Сюжет одной строкой</t>
+          <t>Метки специалистов</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Метки специалистов</t>
+          <t>Фото заказчика (№ в коллаже)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Фото заказчика (№ в коллаже)</t>
+          <t>Новых строк</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Новых строк</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Вопросов</t>
         </is>
@@ -531,56 +525,51 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>v-tech-system</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>v-tech-system</t>
+          <t>V-TECH FACE</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>V-TECH FACE</t>
+          <t>professional</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>professional</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
           <t>Линейка V-TECH FACE: чёрный с золотом. Фон бренда #0a0a0b. Дальний слой — медленный золотой дым и золотые искры: золото #c9a24b, светлое #d8bd7e, глубокое #9c7a2f. Весь слой поворачивается за курсором. За коробкой — узкое тёплое золотое свечение. Своей «капли» у V-TECH нет, поэтому по правилу акцент несёт цвет линейки. Янтарь флаконов и золото фольги — цвета самих упаковок, страницу в них не красим. Плоскость кожи тёплая и тёмная, её освещает золото линейки, нового цвета она не вводит. Коробка в зеркальной фольге отражает дальний слой, так что окружение видно и в самом герое. Страница чёрная, поэтому ставим белый логотип, а не монограмму M. Цветов других линеек на странице нет: финиш EXOCELL MASK и DERMA RECOVERY CREAM дан чипами-ссылками в цветах страницы, без бирюзы MASK, без зелени BIOSPICULE и без 3D-объектов. Самое яркое золото дыма — на экране 4, это сияние результата. Цвет V-TECH FACE совпадает с базой бренда и с линейкой HAIR, поэтому серию называет бейдж: тройка бейджей образца MASK (ui.line_mark, ui.line_name, home.tg) стоит на экране 1 и повторяется на экране 7.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="F2" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Высокая коробка в зеркальной золотой фольге с чёрными полосами сверху и снизу. На фасаде серебряное VM, большой чёрный знак V с треугольником и V-TECH / S Y S T E M. Внутри чёрный ложемент (фото заказчика №44, Figma 113:8161): саше гель-маски из золотой фольги лежат плашмя (на фото видно верхнее), пять янтарных флаконов стоят в гнёздах. В наборе 5 флаконов сыворотки и 5 саше гель-маски.</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Высокая коробка в зеркальной золотой фольге с чёрными полосами сверху и снизу. На фасаде серебряное VM, большой чёрный знак V с треугольником и V-TECH / S Y S T E M. Внутри чёрный ложемент (фото заказчика №44, Figma 113:8161): саше гель-маски из золотой фольги лежат плашмя (на фото видно верхнее), пять янтарных флаконов стоят в гнёздах. В наборе 5 флаконов сыворотки и 5 саше гель-маски.</t>
+          <t>Зеркальная золотая коробка ложится и открывает чёрный ложемент, из гнёзд поднимаются пять янтарных флаконов, капля сыворотки с экзосомами уходит в открытые иглами микроканалы, золотое саше кладёт поверх слой геля без смывания, и рельеф кожи под ним выравнивается; в коробке пять флаконов и пять саше, курс — не меньше четырёх процедур раз в две недели.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Зеркальная золотая коробка ложится и открывает чёрный ложемент, из гнёзд поднимаются пять янтарных флаконов, капля сыворотки с экзосомами уходит в открытые иглами микроканалы, золотое саше кладёт поверх слой геля без смывания, и рельеф кожи под ним выравнивается; в коробке пять флаконов и пять саше, курс — не меньше четырёх процедур раз в две недели.</t>
+          <t>פנים</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>פנים</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
           <t>40, 42, 44–50, 53, 54, 60, 78–80, 82, 83</t>
         </is>
       </c>
+      <c r="K2" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" s="2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -592,56 +581,51 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>exo-nad</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>exo-nad</t>
+          <t>PEELING</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>PEELING</t>
+          <t>professional</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>professional</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
           <t>Линейка PEELING по правилу «лицо / волосы / пилинг — чёрное с золотом». Фон — база бренда #0a0a0b, поверхности #111114 / #1a1a1f, текст крем #f6f3ec. Цвет линейки по таблице палитры — шампань-золото #d8c48a. Им окрашены дым и свечение дальнего слоя, свечение за коробкой и бейдж линейки. Частицы фона — мелкие шампань-золотые искры самого фона, а не хлопья из флакона: хлопья остаются внутри стекла, потому что золота нет в cat.ingredients. На экране 2 искры тускнеют до серо-бежевой матовой пыли, на экране 4 ложатся ровной вуалью. Волосяные линии, кикеры, выносные линии, линия шагов, подсветка гнёзд ложемента и кнопка цены — золото бренда #c9a24b (светлое #d8bd7e). Своей капли у EXO-NAD в правилах нет, поэтому работает цвет линейки. Янтарь и голубизна есть только на самих флаконах. Бирюзового дыма и свечения нет: это окружение MASK, а два цвета линеек на одной странице запрещены. Чёрный ложемент с золотой печатью (фото заказчика 29) сам лежит в этой гамме. Страница чёрная, поэтому логотип белый; монограммы M нет, она для BIOSPICULE. Бейдж линейки: без рамки и без заливки, текст PEELING цветом #d8c48a с маленькой шампань-точкой впереди, отделён промежутком от залитого золотом «מקצועי». Золотой контур не используется: он означает «טיפוח ביתי». Бейдж одинаковый на экранах 1 и 7. Оттенок серии впервые появляется на экране 1 (шампань-свечение за коробкой и бейдж PEELING), на экране 7 повторяется и становится сильнее всего.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="F3" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Квадратная коробка EXO-NAD из брашированного золота. Крышка поднимается прямо вверх, как на фото заказчика 26 и 32, и открывает чёрный ложемент (фото 29). Слева в высоком гнезде стоит флакон пилинга с золотым колпачком, в верхнем ряду — 5 флаконов pH Normalizer, в нижнем — 5 флаконов Longevity Serum. На самом ложементе золотом напечатаны шаги ① EXO-NAD PEELING, ② PH NORMALIZER, ③ LONGEVITY SERUM. Для экранов 3–5 используются отдельные модели, по одной каждого вида: флакон пилинга, флакон pH Normalizer и флакон Longevity Serum.</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Квадратная коробка EXO-NAD из брашированного золота. Крышка поднимается прямо вверх, как на фото заказчика 26 и 32, и открывает чёрный ложемент (фото 29). Слева в высоком гнезде стоит флакон пилинга с золотым колпачком, в верхнем ряду — 5 флаконов pH Normalizer, в нижнем — 5 флаконов Longevity Serum. На самом ложементе золотом напечатаны шаги ① EXO-NAD PEELING, ② PH NORMALIZER, ③ LONGEVITY SERUM. Для экранов 3–5 используются отдельные модели, по одной каждого вида: флакон пилинга, флакон pH Normalizer и флакон Longevity Serum.</t>
+          <t>Закрытая золотая коробка стоит в тусклой пыли, из-за неё по порядку выходят три жидкости одного визита, их общий свет превращает пыль в ровное шампань-сияние, а в конце крышка поднимается, как на фото заказчика, и показывает ложемент с напечатанными шагами 1-2-3: 1 флакон и 5 + 5 флаконов.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Закрытая золотая коробка стоит в тусклой пыли, из-за неё по порядку выходят три жидкости одного визита, их общий свет превращает пыль в ровное шампань-сияние, а в конце крышка поднимается, как на фото заказчика, и показывает ложемент с напечатанными шагами 1-2-3: 1 флакон и 5 + 5 флаконов.</t>
+          <t>פנים</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>פנים</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
           <t>26–32, 35, 39, 51, 63, 64, 84</t>
         </is>
       </c>
+      <c r="K3" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="L3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M3" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -653,58 +637,53 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>exocell-mask</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>exocell-mask</t>
+          <t>V-TECH FACE</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>V-TECH FACE</t>
+          <t>professional</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>professional</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
           <t>MASK — исключение из правила линейки: вместо чёрно-золотого окружения V-TECH FACE у неё своё бирюзово-синее. Фон страницы — база бренда #0a0a0b. Дальний слой: медленный бирюзовый дым (EXOCELL #6fb7ba, фасад коробки #5ca0a5) и редкие светлые частицы, вместе поворачиваются за указателем. Передний план: прозрачные бирюзовые капли сыворотки, слои маски #dcf0f5 и бледно-голубой. Золото бренда #c9a24b — только волосяные линии кикеров, бейдж «מקצועי» (home.tg, золотая заливка) и кнопка цены. Чипы-ссылки на другие средства (экраны 2 и 6) — кремовый контур #f6f3ec, не золото: на шаге «зачем» они не должны выглядеть главным действием. Оттенок серии: бейдж line.mark «V-TECH FACE» на экране 1, а на экране 7 за карточкой «что внутри» горит тёплое золотое свечение V-TECH FACE (эллипс ~900 px) и стоит бейдж линейки, чтобы посетитель видел серию. Зелёный BIOSPICULE не смешивается; бирюза капли не заливает плоскости сверх окружения.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="F4" s="2" t="n">
         <v>7</v>
       </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Коробка EXOCELL MASK — тёмно-бирюзовый портретный картон (#5ca0a5) с тёмно-синей печатью, версия «Your Second Skin» (как на пакшоте и на утверждённом 03-mirror). Кубоид: фасад site/img/exocell-box-front.jpg и левая боковина site/img/exocell-box-side.jpg, обе выпрямлены из protocols/assets/img/exocell-mask.webp. Правая грань, верх, низ и оборот — гладкий #5ca0a5 без печати (их печать неизвестна). Ракурс как на пакшоте: коробка повёрнута вправо, видна левая боковина.</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Коробка EXOCELL MASK — тёмно-бирюзовый портретный картон (#5ca0a5) с тёмно-синей печатью, версия «Your Second Skin» (как на пакшоте и на утверждённом 03-mirror). Кубоид: фасад site/img/exocell-box-front.jpg и левая боковина site/img/exocell-box-side.jpg, обе выпрямлены из protocols/assets/img/exocell-mask.webp. Правая грань, верх, низ и оборот — гладкий #5ca0a5 без печати (их печать неизвестна). Ракурс как на пакшоте: коробка повёрнута вправо, видна левая боковина.</t>
+          <t>Коробка EXOCELL MASK среди капель сыворотки открывается, из неё поднимается двойная маска из биоцеллюлозы и ложится на лицо; потом из коробки разлетаются все пять саше, поверх встают три коротких шага протокола, и всё собирается в экран покупки с тёплым золотом линейки V-TECH FACE.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Коробка EXOCELL MASK среди капель сыворотки открывается, из неё поднимается двойная маска из биоцеллюлозы и ложится на лицо; потом из коробки разлетаются все пять саше, поверх встают три коротких шага протокола, и всё собирается в экран покупки с тёплым золотом линейки V-TECH FACE.</t>
+          <t>פנים</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>פנים</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
           <t>11–24 (саше, двойная маска, нанесение)</t>
         </is>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>7</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M4" s="2" t="n">
-        <v>7</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -714,56 +693,51 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>exosignal-hair</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>exosignal-hair</t>
+          <t>HAIR</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>HAIR</t>
+          <t>professional</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>professional</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
           <t>Линейка HAIR: чёрный и золото. По design-rules.md это тот же цвет, что у V-TECH FACE и у базы бренда. Фон #0a0a0b, тёплый золотой дым малой плотности (#9c7a2f → #c9a24b), золотые частицы #d8bd7e, свечение за коробкой #c9a24b. Капли цвета нет: жидкость в ампулах бесцветная (это видно на пакшоте), поэтому работает цвет линейки (правило «Капля средства»). Стекло ампул даёт только холодный белый блик. Проблема на экране 2 показана тусклым кремово-серым (#f6f3ec, прозрачность около 30%). Золото включается только там, где начинается решение. MITOSCAN и MITOPEN стоят в холодном нейтральном свете своих материалов, без золотой подсветки и без окружения DEVICES: смешивать на одной странице цвета двух линеек нельзя. Золото HAIR совпадает с базой, поэтому оттенок серии передаётся контрастом, а не цветом всей страницы. На экране 5 дым почти гаснет, устройства приглушены, и тёплое золотое пятно остаётся только под ампулой и флаконом EXOSIGNAL SPRAY (оба средства линейки HAIR). Над ними стоит бейдж линейки line.mark. Тот же бейдж есть в ряду бейджей на экранах 1 и 7. Это штатное окружение линейки, а не исключение, как у MASK.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="F5" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Стеклянная ампула EXOSIGNAL HAIR на 5 мл: прозрачное стекло, бесцветная жидкость, белое кольцо на горлышке. Крупная вертикальная надпись 'EXOSIGNAL' ('EXO' жирным), рядом мелкие вертикальные строки: 'EXOSIGNAL HAIR', 'Siero nutriente per il cuoio capelluto' и другие, нечитаемые. На обороте тоже есть печать, сквозь стекло она видна зеркально. Ампула стоит на фоне плоской матово-чёрной коробки с золотыми 'EXOSIGNAL' / 'H A I R'.</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Стеклянная ампула EXOSIGNAL HAIR на 5 мл: прозрачное стекло, бесцветная жидкость, белое кольцо на горлышке. Крупная вертикальная надпись 'EXOSIGNAL' ('EXO' жирным), рядом мелкие вертикальные строки: 'EXOSIGNAL HAIR', 'Siero nutriente per il cuoio capelluto' и другие, нечитаемые. На обороте тоже есть печать, сквозь стекло она видна зеркально. Ампула стоит на фоне плоской матово-чёрной коробки с золотыми 'EXOSIGNAL' / 'H A I R'.</t>
+          <t>Из чёрной коробки выходит одна ампула; на фоне тусклых падающих нитей золотой прицел измерения задаёт точку отсчёта; у ампулы отламывается горлышко, и капля становится экзосомой с PDRN и восемью пептидами; из кожи головы вырастают четыре золотые пряди; путь «измерить → открыть → доставить → дома» отмечен золотом линейки HAIR; в конце пять запечатанных ампул, пять сеансов, собираются в одну коробку.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Из чёрной коробки выходит одна ампула; на фоне тусклых падающих нитей золотой прицел измерения задаёт точку отсчёта; у ампулы отламывается горлышко, и капля становится экзосомой с PDRN и восемью пептидами; из кожи головы вырастают четыре золотые пряди; путь «измерить → открыть → доставить → дома» отмечен золотом линейки HAIR; в конце пять запечатанных ампул, пять сеансов, собираются в одну коробку.</t>
+          <t>קרקפת · טריכולוג/ית</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>קרקפת · טריכולוג/ית</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
           <t>36, 47, 55, 58</t>
         </is>
       </c>
+      <c r="K5" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="L5" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="M5" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -775,56 +749,51 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>exosignal-spray</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>exosignal-spray</t>
+          <t>HAIR</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>HAIR</t>
+          <t>home care</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>home care</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
           <t>Линейка HAIR: чёрный фон #0a0a0b и золото #c9a24b (светлое #d8bd7e, глубокое #9c7a2f). Дальний слой — медленный тёплый золотисто-коричневый дым и золотые частицы на чёрном, он поворачивается за курсором. Туман спрея — матово-белые капли: это цвет самого стекла, а не отдельный цвет. Своей «капли» у спрея нет, поэтому работает цвет линейки (правило палитры). Серебро #d9d4cc из старого site/prompts/exosignal-spray.md не используем: это цвет линейки DEVICES, а два цвета линеек на одной странице смешивать запрещено. Исключением, как MASK, страница не является. Цвет HAIR совпадает с базой бренда и с V-TECH FACE, поэтому одним цветом серию не показать. Серию обозначает знак: пара бейджей ui.line_mark «HAIR» + ui.line_name рядом с ui.use_home «טיפוח ביתי» (золотой контур) на экранах 1, 2 и 7, а на экране 2 — пакшот EXOSIGNAL HAIR, на котором читается надпись, с подписью b6.label4. Самый яркий золотой контровой свет на странице бывает только на экране 7.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="F6" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Флакон-спрей EXOSIGNAL SPRAY HOME на 15 мл: цилиндр из матового полупрозрачного стекла, золотой металлический рифлёный колпачок, вертикальная надпись EXOSIGNAL. Колпачок надет на всех экранах: распылитель под ним не снят на фото. Второй объект — высокая матовая чёрная коробка с золотой и белой печатью. Знак линейки — пакшот EXOSIGNAL HAIR в глубине на экранах 2 и 5.</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Флакон-спрей EXOSIGNAL SPRAY HOME на 15 мл: цилиндр из матового полупрозрачного стекла, золотой металлический рифлёный колпачок, вертикальная надпись EXOSIGNAL. Колпачок надет на всех экранах: распылитель под ним не снят на фото. Второй объект — высокая матовая чёрная коробка с золотой и белой печатью. Знак линейки — пакшот EXOSIGNAL HAIR в глубине на экранах 2 и 5.</t>
+          <t>Матовый стеклянный флакон с золотым колпачком выходит из тени своей чёрной коробки и превращается в золотую нить между двумя визитами EXOSIGNAL HAIR; облачко тумана, входящее в кадр сверху, решает три задачи и ложится на проборы без смывания, а в конце флакон возвращается к своей коробке на экране покупки.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Матовый стеклянный флакон с золотым колпачком выходит из тени своей чёрной коробки и превращается в золотую нить между двумя визитами EXOSIGNAL HAIR; облачко тумана, входящее в кадр сверху, решает три задачи и ложится на проборы без смывания, а в конце флакон возвращается к своей коробке на экране покупки.</t>
+          <t>קרקפת · טריכולוג/ית</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>קרקפת · טריכולוג/ית</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
           <t>2, 3, 21, 33, 34, 41, 43, 59, 65</t>
         </is>
       </c>
+      <c r="K6" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="L6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M6" s="2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -836,56 +805,51 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>exotech-gel</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>exotech-gel</t>
+          <t>V-TECH FACE</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>V-TECH FACE</t>
+          <t>home care</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>home care</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
           <t>Линейка V-TECH FACE, поэтому чёрный с золотом. Фон #0a0a0b. Дальний слой — медленный тёплый дым от #0a0a0b к глубокому золоту #9c7a2f с бликами #c9a24b и частицами-пылинками #d8bd7e; слой поворачивается за указателем. За упаковкой узкое золотое свечение. Своей «капли» у средства нет: упаковка сама золотая, поэтому работает золото линейки. На объектах остаётся собственное, более жёлтое золото фольги с пакшота, брендовым золотом его не подменяем. Свет на предметах и фон разделены. Куб и сфера отражают отдельную тёплую студийную карту окружения с 2–3 крупными софтбоксами: блики сверху слева и справа, как на фото. Дым рендерится только фоном и подмешивается в отражения слабым слоем, поэтому дым только тёплый, без холодных и зелёных оттенков. У фасада куба roughness около 0,35–0,5. Проверка до сборки: один тестовый рендер экрана 1, на котором надписи EXOTECH / GEL на кубе и на сфере читаются на чёрном фоне. На экране 5 BIOSPICULE упоминается только текстом, без зелёного цвета: смешивать цвета линеек запрещено. Логотип белый, так как страница чёрная. Назначение показывает бейдж «טיפוח ביתי» (b0.label1) с золотым контуром, а не цвет фона. Элемент серии (line.mark «V-TECH FACE» с мелкой подписью «סדרת האקסוזומים הסינתטיים») стоит кикером на экране 1 и повторяется на экране 7. На экране 7 золото за упаковками разгорается теплее.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="F7" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Золотая полированная сфера-банка EXOTECH GEL, 30 мл. Крышка — верхняя полусфера со всей надписью: 'EXOTECH' ('EXO' жирным, 'TECH' тонким) и под ним курсив с разрядкой 'GEL'. Шов — экватор. Пакшот снят чуть сверху, поэтому спереди шов проходит под 'GEL'. Основание — гладкое золото без печати. Рядом её внешняя упаковка — зеркально-золотой куб с чёрной левой гранью и золотым диагональным клином.</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Золотая полированная сфера-банка EXOTECH GEL, 30 мл. Крышка — верхняя полусфера со всей надписью: 'EXOTECH' ('EXO' жирным, 'TECH' тонким) и под ним курсив с разрядкой 'GEL'. Шов — экватор. Пакшот снят чуть сверху, поэтому спереди шов проходит под 'GEL'. Основание — гладкое золото без печати. Рядом её внешняя упаковка — зеркально-золотой куб с чёрной левой гранью и золотым диагональным клином.</t>
+          <t>Золотая сфера выходит вперёд от своего зеркального куба, приподнимает крышку со всей надписью над светящейся щелью и выпускает пять капель активов; капли сливаются в невесомую плёнку, которая ложится на зрителя, а свет обходит сферу от утра до вечера — протокол клиники каждый день продолжается дома.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Золотая сфера выходит вперёд от своего зеркального куба, приподнимает крышку со всей надписью над светящейся щелью и выпускает пять капель активов; капли сливаются в невесомую плёнку, которая ложится на зрителя, а свет обходит сферу от утра до вечера — протокол клиники каждый день продолжается дома.</t>
+          <t>פנים</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>פנים</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
           <t>37, 38, 52</t>
         </is>
       </c>
+      <c r="K7" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="L7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M7" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -897,56 +861,51 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>micro-boost-10</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>micro-boost-10</t>
+          <t>BIOSPICULE</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>BIOSPICULE</t>
+          <t>professional</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>professional</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
           <t>Окружение линейки BIOSPICULE (design-rules, «палитра по линейкам»: BIOSPICULE = зелёный). Дым #1E4634 на тёмном #12382A уходит в чёрный бренда #0a0a0b. Золото бренда #c9a24b (светлое #d8bd7e): волосяные линии, кикеры, кнопка цены, искры массажа, дуга-таймер, кольцо-ореол. Золотая монограмма M (site/img/mitoderm-m-gold.png) проступает в дыму. Частицы — тонкие полупрозрачные спикулы с тёмно-зелёным тоном, как на медальоне коробки, с золотыми бликами. Своей капли у MICRO BOOST нет: по design-rules у средства без своего цвета капли нет, работает цвет линейки. Мятный #4fb285 из старого промпта не используется, это капля CELL RENEW; вопрос решён в design-rules, заказчику его не задаём. Шалфей #9AA889 только на мини-коробке DERMA RECOVERY CREAM (та же линейка). Бирюзы MASK и цветов других линеек на странице нет: смешивать две линейки запрещено.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="F8" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Высокая узкая коробка цвета слоновой кости. На ней тёмно-зелёная полоса с золотым «MICRO BOOST 10%» и круглый медальон в золотом кольце: светлый прозрачно-серебристый диск с тёмно-зелёными спикулами. Перед коробкой шприц 3 мл без иглы. Коробка — настоящий пакшот-герой, шприц — модель без печати до фото.</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Высокая узкая коробка цвета слоновой кости. На ней тёмно-зелёная полоса с золотым «MICRO BOOST 10%» и круглый медальон в золотом кольце: светлый прозрачно-серебристый диск с тёмно-зелёными спикулами. Перед коробкой шприц 3 мл без иглы. Коробка — настоящий пакшот-герой, шприц — модель без печати до фото.</t>
+          <t>Рой спикул из медальона на коробке сходится в шприц 3 мл. Спикулы проходят сквозь поверхность там, где пилинг останавливается. В капле они делятся на две длины и уходят на две глубины эпидермиса. Руки косметолога вмассировывают сыворотку, и спикулы могут работать до 72 часов. В конце коробка и шприц стоят на экране покупки.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Рой спикул из медальона на коробке сходится в шприц 3 мл. Спикулы проходят сквозь поверхность там, где пилинг останавливается. В капле они делятся на две длины и уходят на две глубины эпидермиса. Руки косметолога вмассировывают сыворотку, и спикулы могут работать до 72 часов. В конце коробка и шприц стоят на экране покупки.</t>
+          <t>פנים</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>פנים</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
           <t>6, 67–69, 72, 74, 77</t>
         </is>
       </c>
+      <c r="K8" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="L8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M8" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -958,56 +917,51 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>cell-renew-1-5</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>cell-renew-1-5</t>
+          <t>BIOSPICULE</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>BIOSPICULE</t>
+          <t>home care</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>home care</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
           <t>Окружение линейки BIOSPICULE: по правилу цвет линейки — главный акцент. Дальний фон — медленный зелёный дым от #12382A в глубине до #1E4634 у света. Частицы — те же иглы-веретёна в малом масштабе, редкие. Фото spicules-macro.png светлое, кремовое, поэтому в фон его не ставим; оно идёт только маской яркости в тоне #12382A с непрозрачностью не выше 15% на экране 3. Золото бренда #c9a24b появляется только в пяти местах. Первое — волосяные линии: выноски, тонкий кант зеркала, взятый с печати медальона, линия массажа на экране 4. Дальше — кикеры, главная кнопка, бейдж линейки и золотая монограмма M (site/img/mitoderm-m-gold.png) на экранах 1, 5 и 7. Капля средства — мятный #4fb285, не больше ~10% площади: узкое свечение медальона, редкие искры покалывания, контровой свет за каплей, точки меток. Сама капля сыворотки бесцветная, потому что цвет сыворотки нигде не задокументирован. Назначение показывает бейдж «טיפוח ביתי» с золотым контуром, а не цвет фона. Чёрной базы V-TECH и бирюзы MASK нет. Шалфей #9AA889 — только напечатанная полоса на коробке DERMA RECOVERY CREAM на экране 5, фон им не красим. Экран с оттенком серии — 5: за рядом коробок поднимаются золотая M и бейдж линейки «BIOSPICULE™», дым густеет до #1E4634, на двух передних коробках читается напечатанное «BIOSPICULE SYSTEM».</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="F9" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Высокая узкая коробка CELL RENEW 1.5% цвета слоновой кости — куб, фасад выпрямлен из protocols/print/img/cell-renew-15.webp. На ней зелёная полоса с золотой надписью «CELL RENEW / 1.5%» и круглый медальон в зелёном кольце с тёмно-зелёными спикулами. Медальон — сквозной мотив сюжета: его кольцо становится зеркалом, и через него зритель попадает внутрь. Кольцо строим геометрией, а не растягиваем из фото.</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Высокая узкая коробка CELL RENEW 1.5% цвета слоновой кости — куб, фасад выпрямлен из protocols/print/img/cell-renew-15.webp. На ней зелёная полоса с золотой надписью «CELL RENEW / 1.5%» и круглый медальон в зелёном кольце с тёмно-зелёными спикулами. Медальон — сквозной мотив сюжета: его кольцо становится зеркалом, и через него зритель попадает внутрь. Кольцо строим геометрией, а не растягиваем из фото.</t>
+          <t>Узкая коробка CELL RENEW 1.5% встаёт в зелёном дыму, её медальон становится тусклым зеркалом с узнаваемыми проблемами кожи, через него мы попадаем в редкое облако стеклянных игл и активов, после мягкого массажа дымка на стекле редеет и оно начинает сиять, коробка встаёт в ряд линии BIOSPICULE рядом с DERMA RECOVERY CREAM и следующим шагом 2.5%, а в конце идёт экран покупки, где показано, что внутри, и есть одна кнопка «Где купить».</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Узкая коробка CELL RENEW 1.5% встаёт в зелёном дыму, её медальон становится тусклым зеркалом с узнаваемыми проблемами кожи, через него мы попадаем в редкое облако стеклянных игл и активов, после мягкого массажа дымка на стекле редеет и оно начинает сиять, коробка встаёт в ряд линии BIOSPICULE рядом с DERMA RECOVERY CREAM и следующим шагом 2.5%, а в конце идёт экран покупки, где показано, что внутри, и есть одна кнопка «Где купить».</t>
+          <t>פנים</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>פנים</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
           <t>10, 70, 75, 67–69</t>
         </is>
       </c>
+      <c r="K9" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="L9" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M9" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1019,56 +973,51 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>cellular-age-defense-2-5</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>cellular-age-defense-2-5</t>
+          <t>BIOSPICULE</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>BIOSPICULE</t>
+          <t>home care</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>home care</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
           <t>Окружение линейки BIOSPICULE зелёное. Фон #12382A, дым #1E4634, к краям он уходит в базу бренда #0a0a0b. Свечение за продуктом тоже зелёное и светлеет к центру. Частицы, нити пептидов и волосяные линии — золото бренда #c9a24b / #d8bd7e: оно повторяет золотую монограмму M и золотой текст на тёмно-зелёной полосе коробки. Своей капли у средства нет (по design-rules капля есть только у EXOCELL, CELL RENEW и MITOSCAN), поэтому акцент держит цвет линейки. Зелёный CELL RENEW #4fb285 как свечение не используем. Коробки CELL RENEW 1.5% (экран 2) и DERMA RECOVERY CREAM (экран 5; шалфейная полоса #9AA889 на её коробке) несут свой цвет только печатью, второго цвета линейки на странице нет. Шаг «Защита» — это временное потепление света, а не новый цвет. Оттенок серии показан на экране 1: глубокий зелёный, золотая монограмма M в дыму (размытая: файл — растр 600 px) и бейдж линейки. На экране 7 монограмма повторяется. Линейка и назначение передаются парой бейджей из cat.eyebrow: «סרום BIOSPICULE™» — бейдж линейки, «טיפוח ביתי» — золотой контур. Назначение цветом фона не передаём.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="F10" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Высокая узкая ивори-коробка CELLULAR AGE DEFENSE 2.5%: тёмно-зелёная полоса с золотым текстом, круглый медальон со спикулами, сверху золотая M. Это куб с фасадом из пакшота protocols/print/img/cellular-age-25.webp, поворот не больше ±20°. По умолчанию страница собирается только с коробкой. Белый airless-флакон 30 мл (фото №9 в Figma) раньше экрана 4 не появляется. Он добавляется только после ответа заказчика про печать 'CELL CELLULAR' и только на экранах 4 (крупно одна головка помпы) и 7.</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Высокая узкая ивори-коробка CELLULAR AGE DEFENSE 2.5%: тёмно-зелёная полоса с золотым текстом, круглый медальон со спикулами, сверху золотая M. Это куб с фасадом из пакшота protocols/print/img/cellular-age-25.webp, поворот не больше ±20°. По умолчанию страница собирается только с коробкой. Белый airless-флакон 30 мл (фото №9 в Figma) раньше экрана 4 не появляется. Он добавляется только после ответа заказчика про печать 'CELL CELLULAR' и только на экранах 4 (крупно одна головка помпы) и 7.</t>
+          <t>Коробка 2.5% встаёт на ступень выше CELL RENEW 1.5%, камера проходит сквозь её медальон, где через поле спикул идут пять золотых нитей пептидов, Bakuchiol и Adenosine (у 1.5% их нет), всё собирается в одну каплю, которая покалывает и требует мягких движений, а лестница ухода (2.5% → DERMA RECOVERY → дневная защита) ведёт к экрану покупки с одной коробкой 30 мл.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Коробка 2.5% встаёт на ступень выше CELL RENEW 1.5%, камера проходит сквозь её медальон, где через поле спикул идут пять золотых нитей пептидов, Bakuchiol и Adenosine (у 1.5% их нет), всё собирается в одну каплю, которая покалывает и требует мягких движений, а лестница ухода (2.5% → DERMA RECOVERY → дневная защита) ведёт к экрану покупки с одной коробкой 30 мл.</t>
+          <t>פנים</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>פנים</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
           <t>7, 9, 67–69</t>
         </is>
       </c>
+      <c r="K10" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="2" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1080,56 +1029,51 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>derma-recovery-cream</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>derma-recovery-cream</t>
+          <t>BIOSPICULE</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>BIOSPICULE</t>
+          <t>home care</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>home care</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
           <t>Зелёное окружение линейки BIOSPICULE (слово заказчика 11/10). База дальнего слоя — #12382A, дым — #1E4634. Подсветка за объектами — шалфей DERMA #9AA889: это цвет DERMA в таблице линеек и цвет полосы на коробке. Шалфей — «капля» средства, не больше ~10% площади. Он есть только у крема и барьера: свечение за банкой, лента крема, атласный слой, точки меток. Искры в дыму кремовые #f6f3ec. Иглы-спикулы на экране 2 естественного серо-оливкового цвета, как на site/img/spicules-macro.png. Шалфея в них нет, чтобы иглы не читались как часть крема. Золото бренда #c9a24b — волосяные линии, кикеры, главная кнопка, выноски. В шапке вместо белого логотипа стоит золотая монограмма M (site/img/mitoderm-m-gold.png). Оттенок серии — экран 5: дым густеет до насыщенного #1E4634, за объектами проступает крупная полупрозрачная золотая M. Исключений нет: бирюза MASK не используется. Мятный #4fb285 (капля CELL RENEW) тоже не используется, кроме печати на билборде её коробки. Золотые упаковки V-TECH и EXO-NAD в кадр не выводятся, эти средства есть только в тексте b4.line, чтобы на странице не было двух цветов линеек. Назначение показывает бейдж, а не цвет фона. Бейдж ui.use_home с золотым контуром стоит на экранах 1 и 7. У MICRO BOOST 10% на экране 5 маленький бейдж home.tg с золотой заливкой (по design-rules).</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="F11" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Матовая белая банка 50 мл. Материал в источниках не указан. Крышка матовая, над чёрным пояском: в packaging-text.json она clear frosted, на фото 1 выглядит белой. Банка лежит в коробке цвета слоновой кости с шалфейной полосой и золотой надписью DERMA RECOVERY / CREAM. Экран 1 открывает коробка, её фасад готов. Дальше герои — банка и сам белый крем. Фасад банки берётся с фото заказчика в Figma: фото 1, узел 93:8080, фасад с этикеткой. Открытая банка — фото 73, узел 113:8211. Поэтому банку показываем фасадом и поворачиваем не больше чем на ±20°. Задняя сторона банки не снята.</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Матовая белая банка 50 мл. Материал в источниках не указан. Крышка матовая, над чёрным пояском: в packaging-text.json она clear frosted, на фото 1 выглядит белой. Банка лежит в коробке цвета слоновой кости с шалфейной полосой и золотой надписью DERMA RECOVERY / CREAM. Экран 1 открывает коробка, её фасад готов. Дальше герои — банка и сам белый крем. Фасад банки берётся с фото заказчика в Figma: фото 1, узел 93:8080, фасад с этикеткой. Открытая банка — фото 73, узел 113:8211. Поэтому банку показываем фасадом и поворачиваем не больше чем на ±20°. Задняя сторона банки не снята.</t>
+          <t>После игл обновления приходит мягкость: банка поднимается из коробки и открывается без единой иглы, лента крема ложится на кожу у зеркала, а на зелёном экране серии обе ветки BIOSPICULE — домашние сыворотки и MICRO BOOST 10% в клинике — сходятся к DERMA.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>После игл обновления приходит мягкость: банка поднимается из коробки и открывается без единой иглы, лента крема ложится на кожу у зеркала, а на зелёном экране серии обе ветки BIOSPICULE — домашние сыворотки и MICRO BOOST 10% в клинике — сходятся к DERMA.</t>
+          <t>פנים</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>פנים</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
           <t>1, 5, 73</t>
         </is>
       </c>
+      <c r="K11" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M11" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1141,56 +1085,51 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>mitopen</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>mitopen</t>
+          <t>DEVICES</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>DEVICES</t>
+          <t>device</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>device</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
           <t>Фон — тёмная база бренда #0a0a0b. Дальний слой поворачивается за курсором: медленный холодный серебряный дым #d9d4cc с тонкими прожилками шампань-металла #d8c48a и мелкая серебряная пыль. Это цвет линейки DEVICES, как на странице MITOSCAN. Серебро ведущее, потому что шампань #d8c48a у DEVICES совпадает с цветом линейки PEELING (EXO-NAD), и различить их можно только по серебру. К тому же перо цвета шампань лучше читается на серебре. По кромке пера идёт холодный серебряный контровой свет. Золото бренда #c9a24b используется только для волосяных линий, кикеров, бейджа назначения «מקצועי» (золотая заливка) и кнопок цены. Главная кнопка и кнопка в липкой панели — с заливкой #c9a24b и текстом #0a0a0b, как .btn.primary в proto/exocell-3d-template.html. Призрачные кнопки на экранах 1 и 5 — с золотым контуром. «Угольную заливку» из примечания к b6.cta не используем: #1a1a1f на #0a0a0b даёт контраст около 1.1:1. Своей капли у MITOPEN нет, поэтому работает цвет линейки. Единственное тёплое пятно на странице — розово-золотое кольцо и кнопка самого прибора. V-TECH SYSTEM и EXOSIGNAL HAIR на экране 5 стоят только как предметы, их цвета на фон не переносим: два цвета линеек на одной странице запрещены. MICRO BOOST 10% (зелёная BIOSPICULE) упоминается только меткой b4.label4. Оттенок серии — на экране 7: там самый яркий серебряный дым и контровой свет страницы, шампань идёт вторым цветом, а рядом с бейджем «מקצועי» стоит бейдж линейки «מכשור» (home.sl-2) с серебряным контуром.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="F12" s="2" t="n">
         <v>7</v>
       </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>MITOPEN — беспроводная ручка для микронидлинга. Корпус из металла цвета шампань-золото. Розово-золотое ребристое кольцо рукоятки (в packaging-text.json это «rose-gold knurled grip ring»; задаёт ли оно глубину, в источниках не сказано — вопрос 2). Такого же цвета кнопка с маленькой точкой над ней, прозрачный картридж с иглами. Надписи берём только с фото: вертикальная белая «MITOPEN» на корпусе и маленькая гравированная V у верхнего конуса. На пакшоте ось пера отклонена от вертикали примерно на 12° (замер по альфа-каналу mitopen.webp): конус вверху справа, картридж внизу слева. Коробки в источниках нет, поэтому героем идёт сам прибор.</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>MITOPEN — беспроводная ручка для микронидлинга. Корпус из металла цвета шампань-золото. Розово-золотое ребристое кольцо рукоятки (в packaging-text.json это «rose-gold knurled grip ring»; задаёт ли оно глубину, в источниках не сказано — вопрос 2). Такого же цвета кнопка с маленькой точкой над ней, прозрачный картридж с иглами. Надписи берём только с фото: вертикальная белая «MITOPEN» на корпусе и маленькая гравированная V у верхнего конуса. На пакшоте ось пера отклонена от вертикали примерно на 12° (замер по альфа-каналу mitopen.webp): конус вверху справа, картридж внизу слева. Коробки в источниках нет, поэтому героем идёт сам прибор.</t>
+          <t>MITOPEN задаёт глубину 0.25–2.5 мм и одну из пяти скоростей, прозрачный картридж оставляет ровную сетку временных микроканалов, а по ней уходят V-TECH SYSTEM в кожу лица и EXOSIGNAL HAIR в кожу головы: одна ручка — точная и повторяемая процедура.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>MITOPEN задаёт глубину 0.25–2.5 мм и одну из пяти скоростей, прозрачный картридж оставляет ровную сетку временных микроканалов, а по ней уходят V-TECH SYSTEM в кожу лица и EXOSIGNAL HAIR в кожу головы: одна ручка — точная и повторяемая процедура.</t>
+          <t>פנים · קרקפת</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>פנים · קרקפת</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
           <t>56, 57</t>
         </is>
       </c>
+      <c r="K12" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1202,56 +1141,51 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>mitoscan</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>mitoscan</t>
+          <t>DEVICES</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>DEVICES</t>
+          <t>device</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>device</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
           <t>База бренда: фон #0a0a0b. Дальний слой, дым и частицы, сделан в цвете линейки DEVICES по правилу «цветовое окружение по линейке»: холодный серебряный дым #d9d4cc с тёплыми прожилками шампань-металла #d8c48a и мелкая серебряная пыль. На белых корпусах и хроме лежит контровой свет шампань. MITOSCAN не исключение, в отличие от MASK. Капля средства — синий MITOSCAN #5aa9e6, не больше ~10% площади: свечение экрана, активный сегмент ×50 / ×200 и узкий рефлекс на щупе. Страницу целиком в синий не красим. Золото бренда #c9a24b идёт на волосяные выноски, кикеры, кнопку цены и бейдж «מקצועי» (home.tg, золотая заливка). Кнопка цены золотая по правилу палитры. Синяя заливка из EN-описания b6.cta противоречит правилу «капля ≤10%», её не берём. Бирюзово-фиолетовая мишень на экране — это печать экрана с пакшота: её не перекрашиваем и в фон не выносим. Белая клиническая студия и «blue on dark» из site/prompts/mitoscan.md написаны до правила линеек и сюда не идут. Белые объекты стоят на тёмном фоне.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="F13" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Система MITOSCAN целиком, как на пакшоте. Белый планшет на белой подставке с экраном-логотипом (мишень, 'Mitoscan', 'By Mitoderm Ltd'). Справа в держателе щуп-сканер: белый корпус, чёрная овальная панель 'Mitoscan' / 'By Mitoderm Ltd', спиральный кабель. Спереди серебряный цилиндр с хромовым шильдиком 'Mitoscan'. Сюжет ведёт щуп, «המצלמה» из b0.cta, а результат появляется на экране. Пока нет фото частей по отдельности, всё строится одним биллбордом целого пакшота: части не двигаются, работают камера и маски.</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Система MITOSCAN целиком, как на пакшоте. Белый планшет на белой подставке с экраном-логотипом (мишень, 'Mitoscan', 'By Mitoderm Ltd'). Справа в держателе щуп-сканер: белый корпус, чёрная овальная панель 'Mitoscan' / 'By Mitoderm Ltd', спиральный кабель. Спереди серебряный цилиндр с хромовым шильдиком 'Mitoscan'. Сюжет ведёт щуп, «המצלמה» из b0.cta, а результат появляется на экране. Пока нет фото частей по отдельности, всё строится одним биллбордом целого пакшота: части не двигаются, работают камера и маски.</t>
+          <t>Камера поднимается к щупу MITOSCAN, сквозь дымку «на глаз» переходит к экрану, где открываются ×50 и ×200, показывает то, что видит пациент, проводит через «сканирование · объяснение · отслеживание» и отъезжает к целой системе на экране покупки.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Камера поднимается к щупу MITOSCAN, сквозь дымку «на глаз» переходит к экрану, где открываются ×50 и ×200, показывает то, что видит пациент, проводит через «сканирование · объяснение · отслеживание» и отъезжает к целой системе на экране покупки.</t>
+          <t>פנים</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>פנים</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
           <t>81</t>
         </is>
       </c>
+      <c r="K13" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="L13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M13" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1263,56 +1197,51 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>home</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>all lines: V-TECH FACE · PEELING · BIOSPICULE · DEVICES · HAIR (one line per screen 2–6)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>all lines: V-TECH FACE · PEELING · BIOSPICULE · DEVICES · HAIR (one line per screen 2–6)</t>
+          <t>page</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>page</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
           <t>Экраны 1 и 7 — нейтральная база бренда (design-rules, слой 1). Фон #0a0a0b, поверхности #111114 / #1a1a1f, графитовый дым, кремовая пыль #f6f3ec не больше 8%, текст крем #f6f3ec. Золото #c9a24b здесь только в волосяных линиях, кикерах и кнопке. Цветов линеек на этих экранах нет: группы в герое и на полке различаются расстановкой и подписями. Экраны 2–6 — каждый в окружении своей линейки, цвет меняется только в зоне перехода. 2 V-TECH FACE — чёрный, тёплый золотой дым #c9a24b, золотая пыль #d8bd7e, блики зеркальной фольги. 3 PEELING — шампань-золото #d8c48a. 4 BIOSPICULE — зелёный #1E4634 и тёмный #12382A, подложка шалфея #9AA889 под DERMA, золотая монограмма M. 5 DEVICES — холодный шампань-металл #d8c48a и серебро #d9d4cc. 6 HAIR — чёрный, золотой дым и пыль. Золотой дым есть только на экранах 2 и 6, поэтому на переходах 1→2 и 6→7 меняется цвет, а не только плотность дыма. V-TECH FACE и HAIR по правилам одного цвета, их различает бейдж линейки. Это подпись группы под волосяной линией: точка и название в цвете линейки, как бейдж серии на экране покупки MASK. Капля средства — только узкое свечение под упаковкой, не больше ~10% площади: EXOCELL MASK бирюза #6fb7ba на экране 2, CELL RENEW #4fb285 на экране 4, MITOSCAN #5aa9e6 на экране 5. На главной MASK стоит в чёрно-золотом окружении своей серии V-TECH FACE: её бирюзовое окружение — исключение только на её собственной странице. Назначение показывают бейджи, а не фон: «מקצועי» — золотая заливка, домашний уход — золотой контур. Оттенок серии виден на всех экранах 2–6; в поле ниже указан первый из них.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="F14" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Вся линейка: 12 настоящих упаковок пятью группами на пологой дуге (V-TECH FACE · PEELING · BIOSPICULE · DEVICES · HAIR). Ближе всех и в центре — золотой зеркальный картон V-TECH SYSTEM. MITOTECH CELL BOOSTER без фото в 3D не показывается. EXOSIGNAL SPRAY до студийного пакшота — только маленький билборд коробки в глубине, без флакона.</t>
+        </is>
+      </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Вся линейка: 12 настоящих упаковок пятью группами на пологой дуге (V-TECH FACE · PEELING · BIOSPICULE · DEVICES · HAIR). Ближе всех и в центре — золотой зеркальный картон V-TECH SYSTEM. MITOTECH CELL BOOSTER без фото в 3D не показывается. EXOSIGNAL SPRAY до студийного пакшота — только маленький билборд коробки в глубине, без флакона.</t>
+          <t>Главная — прогулка по полке MITODERM: вся линейка стоит дугой из пяти групп, с каждым экраном вперёд выходит одна серия в своём цветовом окружении (лицо, пилинг, биоспикулы, приборы, волосы) и ведёт на страницы своих средств, а в конце все упаковки возвращаются на общую полку с составом каждой линейки и одной кнопкой «לקבלת פרטים על מחירים».</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Главная — прогулка по полке MITODERM: вся линейка стоит дугой из пяти групп, с каждым экраном вперёд выходит одна серия в своём цветовом окружении (лицо, пилинг, биоспикулы, приборы, волосы) и ведёт на страницы своих средств, а в конце все упаковки возвращаются на общую полку с составом каждой линейки и одной кнопкой «לקבלת פרטים על מחירים».</t>
+          <t>פנים · קרקפת · טריכולוג/ית</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>פנים · קרקפת · טריכולוג/ית</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
           <t>66, 71, 76</t>
         </is>
       </c>
+      <c r="K14" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="L14" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="M14" s="2" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1324,25 +1253,20 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>catalog</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>catalog</t>
+          <t>все линейки: V-TECH FACE · HAIR · PEELING · BIOSPICULE · DEVICES</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>все линейки: V-TECH FACE · HAIR · PEELING · BIOSPICULE · DEVICES</t>
+          <t>page</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>page</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Экраны 1, 2 и 7 стоят на базе бренда: фон #0a0a0b, медленный золотой дым #c9a24b, частицы цвета крема и золота, белый логотип. На каталоге есть все линейки, поэтому правило «не смешивать два цвета линеек» соблюдается поэкранно: на каждом экране только один цвет линейки, при переходе дым перетекает за 600 мс.
 Экран 3 (V-TECH FACE + HAIR): чёрный и тёплое золото V-TECH FACE, свечение сильнее, чем на базе. Бирюза EXOCELL #6fb7ba даётся только узкой каплей под её карточкой (не больше 10%), а бирюзово-синее окружение MASK остаётся на её странице.
@@ -1353,33 +1277,33 @@
 Назначение показывается бейджем, а не цветом: home.tg — золотая заливка, catalog.chips[6] — золотой контур. Бейдж и чип домашнего ухода берутся из одного ключа. Оттенок серии виден на каждом из экранов 3–6; в поле стоит экран 3, где он появляется впервые: тёплое золото V-TECH FACE, как на экране покупки MASK.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="F15" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Одного героя нет. На экране 1 стоит «витрина линеек» из пяти представителей: коробки V-TECH SYSTEM, EXO-NAD, EXOSIGNAL HAIR и MICRO BOOST 10% (кубоиды почти фасадом, рыскание не больше 12°, потому что печать их боковин неизвестна) и MITOPEN (строго фронтальный билборд). Дальше 3D работает в карточках: при наведении товар поворачивается к фасаду.</t>
+        </is>
+      </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Одного героя нет. На экране 1 стоит «витрина линеек» из пяти представителей: коробки V-TECH SYSTEM, EXO-NAD, EXOSIGNAL HAIR и MICRO BOOST 10% (кубоиды почти фасадом, рыскание не больше 12°, потому что печать их боковин неизвестна) и MITOPEN (строго фронтальный билборд). Дальше 3D работает в карточках: при наведении товар поворачивается к фасаду.</t>
+          <t>Каталог — спокойная витрина: пять представителей линеек встречают посетителя на чёрно-золотом фоне и спускаются на полку категорий; дальше каждая линейка идёт своим экраном в своём цвете, в каждой карточке видно, что лежит в коробке, а вся страница ведёт к одной кнопке цены.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Каталог — спокойная витрина: пять представителей линеек встречают посетителя на чёрно-золотом фоне и спускаются на полку категорий; дальше каждая линейка идёт своим экраном в своём цвете, в каждой карточке видно, что лежит в коробке, а вся страница ведёт к одной кнопке цены.</t>
+          <t>פנים · קרקפת · טריכולוג/ית</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>פנים · קרקפת · טריכולוג/ית</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
           <t>пакшоты всех средств</t>
         </is>
       </c>
+      <c r="K15" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="L15" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M15" s="2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2201,7 +2125,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут · AHA + BHA ≈30% · NAD⁺ · אקסוזומים סינתטיים · פיצפטריק I–VI</t>
+          <t>PEELING · AHA + BHA ≈30% · NAD⁺ · אקסוזומים סינתטיים · פיצפטריק I–VI</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -2683,7 +2607,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>מקצועי · ⏳ перевод на иврит и две проверки идут · 1 × 15 מ״ל Biphasic Peel · 5 × 5 מ״ל pH Normalizer · 5 × 5 מ״ל Longevity Serum · שילוב חומצות AHA ו-BHA (כ־30%) · חומצה טרנקסמית ורכיבים נוגדי חמצון · קולגן ופפטידים ביומימטיים · ויטמין B12 · מבנים אקסוזומליים סינתטיים · NAD⁺ · Epitalon – אפיטלון · GHK-Cu · ⏳ перевод на иврит и две проверки идут</t>
+          <t>מקצועי · PEELING · 1 × 15 מ״ל Biphasic Peel · 5 × 5 מ״ל pH Normalizer · 5 × 5 מ״ל Longevity Serum · שילוב חומצות AHA ו-BHA (כ־30%) · חומצה טרנקסמית ורכיבים נוגדי חמצון · קולגן ופפטידים ביומימטיים · ויטמין B12 · מבנים אקסוזומליים סינתטיים · NAD⁺ · Epitalon – אפיטלון · GHK-Cu · WhatsApp · טלפון · דוא״ל</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -2853,7 +2777,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>מקצועי · ⏳ перевод на иврит и две проверки идут · שלב מסכם לאחר פרוצדורה · לחות וקרירות · תמיכה במחסום העור</t>
+          <t>מקצועי · V-TECH FACE · שלב מסכם לאחר פרוצדורה · לחות וקרירות · תמיכה במחסום העור</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -3185,7 +3109,7 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>5 · מסכות באריזה · ביו-צלולוז · מבנה דק וגמיש · חד-פעמית · סרום פעיל · ⏳ перевод на иврит и две проверки идут</t>
+          <t>5 · מסכות באריזה · ביו-צלולוז · מבנה דק וגמיש · חד-פעמית · סרום פעיל · מסכה כפולה: שכבה לבנה ושכבה כחולה, שמניחים בזו אחר זו.</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr"/>
@@ -3335,7 +3259,7 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут · מה באריזה · 5× · מסכות · מסכות ביו-צלולוז חד-פעמיות עם סרום פעיל. · ⏳ перевод на иврит и две проверки идут · ⏳ перевод на иврит и две проверки идут · רכיבים פעילים · מבנים אקסוזומליים סינתטיים · פולינוקלאוטידים · חומצה היאלורונית, גליצרול ושמנים צמחיים · תמציות צמחיות ותמצית אצה · Hexapeptide-8 · Ubiquinone – קו־אנזים Q10 · Nannochloropsis Oculata Extract · Spilanthes Acmella Extract · טלפון · ⏳ перевод на иврит и две проверки идут · דוא״ל · ⏳ перевод на иврит и две проверки идут · הוסיפו לפנייה על V-TECH / EXO-NAD</t>
+          <t>V-TECH FACE · מה באריזה · 5× · מסכות · מסכות ביו-צלולוז חד-פעמיות עם סרום פעיל. · כל מסכה מורכבת משתי שכבות – לבנה וכחולה – שמניחים בזו אחר זו. · Net 5 x 25 ml · רכיבים פעילים · מבנים אקסוזומליים סינתטיים · פולינוקלאוטידים · חומצה היאלורונית, גליצרול ושמנים צמחיים · תמציות צמחיות ותמצית אצה · Hexapeptide-8 · Ubiquinone – קו־אנזים Q10 · Nannochloropsis Oculata Extract · Spilanthes Acmella Extract · טלפון · 054-326-2182 · דוא״ל · info@mitoderm.com · הוסיפו לפנייה על V-TECH / EXO-NAD</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -4778,7 +4702,7 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>V-TECH FACE</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
@@ -5252,7 +5176,7 @@
       <c r="F48" s="2" t="inlineStr"/>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>V-TECH FACE</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
@@ -9426,7 +9350,7 @@
       </c>
       <c r="K98" s="3" t="inlineStr">
         <is>
-          <t>צרו קשר · מוצרים מקצועיים · מקצועי · הכל · ⏳ перевод на иврит и две проверки идут</t>
+          <t>צרו קשר · מוצרים מקצועיים · מקצועי · הכל · גללו</t>
         </is>
       </c>
       <c r="L98" s="2" t="inlineStr">
@@ -9491,7 +9415,7 @@
       </c>
       <c r="G99" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>V-TECH FACE</t>
         </is>
       </c>
       <c r="H99" s="3" t="inlineStr">
@@ -9501,7 +9425,7 @@
       </c>
       <c r="I99" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>בקליניקה – V-TECH SYSTEM, ולסיום EXOCELL MASK; בבית – EXOTECH GEL.</t>
         </is>
       </c>
       <c r="J99" s="3" t="inlineStr">
@@ -9932,7 +9856,7 @@
       </c>
       <c r="K104" s="3" t="inlineStr">
         <is>
-          <t>לקבלת פרטים על מחירים · ⏳ перевод на иврит и две проверки идут · טלפון · דוא״ל · צרו קשר · צרו קשר</t>
+          <t>לקבלת פרטים על מחירים · WhatsApp · טלפון · דוא״ל · צרו קשר · צרו קשר</t>
         </is>
       </c>
       <c r="L104" s="2" t="inlineStr">
@@ -10168,7 +10092,7 @@
       <c r="G107" s="3" t="inlineStr"/>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>בחרו קטגוריה</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr"/>
@@ -10232,7 +10156,7 @@
       </c>
       <c r="G108" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут · שיער</t>
+          <t>V-TECH FACE · שיער</t>
         </is>
       </c>
       <c r="H108" s="3" t="inlineStr">
@@ -10583,7 +10507,7 @@
       </c>
       <c r="J112" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут · טלפון · דוא״ל · היבואנית הבלעדית של VM בישראל</t>
+          <t>WhatsApp · טלפון · דוא״ל · היבואנית הבלעדית של VM בישראל</t>
         </is>
       </c>
       <c r="K112" s="3" t="inlineStr">
@@ -16888,7 +16812,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>אריזת V-TECH SYSTEM עם 5 אמפולות סרום ו-5 שקיות מסכת ג׳ל</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -16915,7 +16839,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>PEELING</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -16942,7 +16866,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>WhatsApp · טלפון · דוא״ל</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -16969,7 +16893,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>V-TECH FACE</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -16996,7 +16920,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>מסכה כפולה: שכבה לבנה ושכבה כחולה, שמניחים בזו אחר זו.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -17023,7 +16947,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>כל מסכה מורכבת משתי שכבות – לבנה וכחולה – שמניחים בזו אחר זו.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -17050,7 +16974,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>Net 5 x 25 ml</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -17077,7 +17001,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>054-326-2182</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -17104,7 +17028,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>info@mitoderm.com</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -17158,7 +17082,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>HAIR</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -17185,7 +17109,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>שלום, אשמח לקבל פרטים על מחירי EXOSIGNAL HAIR</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -17212,7 +17136,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>שלום, אשמח לתאם הדגמת MITOSCAN עבור EXOSIGNAL HAIR</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -17293,7 +17217,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>V-TECH FACE</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -17320,7 +17244,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>שלום! איפה אפשר לקנות את EXOTECH GEL?</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -17347,7 +17271,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>BIOSPICULE™</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -17374,7 +17298,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>אריזת MICRO BOOST 10% ומזרק של 3 מ״ל</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -17401,7 +17325,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>BIOSPICULE™</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -17428,7 +17352,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>טיפוח ביתי</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -17455,7 +17379,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>אריזת DERMA RECOVERY CREAM וצנצנת של 50 מ״ל</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -17509,7 +17433,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>V-TECH FACE</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -17536,7 +17460,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>בקליניקה – V-TECH SYSTEM, ולסיום EXOCELL MASK; בבית – EXOTECH GEL.</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -17563,7 +17487,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>Net 5 x 25 ml</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -17590,7 +17514,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -17617,7 +17541,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>גללו</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -17671,7 +17595,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>⏳ перевод на иврит и две проверки идут</t>
+          <t>בחרו קטגוריה</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Remove a photo with a person from the repo; add the facts check
The spray photo held at a cheek shows a person and must not sit in the
public repo; it moves to private storage and references point to the
owner's box-and-bottle photos in Figma. It remains in earlier history.
The workbook gains the sheet of 59 story facts checked against the
owner's protocols, mitoderm.com and the catalogue.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/MITODERM-3D-story.xlsx
+++ b/mitoderm-catalog/site/MITODERM-3D-story.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mitoderm.com" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сверка с источниками" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4287,7 +4288,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Герой экрана — кожа головы, а не флакон. Справа в 3D под небольшим углом плавает фото-рамка: вид сверху на пробор, капли на коже впитываются (новый кадр, см. вопрос 3). Рамка слегка наклоняется за курсором. На её поверхность оседают последние капли дымки с экрана 3 и исчезают без следа — это «ללא שטיפה». Флакон маленький и тёмный, в глубине сбоку, стоит фасадом. Метки b3.label1–4 ложатся по краю рамки. Фото site/img/exosignal-spray-hand.jpg на странице не используется: на нём флакон у щеки, видно лицо, а кожи головы нет.</t>
+          <t>Герой экрана — кожа головы, а не флакон. Справа в 3D под небольшим углом плавает фото-рамка: вид сверху на пробор, капли на коже впитываются (новый кадр, см. вопрос 3). Рамка слегка наклоняется за курсором. На её поверхность оседают последние капли дымки с экрана 3 и исчезают без следа — это «ללא שטיפה». Флакон маленький и тёмный, в глубине сбоку, стоит фасадом. Метки b3.label1–4 ложатся по краю рамки. Фото фото флакона в руке (с человеком: хранится закрыто, не в репозитории) на странице не используется: на нём флакон у щеки, видно лицо, а кожи головы нет.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -13308,7 +13309,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Цилиндр из матового полупрозрачного стекла и рифлёный золотой колпачок. Наклейку снять с site/img/exosignal-spray-hand.jpg (565×1340) и выпрямить наклон. Видимые строки по packaging-text.json: VM-монограмма, вертикальная 'EXOSIGNAL' ('EXO' жирным), 'S P R A Y · H O M E', 'EXOSIGNAL SPRAY HOME', 'Deep nourishing scalp serum', 'HOME USE'. Строки, помеченные [unreadable], и строки под пальцами рисуются тонкими серыми линиями. Файл site/img/exosignal-spray.png не использовать: это скриншот 400×300, и флакон на нём непрозрачный белый с гладким колпачком, то есть не настоящий. Показывать только мелким планом. Нужен студийный пакшот флакона на прозрачном фоне.</t>
+          <t>Цилиндр из матового полупрозрачного стекла и рифлёный золотой колпачок. Наклейку снять с фото флакона в руке (с человеком: хранится закрыто, не в репозитории) (565×1340) и выпрямить наклон. Видимые строки по packaging-text.json: VM-монограмма, вертикальная 'EXOSIGNAL' ('EXO' жирным), 'S P R A Y · H O M E', 'EXOSIGNAL SPRAY HOME', 'Deep nourishing scalp serum', 'HOME USE'. Строки, помеченные [unreadable], и строки под пальцами рисуются тонкими серыми линиями. Файл site/img/exosignal-spray.png не использовать: это скриншот 400×300, и флакон на нём непрозрачный белый с гладким колпачком, то есть не настоящий. Показывать только мелким планом. Нужен студийный пакшот флакона на прозрачном фоне.</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -13389,7 +13390,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Полоса этикетки выпрямляется из site/img/exosignal-spray-hand.jpg (565×1340). Печать настоящая, но снята в перспективе, нижние строки у края частично закрыты пальцем, оборот не виден. Фото служит только источником текстуры и на странице не показывается. Поворот не больше ±30° от фасада. Для финала нужен пакшот флакона спереди и сзади на прозрачном фоне.</t>
+          <t>Полоса этикетки выпрямляется из фото флакона в руке (с человеком: хранится закрыто, не в репозитории) (565×1340). Печать настоящая, но снята в перспективе, нижние строки у края частично закрыты пальцем, оборот не виден. Фото служит только источником текстуры и на странице не показывается. Поворот не больше ±30° от фасада. Для финала нужен пакшот флакона спереди и сзади на прозрачном фоне.</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -13470,7 +13471,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Кадра пока нет. Подойдёт фото заказчика или генерация по промпту кадра «Why» (вид сверху на пробор) из site/prompts/exosignal-spray.md. Сначала один образец, цена и баланс — до запуска. site/img/exosignal-spray-hand.jpg не подходит: на нём флакон у щеки, видны лицо и шея, а кожи головы нет.</t>
+          <t>Кадра пока нет. Подойдёт фото заказчика или генерация по промпту кадра «Why» (вид сверху на пробор) из site/prompts/exosignal-spray.md. Сначала один образец, цена и баланс — до запуска. фото флакона в руке (с человеком: хранится закрыто, не в репозитории) не подходит: на нём флакон у щеки, видны лицо и шея, а кожи головы нет.</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -15954,7 +15955,7 @@
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>Студийного пакшота нет: есть фото в руке (site/img/exosignal-spray-hand.jpg, низ флакона закрыт пальцами) и снимок 400×300 (site/img/exosignal-spray.png), где флакон ~40 px и выглядит непрозрачно-белым, а не матовым стеклом. Замену из него не делать: до пакшота флакон и туман на главной не показываются. Нужен пакшот флакона на прозрачном фоне, без руки, фасадом с этикеткой</t>
+          <t>Студийного пакшота нет: есть фото в руке (фото флакона в руке (с человеком: хранится закрыто, не в репозитории), низ флакона закрыт пальцами) и снимок 400×300 (site/img/exosignal-spray.png), где флакон ~40 px и выглядит непрозрачно-белым, а не матовым стеклом. Замену из него не делать: до пакшота флакон и туман на главной не показываются. Нужен пакшот флакона на прозрачном фоне, без руки, фасадом с этикеткой</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
@@ -21258,7 +21259,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Фото site/img/exosignal-spray-hand.jpg (флакон у щеки, видно лицо) на странице не ставим и берём только как источник этикетки. Но это фото с человеком, и оно уже лежит в публичном репозитории, хотя по правилу проекта таким фото там не место. Убрать его из репозитория и хранить копию только локально?</t>
+          <t>Фото фото флакона в руке (с человеком: хранится закрыто, не в репозитории) (флакон у щеки, видно лицо) на странице не ставим и берём только как источник этикетки. Но это фото с человеком, и оно уже лежит в публичном репозитории, хотя по правилу проекта таким фото там не место. Убрать его из репозитория и хранить копию только локально?</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr"/>
@@ -22168,6 +22169,2861 @@
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Страница</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Экран</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Что</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Тип</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>В сюжете</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>В источнике</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Источник</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Предложение</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Проверка скептика</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>V-TECH SYSTEM</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>b4.line, b4.label2 «2 · סרום 1–1.5 מ״ל», cat.steps[1][1] (доза сыворотки и как наносится гель-маска)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>источники расходятся</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>b4.line: «המיקרונידלינג פותח את מסלול החדירה, 1–1.5 מ״ל סרום מוחדרים פנימה ומסכת הג׳ל נשארת על העור – ללא שטיפה.» / cat.steps[1][1]: «בין 1 ל־1.5 מ״ל סרום אקסוזומים סינתטיים לטיפול: פנים, צוואר, דקולטה או כפות ידיים.»</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Протокол: «לאזור טיפול אחד – פנים / צוואר / מחשוף:» «V-TECH Serum: עד 2 מ״ל» «V-TECH Gel Mask: עד 2 מ״ל»; про гель: «יש לעסות בעדינות עד לספיגה מלאה. אין צורך בשטיפה.» Каталог (проигрывает): «כמות: בין 1 ל1.5 מל לטיפול». PLAN §7: «до 2 мл сыворотки и до 2 мл гель-маски на зону».</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:35 (vtech-mitopen, «מינון מומלץ») и :46 (V-TECH GEL MASK); каталог source-texts.md:112; PLAN.md:118</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Побеждает протокол. Метка шага 2 — «2 · סרום עד 2 מ״ל לאזור». В b4.line «1–1.5 מ״ל סרום» заменить на «עד 2 מ״ל סרום לאזור טיפול». Про гель написать по протоколу: втирается мягкими движениями до полного впитывания, смывать не нужно («יש לעסות בעדינות עד לספיגה מלאה. אין צורך בשטיפה.»). В cat.steps[1][1] дозу дать по протоколу: до 2 мл на одну зону (лицо, шея или декольте). Кисти рук протокол не упоминает: зону из каталога не убирать без слова заказчика или задать ему вопрос. Новые строки на иврите — через переводчика и рецензентов.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В content.he.mjs:35 стоит «לאזור טיפול אחד – פנים / צוואר / מחשוף:», а ниже «V-TECH Serum: עד 2 מ״ל» и «V-TECH Gel Mask: עד 2 מ״ל». В :46 сказано «יש לעסות בעדינות עד לספיגה מלאה. אין צורך בשטיפה.». В каталоге (source-texts.md:112) «כמות: בין 1 ל1.5 מל לטיפול». PLAN.md:118 подтверждает, что главный источник — протокол: «до 2 мл сыворотки и до 2 мл гель-маски на зону». В сюжете действительно «1–1.5 מ״ל» в b4.line, b4.label2 и cat.steps[1][1], а гель «נשארת על העור». Поправка: протокол даёт дозу на зону «פנים / צוואר / מחשוף» и про кисти рук молчит. Значит, убирать кисти, которые есть в каталоге, без слова заказчика нельзя.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>V-TECH SYSTEM</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>b4.label4 «בסיום: EXOCELL MASK + SPF» и cat.steps[2][1] (чем заканчивается протокол)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>источники расходятся</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>b4.label4: «בסיום: EXOCELL MASK + SPF»; cat.steps[2][1]: «לאחר האמפולה, ללא שטיפה. בסיום הטיפול: EXOCELL MASK או DERMA RECOVERY ומקדם הגנה.»</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Протокол, «לאחר הסרום»: «מומלץ להניח מסכת EXOCELL MASK להחדרה של חומצה הילארונית , תמציות צמחים ואלוורה.» → «בסיום DERMA RECOVERY CREAM» → «מקדם הגנה חובה». PLAN §7: «финиш EXOCELL MASK → DERMA RECOVERY → SPF».</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:51-53 (vtech-mitopen, after); PLAN.md:118</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Финиш дать последовательностью протокола, а не через «или»: EXOCELL MASK (рекомендуется), затем DERMA RECOVERY CREAM, затем обязательно SPF. В b4.label4 добавить DERMA RECOVERY CREAM в этом порядке. В cat.steps[2][1] вместо «EXOCELL MASK או DERMA RECOVERY» написать порядок протокола. Два чипа-ссылки оставить в том же порядке: EXOCELL MASK, потом DERMA RECOVERY CREAM. Иврит — через переводчика.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В content.he.mjs:51–53 блок «לאחר הסרום» идёт по порядку: «מומלץ להניח מסכת EXOCELL MASK…», затем «בסיום DERMA RECOVERY CREAM», затем «מקדם הגנה חובה». В PLAN.md:118 тот же порядок: «финиш EXOCELL MASK → DERMA RECOVERY → SPF». В сюжете b4.label4 — «בסיום: EXOCELL MASK + SPF» (без DERMA RECOVERY), а в cat.steps[2][1] стоит «או». Уточнение: маска в протоколе «מומלץ» (рекомендуется), а SPF — «חובה» (обязательно).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>V-TECH SYSTEM</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>b4.title / b4.line («каждые две недели, 4 процедуры») вместе с cat.steps[0][1], где BIOSPICULE™ 10% стоит среди способов открыть каналы</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>источники расходятся</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>b4.title «שלושה שלבים, כל שבועיים»; b4.line «…4 טיפולים, בהפרש של שבועיים.»; cat.steps[0][1] «…מיקרונידלינג, RF microneedling, BIOSPICULE™ 10% או Laser CO₂ פותחים את מסלול החדירה.»</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Отдельный протокол «BIOSPICULE™ MICROBOOST 10% + VTECH»: «ניתן לבצע סדרה של 4–3 טיפולים, במרווח של 4 שבועות בין טיפול לטיפול.»; финиш там: «SPF   מסנן קרינה של 30 לפחות חובה». Ритм раз в 14 дней относится к протоколу «VTECH+ MITOPEN».</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:65-69 (biospicule-vtech, aside «סדרת טיפולים»), :91; :32, :56 (vtech-mitopen)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Не обещать «каждые две недели» для любого способа. Указать, что ритм 14 дней и курс 4–6 относятся к протоколу с MITOPEN / мезопеном. С BIOSPICULE™ MICRO BOOST 10% — 3–4 процедуры с интервалом 4 недели (протокол «BIOSPICULE™ MICROBOOST 10% + VTECH»). Достаточно уточнения в раскрытом шаге 1 (cat.steps[0][1]) или короткой сноски под b4.line. BIOSPICULE™ 10% из шага 1 не убирать. Иврит — через переводчика.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. У протокола «BIOSPICULE™ MICROBOOST 10% + VTECH» свой ритм (content.he.mjs:69): «ניתן לבצע סדרה של 4–3 טיפולים, במרווח של 4 שבועות בין טיפול לטיפול.» Ритм «каждые 14 дней» взят из протокола «VTECH+ MITOPEN» (:56). Сюжет ставит BIOSPICULE™ 10% среди способов шага 1 (b4.label1, cat.steps[0][1]) и при этом обещает «כל שבועיים» (b4.title, b4.line, b5.label4). Поправка к предложению: вариант «убрать BIOSPICULE™ 10%» не подходит. Этот способ есть и в каталоге, и в протоколах заказчика.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>V-TECH SYSTEM</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>b5.line (курс и поддержка), b5.label3</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>источники расходятся</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>«5 אמפולות סרום של 5 מ״ל ו-5 שקיות מסכת ג׳ל של 5 מ״ל. סדרה מומלצת: לפחות 4 טיפולים; תחזוקה אחת לחצי שנה.» / b5.label3 «4 טיפולים בסדרה»</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Протокол: «טיפול אחד בכל 14 יום.» «סדרה מומלצת: 6-4טיפולים, בהתאם למצב העור ולמטרת הטיפול.» «פרוטוקול בסיס של 4 טיפולים רצופים: כל שבועיים» «לאחר השלמת הסדרה מומלץ לבצע טיפול תחזוקה אחת לחודשיים-שלושה, בהתאם למצב העור...» Каталог (проигрывает): «לפחות 4 טיפולים תחזוקה : אחת לחצי שנה».</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:56-59 (vtech-mitopen, «תדירות וסדרת טיפולים»); source-texts.md:112</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Заменить в b5.line по протоколу: «סדרה מומלצת: 4–6 טיפולים; טיפול תחזוקה אחת לחודשיים-שלושה». b5.label3 сделать «4–6 טיפולים בסדרה» (4 — это базовый протокол «4 טיפולים רצופים: כל שבועיים», поэтому так и подписать, если нужна одна цифра). Поддержку раз в полгода убрать со всей страницы. Иврит — через переводчика.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В content.he.mjs:56–59: «טיפול אחד בכל 14 יום.», «סדרה מומלצת: 6-4טיפולים», «פרוטוקול בסיס של 4 טיפולים רצופים: כל שבועיים» и «טיפול תחזוקה אחת לחודשיים-שלושה». В каталоге (:112) «לפחות 4 טיפולים … תחזוקה : אחת לחצי שנה». PLAN.md:118 — «курс 4–6». В сюжете b5.line: «סדרה מומלצת: לפחות 4 טיפולים; תחזוקה אחת לחצי שנה.» Поддержка раз в полгода прямо противоречит протоколу.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>V-TECH SYSTEM</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>список «что внутри»: строка дозы cat.steps[1][1] под cat.kit[0]; cat.kit[1] без дозы («дозы в каталоге нет, её не пишем»)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>источники расходятся</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Доза сыворотки: «בין 1 ל־1.5 מ״ל סרום אקסוזומים סינתטיים לטיפול: פנים, צוואר, דקולטה או כפות ידיים.»; у гель-маски: «дозы в каталоге нет, её не пишем»</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>«לאזור טיפול אחד – פנים / צוואר / מחשוף:» «V-TECH Serum: עד 2 מ״ל» «V-TECH Gel Mask: עד 2 מ״ל»</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:35 (vtech-mitopen, «מינון מומלץ»)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>В списке «что внутри» под сывороткой написать «עד 2 מ״ל לאזור טיפול» вместо 1–1,5 мл. Под гель-маской добавить дозу из протокола: «עד 2 מ״ל לאזור טיפול». Иврит — через переводчика.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. На экране 7 сюжет ставит под сыворотку cat.steps[1][1] («בין 1 ל־1.5 מ״ל…»), а про гель-маску пишет «дозы в каталоге нет, её не пишем». В основном протоколе (content.he.mjs:35) есть обе дозы: «V-TECH Serum: עד 2 מ״ל» и «V-TECH Gel Mask: עד 2 מ״ל» на одну зону. Довод «в каталоге нет» больше не работает. Правка та же, что в находке 0, но поле другое — экран покупки.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>V-TECH SYSTEM</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>inside</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>inside.components[0].volume_dose; inside.components[1].volume_dose</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>[0]: «5 мл во флаконе; на процедуру 1–1,5 мл (cat.steps[1][1])»; [1]: «5 мл в саше; наносится после сыворотки, без смывания. Дозы на процедуру в каталоге нет, на странице её не указываем»</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>«V-TECH Serum: עד 2 מ״ל», «V-TECH Gel Mask: עד 2 מ״ל» на одну зону; «יש לעסות בעדינות עד לספיגה מלאה. אין צורך בשטיפה.»; «יש להשתמש באמפולה עד חודש ממועד הפתיחה, בהתאם להנחיות האחסון של המוצר.»</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:35-36, :46</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>[0]: «5 мл во флаконе; до 2 мл на одну зону (лицо / шея / декольте); набирают шприцем 3 мл через иглу для набора; открытую ампулу использовать в течение месяца». [1]: «5 мл в саше; до 2 мл на одну зону; после сыворотки втирается до полного впитывания, без смывания».</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В inside.components[0] стоит «на процедуру 1–1,5 мл», в [1] — «Дозы … в каталоге нет». Протокол (content.he.mjs:35–36, 40, 46) даёт: до 2 мл сыворотки и до 2 мл гель-маски на зону; набор шприцем 3 мл через иглу для набора («מחט שאיבה למזרק 3 מ״ל»); открытую ампулу использовать до месяца; гель втирать до полного впитывания, без смывания.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>V-TECH SYSTEM</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[2] — как берут сыворотку из флакона (шприц, пипетка, пробка)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>«И как сыворотку берут из флакона: шприцем, пипеткой, снимают пробку? Пока ответа нет, колпачок закрыт, а капля возникает в воздухе над флаконом.»</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>«יש לשאוב את V-TECH Serum באמצעות מחט שאיבה למזרק 3 מ״ל.» «יש ליישם את הסרום באמצעות MITOPEN / מזופן או מכשור מקצועי מתאים אחר.»</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:40-41 (vtech-mitopen, шаг V-TECH SERUM); PLAN.md:118</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Ответ есть: сыворотку набирают шприцем 3 мл через иглу для набора и наносят MITOPEN / мезопеном (или другим подходящим профессиональным прибором). В вопросе оставить только цвет колпачка. Капля над флаконом в 3D может остаться схемой, а в раскрытом шаге 2 сказать про шприц 3 мл и MITOPEN / мезопен.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В content.he.mjs:40–41: «יש לשאוב את V-TECH Serum באמצעות מחט שאיבה למזרק 3 מ״ל.» и «יש ליישם את הסרום באמצעות MITOPEN / מזופן או מכשור מקצועי מתאים אחר.» PLAN.md:118: «сыворотку набирают шприцем 3 мл». Значит, на вопрос «шприцем, пипеткой, пробку снимают?» ответ есть. Цвет колпачка протокол не называет, этот вопрос остаётся.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>V-TECH SYSTEM</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[4] и экран 3 (cat.ingredients[7] отдельной строкой) — к какому компоненту относятся гиалуроновая кислота и алоэ</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>«Гиалуроновая кислота и алоэ вера (последний пункт состава) — в сыворотке или в гель-маске? Пока в раскрытом составе это отдельная строка после двух групп.»</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm.com, Gel Mask: «חומצה היאלורונית במשקל מולקולרי נמוך, אלוורה» (EN: «Low molecular weight hyaluronic acid, aloe vera»); каталог HE — под «מסכת גל לאחר האמפולה ללא שטיפה»: «חומצה היאלורונית / אלוורה»; каталог RU — под «Гелевая маска»: «Гиалуроновая кислота / Алоэ вера».</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>site/sources/mitoderm-com/products-he.json:11 (solution.main.item2textP5); source-texts.md:104-110; source-texts-ru-2026-09-18.md (Полоса 06, «Гелевая маска»)</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Гиалуроновая кислота и алоэ — в гель-маске. На экране 3 перенести cat.ingredients[7] в группу гель-маски (после «PDRN 1% … – מסכת ג׳ל») и не давать его отдельной строкой. Вопрос закрыть.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. На mitoderm.com гиалуроновая кислота и алоэ стоят в блоке гель-маски: products-he.json:11, item2 «V-Tech Gel Mask 5ml», item2textP5 «חומצה היאלורונית במשקל מולקולרי נמוך, אלוורה»; на английской версии «Low molecular weight hyaluronic acid, aloe vera». В каталоге HE (source-texts.md:104–110) они стоят под «מסכת גל לאחר האמפולה ללא שטיפה». В каталоге RU (:111–118) — под «Гелевая маска». Отдельный пункт cat.ingredients[7] «חומצה היאלורונית ואלוורה» в сюжете идёт отдельной строкой — это подтверждено.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>V-TECH SYSTEM</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[5] — сколько уходит на процедуру и хватает ли коробки на курс</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>«Сколько флаконов и саше уходит на одну процедуру и хватает ли одной коробки на курс? … сыворотки на процедуру 1–1,5 мл из флакона на 5 мл.»</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>«V-TECH Serum: עד 2 מ״ל» / «V-TECH Gel Mask: עד 2 מ״ל» на одну зону; «יש להשתמש באמפולה עד חודש ממועד הפתיחה, בהתאם להנחיות האחסון של המוצר.»; «טיפול אחד בכל 14 יום.» «סדרה מומלצת: 6-4טיפולים».</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:35-36, :56-57</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Ответ частичный. Протокол даёт дозу (до 2 мл сыворотки и до 2 мл гель-маски на одну зону) и срок: открытую ампулу использовать до месяца. Сколько коробок нужно на курс, в протоколе не сказано, поэтому набор и курс по-прежнему показываем отдельными фактами. В факты (экран 6 или 7) добавить срок после вскрытия — до месяца. В тексте вопроса заменить «1–1,5 мл» на «до 2 мл на зону», а курс «не меньше четырёх» — на «4–6».</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено, ответ частичный. Протокол даёт дозу на зону (:35), срок открытой ампулы — до месяца (:36), ритм и курс (:56–57). Сколько коробок нужно на курс, не сказано. Вопрос в сюжете опирается на «1–1,5 мл», а это вытеснено протоколом.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>V-TECH SYSTEM</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[6] — шаг 1: абстрактное поле или MITOPEN</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>«Шаг 1 протокола: оставить абстрактное поле микроканалов … или показать там MITOPEN как перекрёстную продажу?»</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Основной протокол называется «VTECH+ MITOPEN»: «יש ליישם את הסרום באמצעות MITOPEN / מזופן או מכשור מקצועי מתאים אחר.»; второй протокол — «BIOSPICULE™ MICROBOOST 10% + VTECH».</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:32, :41, :65</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>MITOPEN на шаге 1 — часть основного протокола заказчика, а не придуманная перекрёстная продажа. Можно назвать MITOPEN основным прибором (со ссылкой на его страницу) с подписью «או מזופן / מכשור מקצועי מתאים אחר». Для BIOSPICULE™ 10% остаётся свой протокол (см. находку 3). Открытым остаётся только одно: показывать ли сам прибор в 3D.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. Основной протокол называется «VTECH+ MITOPEN» (:32), на плитке ссылка «MITOPEN + VTECH» (:22), сыворотку наносят «באמצעות MITOPEN / מזופן או מכשור מקצועי מתאים אחר» (:41). Посылка вопроса («перекрёстная продажа») неверна: MITOPEN входит в протокол самого заказчика. Показывать ли прибор в 3D — по-прежнему решение по дизайну.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>V-TECH SYSTEM</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[7] — финиш: только EXOCELL MASK + SPF или и DERMA RECOVERY</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>«Финиш: в каталоге — «EXOCELL MASK или DERMA RECOVERY и защита от солнца», а в метке протокола на сайте только EXOCELL MASK + SPF … Попросить редактора иврита добавить DERMA RECOVERY в эту метку?»</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>«מומלץ להניח מסכת EXOCELL MASK…» → «בסיום DERMA RECOVERY CREAM» → «מקדם הגנה חובה»</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:51-53</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Да, DERMA RECOVERY CREAM добавить, и не через «или», а по порядку: EXOCELL MASK (рекомендуется) → DERMA RECOVERY CREAM → SPF (обязательно). Правка — в находке 2 (экран 5). Вопрос закрыть.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено (content.he.mjs:51–53; PLAN.md:118). Протокол даёт финиш последовательностью EXOCELL MASK → DERMA RECOVERY CREAM → SPF (обязательно), а не через «или». Это ответ на вопрос сюжета.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>V-TECH SYSTEM</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[1] — флакон или ампула в тексте</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>«Флакон или ампула? … в каталоге и текстах сайта — אמפולות. В 3D показываем как на фото. Слово в тексте оставляем или меняем?»</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Протокол: «יש להשתמש באמפולה עד חודש ממועד הפתיחה»; mitoderm.com: «5 אמפולות V-Tech Serum בנפח 5 מ׳׳ל כל אחת»; PLAN §7: «в коробке 5 ампул сыворотки по 5 мл»; только схема набора (фото 78/83) пишет «VIALS».</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:36; site/sources/mitoderm-com/products-he.json:11 (bundleText1); PLAN.md:119</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Протокол, сайт, каталог и слова заказчика в PLAN называют её ампулой, поэтому в тексте оставляем «אמפולות». Форма в 3D — как на фото (флакон). Вопрос снять.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В протоколе :36 — «יש להשתמש באמפולה עד חודש ממועד הפתיחה». На mitoderm.com (bundleText1): «5 אמפולות V-Tech Serum בנפח 5 מ׳׳ל כל אחת». В каталоге RU: «Сыворотка: 5 ампул × 5 мл». У заказчика в PLAN.md:79 и :119: «V-TECH — ампулы», «5 ампул сыворотки по 5 мл». «VIALS» есть только на схеме набора.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>EXO-NAD</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>b4.line и метки шагов b4.label1–3 (раскрытые шаги) — нет доз, времени и смывания</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>b4.line: «פילינג, נטרול והחדרת ה-Longevity Serum. טיפול בודד או סדרה, בכל ימות השנה; בסיום – EXOCELL MASK ומקדם הגנה.»; метки «1 · Biphasic Peel», «2 · pH Normalizer», «3 · Longevity Serum» — без доз и времени</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>«לפני השימוש יש לנער היטב את התמיסה הדו־פאזית.»; «אפשרות 1 – עור דק, רגיש או מעט מבוגר: יש לשאוב 1 מ״ל … יש להשאיר את התמיסה על העור עד 20 דקות»; «אפשרות 2 – עור עבה או מבוגר יותר: … 1 מ״ל … 15 דקות … 1 מ״ל נוסף … עד 15 דקות נוספות. זמן חשיפה כולל: עד 30 דקות.»; «יש לשאוב  1.5 -2 מ״ל מהמנטרל…» «יש להשאיר על העור למשך 2–3 דקות. לאחר מכן יש לשטוף היטב במים ולייבש את העור לחלוטין.»; «יש לשאוב כ 2 מל מ״ל מסרום ה־Longevity…» «יש לאפשר לסרום להיספג בעור. אין לשטוף.»; «יש להחליף כפפות, מחטים ומזרקים בין שלב לשלב»</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:167-179, :186 (exo-nad)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Добавить в метки шагов коротко время и смывание (это важно для безопасности), а дозы — в раскрытие шагов:
+- 1 — 1 мл пилинга до 20 мин (тонкая или чувствительная кожа); для плотной кожи 1 мл на 15 мин, затем ещё 1 мл до 15 мин, всего до 30 мин; перед работой встряхнуть.
+- 2 — 1,5–2 мл нейтрализатора на 2–3 мин, затем тщательно смыть водой и полностью высушить кожу.
+- 3 — около 2 мл Longevity Serum, нанести равномерно, дать впитаться, не смывать.
+Между шагами менять перчатки, иглы и шприцы. Слово «החדרת» в b4.line оставить: оно из каталога. Иврит — через переводчика.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Пропуск подтверждён. Протокол EXO-NAD (content.he.mjs:167–179, 186) даёт:
+- встряхнуть флакон;
+- 1 мл до 20 минут, а для плотной кожи — 1 мл на 15 минут и ещё 1 мл до 15 минут (всего до 30);
+- 1,5–2 мл нейтрализатора на 2–3 минуты, затем смыть и высушить;
+- около 2 мл Longevity Serum без смывания;
+- между шагами менять перчатки, иглы и шприцы.
+В сюжете метки только с названиями шагов, а страница V-TECH дозы показывает. Поправка к предложению: замену «החדרת» снимаю. Это слово каталога («ולבסוף החדרת סרום פעיל», source-texts.md), то есть вопрос стиля, а не ошибка.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>EXO-NAD</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>b4.label4 «בסיום: EXOCELL MASK + SPF» и финиш в b4.line</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>ошибка</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>b4.label4: «בסיום: EXOCELL MASK + SPF»; b4.line: «…בסיום – EXOCELL MASK ומקדם הגנה.»</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Каталог HE: «בסיום: exocell mask | DERMA RECOVERY»; каталог RU: «По завершении процедуры: Солнцезащитное средство / EXOCELL MASK | DERMA RECOVERY CREAM»; cta каталога: «בסיום הטיפול – EXOCELL MASK או DERMA RECOVERY CREAM ומקדם הגנה.» В протоколе EXO-NAD финиша нет; в протоколе EXOCELL MASK «פילינג» назван среди процедур, после которых ставится маска.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>source-texts.md:154; source-texts-ru-2026-09-18.md:208-211; site/product-pages.he.json (EXO-NAD, cta[1]); protocols/src/content.he.mjs:212</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Вернуть DERMA RECOVERY CREAM дословно по cta каталога: «בסיום הטיפול – EXOCELL MASK או DERMA RECOVERY CREAM ומקדם הגנה.» На маркере финиша дать вторую ссылку — на DERMA RECOVERY CREAM.</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В каталоге HE (source-texts.md:154) «בסיום: exocell mask | DERMA RECOVERY». В каталоге RU (:208–211) «Солнцезащитное средство / EXOCELL MASK | DERMA RECOVERY CREAM». В cta[1] каталога (product-pages.he.json, EXO-NAD) «בסיום הטיפול – EXOCELL MASK או DERMA RECOVERY CREAM ומקדם הגנה.» В протоколе EXO-NAD финиша нет. В протоколе EXOCELL MASK (:212) «פילינג» стоит среди процедур, после которых ставят маску. В сюжете b4.label4 и b4.line содержат только EXOCELL MASK + SPF, DERMA RECOVERY CREAM выпал.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>EXO-NAD</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>inside</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>inside.components[1].what и [2].what — цвет жидкости</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>ошибка</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>«pH Normalizer — флакон с янтарной жидкостью…», «Longevity Serum — флакон с голубой жидкостью…»</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>packaging-text.json: «amber vial» — «amber glass vial, silver crimp cap»; «teal vial» — «blue-teal glass vial, silver crimp cap»</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>site/packaging-text.json → exo-nad.objects[2], objects[3]</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Писать «флакон из янтарного стекла» (pH Normalizer) и «флакон из сине-бирюзового стекла» (Longevity Serum), оба с серебристым обжимным колпачком. Цвет самой жидкости в источниках не указан, в 3D его не придумывать.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В packaging-text.json (exo-nad.objects[2], [3]): «amber glass vial, silver crimp cap» и «blue-teal glass vial, silver crimp cap». Цветное здесь стекло, а не жидкость. В сюжете написано «флакон с янтарной жидкостью» и «флакон с голубой жидкостью». photo-catalog.md тоже говорит о цвете флаконов, не жидкости.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>EXO-NAD</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[4] — финиш протокола</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>«Финиш протокола: в раскадровке «EXOCELL MASK + SPF», в каталоге «EXOCELL MASK או DERMA RECOVERY CREAM ומקדם הגנה». Какой вариант верный?»</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Каталог HE «בסיום: exocell mask | DERMA RECOVERY»; RU «Солнцезащитное средство / EXOCELL MASK | DERMA RECOVERY CREAM». Протокол EXO-NAD финиша не называет и с каталогом не спорит.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>source-texts.md:154; source-texts-ru-2026-09-18.md:208-211</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Ответ на первую половину: верен вариант каталога — EXOCELL MASK или DERMA RECOVERY CREAM, плюс SPF. Добавляем вторую ссылку, на DERMA RECOVERY CREAM (правка — в находке 13). Вторая половина вопроса (не показывать саше MASK объектом) остаётся вопросом по дизайну.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено: все три текста каталога называют EXOCELL MASK и DERMA RECOVERY CREAM плюс SPF, протокол EXO-NAD финиша не называет и каталогу не противоречит. Поправка к предложению: «заказчику её можно не задавать» — это мнение, не вывод из источника. Вторая половина вопроса (саше MASK объектом не показываем) просто остаётся вопросом по дизайну.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>EXO-NAD</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[2] — сколько процедур на коробку (и экраны 6–7, где числа нет)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>«Сколько процедур рассчитано на одну коробку (15 мл пилинга, 5 + 5 флаконов по 5 мл)? В каталоге этого нет, поэтому на экране покупки число не пишем.»</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>«הערכה מאפשרת עד 15 טיפולים, בהתאם לכמות הנצרכת בכל טיפול.»; «לאחר הפתיחה ניתן להשתמש במוצר במשך עד חודש, באחסון במקום קריר ובהתאם להוראות האחסון.»</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:184-185 (exo-nad, «אחסון ושימוש לאחר פתיחה»)</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Ответ есть: набора хватает до 15 процедур, в зависимости от расхода на каждую. На экран 6 (факты) или 7 (что внутри) добавить «עד 15 טיפולים בערכה, בהתאם לכמות הנצרכת בכל טיפול» и срок после вскрытия: до месяца, хранить в прохладном месте. Вопрос закрыть.</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В content.he.mjs:184–185 «הערכה מאפשרת עד 15 טיפולים, בהתאם לכמות הנצרכת בכל טיפול.» и «לאחר הפתיחה ניתן להשתמש במוצר במשך עד חודש, באחסון במקום קריר…». В сюжете вопрос «В каталоге этого нет, поэтому … число не пишем» — а ответ есть в основном протоколе.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>EXO-NAD</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[5] — контакты экрана покупки и бейдж PEELING</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>«Контакты для экрана покупки: номер WhatsApp, телефон и e-mail. Бейдж линейки: «PEELING» латиницей, как BIOSPICULE, или на иврите…?»</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>contacts.json: «"phone": "054-326-2182"», «"whatsapp": "+972-54-762-1889"», «"email": "info@mitoderm.com"», «callback_time: null». Протокол на иврите называет семейство латиницей: «nav: 'PEELING', title: 'PEELING'».</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>site/sources/mitoderm-com/contacts.json:3-8; protocols/src/content.he.mjs:154; PLAN.md:117</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Контакты: WhatsApp +972-54-762-1889 (wa.me/972547621889), телефон 054-326-2182, info@mitoderm.com; срок обратного звонка не пишем. Бейдж — латиницей «PEELING», как в ивритской версии протоколов заказчика. Вопрос закрыть.</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. contacts.json: phone «054-326-2182», whatsapp «+972-54-762-1889», whatsapp_link «https://wa.me/972547621889», email «info@mitoderm.com», callback_time null. PLAN.md:117 повторяет это и запрещает срок обратного звонка. Протокол на иврите (:154) называет семейство латиницей: nav и title «PEELING».</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>EXOCELL MASK</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>b1.line и чипы b1.label2–5 — после каких процедур</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>b1.line «לאחר מיקרונידלינג, פילינגים וספיקולות, העור זקוק ללחות…»; чипы: V-TECH SYSTEM, פילינג EXO-NAD, MICRO BOOST 10%, מיקרונידלינג</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>«EXOCELL MASK מתאימה במיוחד כשלב מסיים ומרגיע לאחר טיפולים מקצועיים, לרבות:» chips: 'לייזר', 'פילינג', 'טיפולי הזרקה ופילרים', 'מזותרפיה רפואית', 'RF מיקרונידלינג', 'RF', 'מיקרונידלינג'</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:210-212 (exocell-mask, blocks[0])</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Добавить перечень из протокола строкой без ссылок под чипами (b1.line можно не трогать), дословно: «לייזר · פילינג · טיפולי הזרקה ופילרים · מזותרפיה רפואית · RF מיקרונידלינג · RF · מיקרונידלינג». Чипы-ссылки на свои средства оставить.</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В content.he.mjs:211–212: «EXOCELL MASK מתאימה במיוחד כשלב מסיים ומרגיע לאחר טיפולים מקצועיים, לרבות:» и чипы «לייזר, פילינג, טיפולי הזרקה ופילרים, מזותרפיה רפואית, RF מיקרונידלינג, RF, מיקרונידלינג». В сюжете b1.line «לאחר מיקרונידלינג, פילינגים וספיקולות» и четыре чипа своих средств. Лазер, инъекции и филлеры, мезотерапия и RF пропущены — а это заметная часть применения для клиник.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>EXOCELL MASK</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>b4.label2 «2 · ספיגה» и b4.line — нет времени экспозиции</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Метка «2 · ספיגה» без времени; в action_3d_ru и в вопросе 6: «В каталоге нет времени экспозиции маски, поэтому шаг «ספיגה» на экране 6 идёт без времени.»</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>«יש להשאיר את המסכה על העור למשך עד־30 דקות.» PLAN §7: «EXOCELL MASK — до 30 минут».</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:206 (exocell-mask, use.steps[1]); PLAN.md:118</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Метка шага 2: «2 · ספיגה · עד 30 דקות» (время из протокола: «למשך עד־30 דקות»). Иврит — через переводчика.</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В content.he.mjs:206 «יש להשאיר את המסכה על העור למשך עד־30 דקות.» (EN: «Leave the mask on the skin for up to 30 minutes.»). PLAN.md:118: «EXOCELL MASK — до 30 минут». В сюжете метка «2 · ספיגה» без времени, а в вопросе 6 стоит «В каталоге нет времени экспозиции».</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>EXOCELL MASK</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>b4.label3 «3 · סיום» — нет действия протокола</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>«3 · סיום» / «3 · Finish», без действия</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>«לאחר מכן יש להסיר את המסכה ולהספיג בעדינות את שאריות הסרום שנותרו על העור.»</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:207 (exocell-mask, use.steps[2])</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>В метке шага 3 сказать, что делают с остатком сыворотки, не выделяя снятие маски. Например: «3 · סיום · מספיגים בעדינות את שאריות הסרום לעור» — по фразе протокола «להספיג בעדינות את שאריות הסרום שנותרו על העור». Через переводчика и рецензентов.</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В content.he.mjs:207 «לאחר מכן יש להסיר את המסכה ולהספיג בעדינות את שאריות הסרום שנותרו על העור.» (EN :207 — «gently pat the remaining serum into the skin»). В сюжете метка «3 · סיום» без действия. Предложение соблюдает слово заказчика «Снятие не выделять» (PLAN.md:81).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>EXOCELL MASK</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>b6.line «לשימוש מקצועי בלבד.»; use: professional; inside.pro_only: true</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>источники расходятся</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>«לשימוש מקצועי בלבד.» / «For professional use only.»</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Протокол: «sub: 'פרוטוקול שימוש מקצועי וביתי'» (EN: «Professional and home-use protocol»). PLAN §7, слово заказчика 11/10: «В клинике её снимает специалист; клиент может пользоваться маской и после процедуры.» packaging-text: «clients can also use it after the procedure (owner, 11/10)». Каталог HE: «ניתן להשתמש בה גם כטיפול עצמאי לעור יבש, עייף, רגיש או חסר חיוניות.»</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:202; PLAN.md:81; site/packaging-text.json → exocell-mask.objects[3].look; source-texts.md:164</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>«Только для профессионального использования» противоречит слову заказчика и подзаголовку протокола «מקצועי וביתי». Убрать «בלבד»: маска — для клиник, а клиент может пользоваться ею и после процедуры. Формулировку на иврите сделать через переводчика и подтвердить у заказчика, потому что это заявление о продаже. Флаг inside.pro_only пересмотреть вместе с ней. Текст про двойную маску не трогаем.</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В подзаголовке протокола (:202) «פרוטוקול שימוש מקצועי וביתי» (EN: «Professional and home-use protocol»). Заказчик 11/10 (PLAN.md:81): «клиент может пользоваться маской и после процедуры»; то же в packaging-text exocell-mask.objects[3].look. Печатный каталог HE (source-texts.md:164) пишет «ניתן להשתמש בה גם כטיפול עצמאי…», а «לשימוש מקצועי בלבד» у EXOCELL в печатном тексте нет — оно есть только в веб-cta product-pages.he.json. В сюжете b6.line «לשימוש מקצועי בלבד.» и pro_only: true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>EXOCELL MASK</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[5] — время экспозиции</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>«В каталоге нет времени экспозиции маски, поэтому шаг «ספיגה» на экране 6 идёт без времени. Если в техлисте VM время есть, добавить?»</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>«יש להשאיר את המסכה על העור למשך עד־30 דקות.»</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs:206</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Ответ есть в основных протоколах заказчика: до 30 минут. Добавить в шаг 2 (находка 18), вопрос закрыть.</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено: в content.he.mjs:206 «יש להשאיר את המסכה על העור למשך עד־30 דקות.», в PLAN.md:118 — «EXOCELL MASK — до 30 минут». Вопрос сюжета исходит из того, что времени нет, а оно есть.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>EXOCELL MASK</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[6] — WhatsApp 054-762-1889 и телефон 054-326-2182</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>«Главная кнопка WhatsApp ведёт на номер 054-762-1889, а на экране 7 указан телефон 054-326-2182 (оба из site/proto/exocell-he-ui.json). Так и задумано?»</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>contacts.json: «"phone": "054-326-2182"», «"whatsapp": "+972-54-762-1889"», «"whatsapp_link": "https://wa.me/972547621889"»; «Owner 11/10: everything on mitoderm.com is correct»</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>site/sources/mitoderm-com/contacts.json:2-7; PLAN.md:117</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Да, так задумано: на mitoderm.com WhatsApp +972-54-762-1889, телефон 054-326-2182, почта info@mitoderm.com. Вопрос закрыть; срок обратного звонка нигде не писать.</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. contacts.json: «phone»: «054-326-2182», «whatsapp»: «+972-54-762-1889», «whatsapp_link»: «https://wa.me/972547621889»; в _source: «Owner 11/10: everything on mitoderm.com is correct». PLAN.md:117 — то же. Номер 054-762-1889 из сюжета совпадает с WhatsApp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL HAIR</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>b2.label4 + b2.line + inside.actives_text (витамины)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>источники расходятся</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>«ויטמינים B5 · B7 · B6 · B1» / «Vitamins B5 · B7 · B6 · B1»; в составе «Vitamins B5, B7, B6, B1»</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Каталог HE: «ויטמינים ורכיבים תומכים : פנתנול – פרו־ויטמין B5, ביוטיו– ויטמין B7 פירידוקסין – ויטמין B6 תיאמין – ויטמין B1»; каталог RU: «Витамины: Panthenol — провитамин B5, Biotin — витамин B7, Pyridoxine — витамин B6, Thiamine — витамин B1». mitoderm.com: «ויטמינים (פנתנול, גלוטתיון, ביוטין)» / «Vitamins (panthenol glutathione biotin)».</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/source-texts.md → Стр. 10 EXOSIGNAL HAIR; mitoderm-catalog/source-texts-ru-2026-09-18.md → Полоса 12; site/sources/mitoderm-com/products-he.json и products-en.json → solution.signal.item5</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Текст не менять: оставить B5 · B7 · B6 · B1, как в обеих печатных редакциях. Глутатион, который есть только на mitoderm.com, без подтверждения заказчика не добавлять. По желанию задать один короткий вопрос: входит ли глутатион в формулу (в лиде каталога есть «ויטמינים ונוגדי חמצון»).</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Цитаты точные. Печатный каталог на иврите: «פנתנול – פרו־ויטמין B5, ביוטיו– ויטמין B7 פירידוקסין – ויטמין B6 תיאמין – ויטמין B1». Русская версия называет те же четыре витамина. mitoderm.com: «ויטמינים (פנתנול, גלוטתיון, ביוטין)». Страница следует обеим печатным редакциям, ошибки на ней нет. Это расхождение источников только для сведения, текст менять не нужно.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL HAIR</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>b4.label3 + transition_ru 5→6 + story_one_line (ампула «израсходована в сеансе»; связано с вопросом 3 об отламывании горлышка)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>ошибка</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>b4.label3: «3 · החדרה · אמפולה אחת» / «3 · Apply · one ampoule»; переход 5→6: «открытая ампула гаснут и уходят назад в темноту: ампула израсходована в сеансе»; story_one_line: «в конце пять запечатанных ампул, пять сеансов, собираются в одну коробку»</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>«יש להשתמש בכ־2–1.5 מ״ל מהסרום, בהתאם לגודל האזור המטופל.» / «Use about 1.5-2 ml of serum…»; «לאחר הפתיחה יש לשמור את האמפולה בקירור. עמידות לאחר פתיחה: עד חודש.» / «After opening, keep the ampoule refrigerated. Shelf life after opening: up to one month.»</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/protocols/src/content.he.mjs / content.en.mjs → protocol id 'exosignal-hair': steps[2] и aside 'Storage'</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>b4.label3 — по дозе протокола: «3 · EXOSIGNAL HAIR · 1.5–2 מ״ל» / «3 · EXOSIGNAL HAIR · 1.5–2 ml». В переходе 5→6 не говорить, что ампула израсходована. Факт хранения дать на экране 6 или в карточке экрана 7 дословно: «לאחר הפתיחה יש לשמור את האמפולה בקירור. עמידות לאחר פתיחה: עד חודש.» В story_one_line вместо «пять сеансов» — «пять ампул по 5 мл в одной коробке». Вопрос 3 (как вскрывается ампула) задать заказчику вместе с фактом о хранении вскрытой ампулы, до сборки перехода 2→3.</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В истории b4.label3 — «3 · החדרה · אמפולה אחת» / «3 · Apply · one ampoule». Переход 5→6 говорит, что ампула «израсходована в сеансе», а story_one_line — «пять запечатанных ампул, пять сеансов». Протокол даёт дозу около 1,5–2 мл на процедуру и хранение вскрытой ампулы в холодильнике до месяца. Так что ампула за сеанс не расходуется. Как вскрывается ампула, источники не говорят. Но вскрытую ампулу хранят, поэтому сцену с отломанной и улетевшей головкой (вопрос 3) нужно согласовать.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL HAIR</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>b4.title + b4.line + b4.label1–3 + action_3d_ru (порядок шагов: сначала MITOPEN, потом средство)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>ошибка</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>«מודדים, פותחים, מחדירים» / «Measure, open, deliver»; «MITOSCAN קובע את נקודת הפתיחה, MITOPEN פותח את מסלול החדירה, EXOSIGNAL HAIR מוחדר לקרקפת המטופלת…» / «MITOSCAN sets the baseline, MITOPEN opens the pathway, EXOSIGNAL HAIR goes on the treated scalp…»; метки «1 · Diagnose · MITOSCAN», «2 · Microneedle · MITOPEN», «3 · Apply · one ampoule»</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Протокол: шаг 1 «יש לנקות היטב את אזור הקרקפת…», «ניתן לבצע את החיטוי…», «ניתן להשתמש במצלמת MITOSCAN  לסקירת הקרקפת , מצב הזקיקים, דלילות ודלקות»; шаг 2 «יש לייבש את אזור הטיפול לחלוטין»; шаг 3 «הטיפול מתבצע בשילוב MITOPEN / מזופן.», «עומק עבודה: עד 0.6 מ״מ, בהתאם לאזור, למצב הקרקפת ולאבחון המקצועי.», «בסימולטניות עוברים ביחד עם החומר והמכשיר . לחלק את העבודה לאזורים : קודם לטפטף מעט מהחומר על אזור מסוים ואז לעשות סטמפינג» / «Product and device work at the same time. Divide the work into sections: first drip a little product onto a section, then stamp.»; шаг 4 «לאחר העבודה יש לעסות עם הכפפות את הקרקפת בעדינות עד לספיגה מלאה של החומר.» Каталог (product-pages.json steps) даёт ту же неверную последовательность: «Scalp microneedling with MITOPEN creates the pathway for the actives.» → «EXOSIGNAL HAIR on the treated scalp» — побеждает протокол.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/protocols/src/content.he.mjs / content.en.mjs → protocol id 'exosignal-hair' steps[0..3]; mitoderm-catalog/site/product-pages.json → exosignal-hair.steps</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Шаги по протоколу. 1 — очищение и дезинфекция кожи головы; MITOSCAN по желанию, для осмотра кожи головы и фолликулов. 2 — полностью высушить. 3 — EXOSIGNAL HAIR и MITOPEN (или мезопен) одновременно: по участкам сначала капнуть немного средства, затем стемпинг; глубина до 0,6 мм, около 1,5–2 мл. 4 — помассировать кожу головы руками в перчатках до полного впитывания. Дома — EXOSIGNAL SPRAY. В 3D ампула и MITOPEN работают в одном шаге: капля на участок, затем стемпинг. Заголовок и фраза не должны говорить, что средство наносят после микронидлинга на уже обработанную кожу. Иврит брать из протокола, например «קודם לטפטף מעט מהחומר על אזור מסוים ואז לעשות סטמפינג».</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В истории (экран 5): «MITOPEN פותח את מסלול החדירה, EXOSIGNAL HAIR מוחדר לקרקפת המטופלת» / «…goes on the treated scalp», шаги идут по порядку: MITOSCAN → MITOPEN → ампула. В протоколе шаг 3 другой: «הטיפול מתבצע בשילוב MITOPEN / מזופן», «בסימולטניות עוברים ביחד עם החומר והמכשיר . לחלק את העבודה לאזורים : קודם לטפטף מעט מהחומר על אזור מסוים ואז לעשות סטמפינג». Значит, средство и прибор работают в одном шаге, и средство капают до стемпинга. Глубина — до 0,6 мм, затем массаж в перчатках до впитывания. MITOSCAN в шаге 1 стоит как «ניתן להשתמש», то есть по желанию. Порядок «сначала прибор» есть в product-pages.json и на mitoderm.com («לאחר פציעה מבוקרת מטפטפים את החומר»), но по порядку шагов главный источник — протокол.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL HAIR</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>частота и курс процедур (нет ни на одном экране)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Частоты процедур, числа процедур в курсе и поддерживающих процедур на странице нет; вместо курса — «пять сеансов» по числу ампул.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>«טיפול אחד בכל 14 יום.», «מומלץ לבצע לפחות 4 טיפולים רצופים.», «לאחר השלמת הסדרה ניתן לבצע טיפול תחזוקה אחת לחודשיים.» / «One treatment every 14 days.», «At least 4 consecutive treatments are recommended.», «After the course, a maintenance treatment can be done once every two months.»</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/protocols/src/content.he.mjs / content.en.mjs → protocol id 'exosignal-hair' → after 'תדירות וסדרת טיפולים / Frequency and treatment course'</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>На экран 5 или на экран 6 вместо «пяти сеансов» добавить строку курса дословно из протокола: «טיפול אחד בכל 14 יום · מומלץ לבצע לפחות 4 טיפולים רצופים · לאחר השלמת הסדרה ניתן לבצע טיפול תחזוקה אחת לחודשיים» / «One treatment every 14 days · at least 4 consecutive treatments · maintenance once every two months». По желанию добавить оговорку протокола «התדירות ומספר הטיפולים עשויים להשתנות…».</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. Ни на одном экране истории нет частоты процедур и длины курса. В протоколе exosignal-hair, в блоке «תדירות וסדרת טיפולים», дословно: «טיפול אחד בכל 14 יום.», «מומלץ לבצע לפחות 4 טיפולים רצופים.», «לאחר השלמת הסדרה ניתן לבצע טיפול תחזוקה אחת לחודשיים.» Для профессионального средства это важный факт протокола.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL HAIR</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>b5.title + b5.line + action_3d_ru («пять запечатанных ампул — курс из пяти сеансов», цифры 1–5 под ампулами)</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>ошибка</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>«חמישה טיפולים באריזה אחת» / «Five sessions in one box»; «חמש אמפולות זכוכית של 5 מ״ל – אחת לכל טיפול מקצועי – …» / «Five 5 ml glass ampoules — one per professional session — …»; 3D: «пять запечатанных ампул — курс из пяти сеансов. Под каждой цифра от 1 до 5»</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Протокол, шаг EXOSIGNAL HAIR SERUM: «יש להשתמש בכ־2–1.5 מ״ל מהסרום, בהתאם לגודל האזור המטופל.» / «Use about 1.5-2 ml of serum, depending on the size of the area.» Хранение: «לאחר הפתיחה יש לשמור את האמפולה בקירור. עמידות לאחר פתיחה: עד חודש.» / «After opening, keep the ampoule refrigerated. Shelf life after opening: up to one month.» Печать коробки: 'Net 5 x 5 ml ℮ 5 x 0.17 fl.oz.'</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/protocols/src/content.he.mjs и content.en.mjs → protocol id 'exosignal-hair': steps[2] 'EXOSIGNAL HAIR SERUM' и aside 'אחסון / Storage'; mitoderm-catalog/site/packaging-text.json → exosignal-hair → flat box</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Убрать «одна ампула — один сеанс» и «пять сеансов в коробке». Заголовок экрана 6 — о составе коробки, например «5 אמפולות × 5 מ״ל» / «5 ampoules × 5 ml», как на печати 'Net 5 x 5 ml'. b5.line: «חמש אמפולות זכוכית של 5 מ״ל», затем дословно из протокола «יש להשתמש בכ־2–1.5 מ״ל מהסרום, בהתאם לגודל האזור המטופל», затем PDRN 2% (20 מ״ג/מ״ל) и восемь пептидов. В 3D убрать цифры 1–5 и «курс из пяти сеансов». Если курс показывать, то протокольный: процедура раз в 14 дней, не меньше 4 подряд.</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В истории (экран 6) стоит «חמישה טיפולים באריזה אחת» / «Five sessions in one box», «אחת לכל טיפול מקצועי», а в 3D: «курс из пяти сеансов, цифры 1–5». Протокол exosignal-hair (content.he/en.mjs): шаг EXOSIGNAL HAIR SERUM — «יש להשתמש בכ־2–1.5 מ״ל מהסרום…», в aside — «לאחר הפתיחה יש לשמור את האמפולה בקירור. עמידות לאחר פתיחה: עד חודש.» Вскрытую ампулу 5 мл, значит, хранят и используют снова. При процедуре раз в 14 дней одна ампула идёт на 2–3 сеанса, а не на один. На коробке (packaging-text.json) напечатано 'Net 5 x 5 ml ℮ 5 x 0.17 fl.oz.'. «Один сеанс» встречается только в product-pages.json, а протокол важнее.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL HAIR</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>карточка «что внутри»: cat.kit[0][2]; inside.components[0].volume_dose</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>источники расходятся</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>cat.kit[0][2]: «5 מ״ל כל אחת – הפורמולה המלאה לקרקפת לטיפול מקצועי אחד.» / «5 ml each — the full scalp formula for one professional session.»; inside.volume_dose: «5 мл каждая, одна ампула на один профессиональный сеанс»</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Протокол: «יש להשתמש בכ־2–1.5 מ״ל מהסרום, בהתאם לגודל האזור המטופל.» и «לאחר הפתיחה יש לשמור את האמפולה בקירור. עמידות לאחר פתיחה: עד חודש.» Печатный каталог HE говорит только «תכולת האריזה: 5 אמפולות *5 מל», RU — «5 ампул × 5 мл»; mitoderm.com — «5 ml x 5 Ampules». «Один сеанс» есть только в product-pages.json.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/site/product-pages.json и product-pages.he.json → exosignal-hair.kit[0]; mitoderm-catalog/protocols/src/content.he.mjs → 'exosignal-hair' steps[2], aside; mitoderm-catalog/source-texts.md → Стр. 10; site/sources/mitoderm-com/products-he.json → solution.signal.item1</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>В карточке: «5× · אמפולות · 5 מ״ל כל אחת», без «לטיפול מקצועי אחד». По желанию добавить из протокола «כ־1.5–2 מ״ל לטיפול» и «לאחר הפתיחה – בקירור, עד חודש». inside.volume_dose: «5 мл каждая; на процедуру около 1,5–2 мл; после вскрытия — в холодильнике до одного месяца».</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. product-pages(.he).json → kit[0]: «5 מ״ל כל אחת – הפורמולה המלאה לקרקפת לטיפול מקצועי אחד.» / «…for one professional session». Печатный каталог говорит только «תכולת האריזה: 5 אמפולות *5 מל», русская версия — «5 ампул × 5 мл», mitoderm.com — «5 ml x 5 Ampules». Протокол даёт 1,5–2 мл на процедуру и хранение вскрытой ампулы до месяца. Источники расходятся, и по процедуре прав протокол.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL HAIR</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[0] (фото коробки, открытая коробка с вкладышем) + assets (торцы коробки «needs photo», крупная ампула «needs photo») + экран 6 «фото вкладыша нет»</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>«Нужны фото коробки: фасад без ампул…, торцы, задняя сторона, глубина, а также открытая коробка с вкладышем»; экран 6: «Внутренность коробки не показываем: фото вкладыша нет.»</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>«| 36, 47 | 113:8145, 113:8164 | EXOSIGNAL HAIR | чёрная коробка с золотым «EXOSIGNAL HAIR» | текстура коробки |» и «| 55, 58 | 113:8174, 113:8177 | EXOSIGNAL HAIR | открытая чёрная коробка со стеклянными ампулами | раскрытие набора, 3D-ампулы |»</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/site/photo-catalog.md → строки 36, 47 и 55, 58</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Фото заказчика уже есть в Figma: коробка (113:8145, 113:8164) и открытая коробка со стеклянными ампулами (113:8174, 113:8177). Сначала посмотреть по ним фасад без ампул, торцы, вкладыш и ампулы крупно. У заказчика спрашивать только то, чего на этих снимках нет. Сцену с открытой коробкой на экранах 6–7 можно вернуть по фото 55/58.</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В photo-catalog.md есть строки «36, 47 | 113:8145, 113:8164 | EXOSIGNAL HAIR | чёрная коробка с золотым «EXOSIGNAL HAIR» | текстура коробки» и «55, 58 | 113:8174, 113:8177 | … открытая чёрная коробка со стеклянными ампулами | раскрытие набора, 3D-ампулы». Сборщик (story3d_xlsx.py, PHOTOS) тоже относит к этой странице фото 36, 47, 55, 58. А история говорит «фото вкладыша нет» и просит у заказчика открытую коробку. Есть ли на этих снимках торцы и фасад без ампул, неизвестно, поэтому сначала их нужно посмотреть.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL SPRAY</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>kicker (ui.line_mark + ui.line_name + ui.use_home), то же на экранах 2 и 7</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>ошибка</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>«V-TECH FACE · התחדשות הפנים · טיפוח ביתי» / «V-TECH FACE»</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>product-pages.he.json: «eyebrow»: «טיפוח ביתי · קרקפת»; product-pages.json: «filter»: «Hair», «eyebrow»: «HOME CARE · SCALP»; каталог: «ספריי ביתי מתקדם לטיפוח הקרקפת ולתמיכה בשיער». В самом сюжете new_strings: ui.line_mark = «HAIR».</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/site/product-pages.he.json и product-pages.json → EXOSIGNAL SPRAY; mitoderm-catalog/source-texts.md → Стр. 18; site/proto/exocell-he-ui.json (line_mark «V-TECH FACE», line_name «התחדשות הפנים»)</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Для спрея значения ui.line_mark и ui.line_name из строк страницы (story3d.json: «HAIR» и вычитанное «שיער וקרקפת», ждёт вопроса 8) должны иметь приоритет над UI-файлом MASK. Это правка в resolve() или отдельный UI-файл спрея. До ответа заказчика ui.line_name не брать у MASK: ставить «שיער וקרקפת» с пометкой «на ответе» или показывать только «HAIR» + «טיפוח ביתי».</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В истории спрея кикер экрана 1 разрешился в «V-TECH FACE · התחדשות הפנים · טיפוח ביתי» / «V-TECH FACE», хотя в new_strings стоит ui.line_mark = «HAIR». Причина в коде: resolve() в story3d_xlsx.py берёт все ключи ui.* только из UI-файла MASK (exocell-he-ui.json: line_mark «V-TECH FACE», line_name «התחדשות הפנים»). Строки самой страницы спрея ему не видны, хотя в story3d.json для спрея уже есть HE «HAIR» и «שיער וקרקפת». Ошибка повторится в бейджах экранов 2 и 7. Средство для кожи головы подписано линейкой для лица. Предложение находки поставить «טיפוח ביתי · קרקפת» продублировало бы «טיפוח ביתי»: эта надпись уже есть в бейдже ui.use_home.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL SPRAY</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>b4.line + b4.label1–3 (как применять)</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>«לחלק את השיער כדי לחשוף את הקרקפת, להתיז ישירות עליה ולעסות בעדינות – ללא צורך בשטיפה. מדי יום…» / «Part the hair…, spray directly on, massage lightly — no rinsing. Daily…»; шаги «1 · Part · 2 · Spray · 3 · Massage»</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm.com: «פעם ביום, על קרקפת נקייה ויבשה. לנער לפני השימוש ולהתיז על האזור הרצוי בשורשים. לעסות בעדינות לפיזור. מומלץ בערב, למשך חודשיים.» / «Once a day, on a clean and dry scalp. Shake before use and spray on the desired area at the roots. Gently massage to distribute. Recommended for evening use, for a duration of two months.»</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/site/sources/mitoderm-com/products-he.json и products-en.json → solution.hair.bundleText2</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Дополнить способ применения данными mitoderm.com. Например, b4.line: «פעם ביום, על קרקפת נקייה ויבשה. לנער לפני השימוש, לחלק את השיער ולהתיז על האזור הרצוי בשורשים, לעסות בעדינות – ללא צורך בשטיפה. מומלץ בערב, למשך חודשיים.» Шаги можно начать с «לנער».</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В протоколах спрея нет. На mitoderm.com (products-he/en.json → solution.hair.bundleText2): «פעם ביום, על קרקפת נקייה ויבשה. לנער לפני השימוש ולהתיז על האזור הרצוי בשורשים. לעסות בעדינות לפיזור. מומלץ בערב, למשך חודשיים.» В b4.line истории есть только «разделить волосы → распылить → помассировать, без смывания, ежедневно». Нет того, что встряхивать, наносить на чистую сухую кожу у корней, раз в день, лучше вечером и курсом два месяца. Каталогу это не противоречит.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL SPRAY</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[6] (состав спрея) + inside.actives_key + экран 3 / карточка экрана 7</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>«Есть ли состав спрея (INCI или активы)? В каталоге есть только «что делает спрей»…»; inside.actives_key: «в каталоге только «что делает спрей», INCI нет»</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm.com: «קומפלקס פעיל לטיפול יומיומי»: «15 מל», «אקסוזומים סינתטיים», «PDRN במשקל מולקולרי נמוך», «פנתנול», «ביוטין», «פפטידים ביומימטיים 8 סוגים» / «Active complex for daily treatment»: «15 ml», «Synthetic exosomes», «PDRN with low molecular weight», «Panthenol», «Biotin», «Biomimetic peptides 8 types»</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/site/sources/mitoderm-com/products-he.json и products-en.json → solution.hair.itemTitle, item1–item6</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Вопрос снять. В карточку «מה בפנים» (экран 7) и на экран 3 добавить подзаголовок «רכיבים פעילים» и список с mitoderm.com: «אקסוזומים סינתטיים · PDRN במשקל מולקולרי נמוך · פנתנול · ביוטין · פפטידים ביומימטיים 8 סוגים». Блок «מה הספריי עושה» можно оставить рядом.</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. Вопрос 7 истории («Есть ли состав спрея…? В каталоге только «что делает спрей»») закрывается mitoderm.com. В solution.hair (это ExoSignal Hair Spray, «בקבוק ספריי 15 מל») есть «קומפלקס פעיל לטיפול יומיומי» со списком: «אקסוזומים סינתטיים», «PDRN במשקל מולקולרי נמוך», «פנתנול», «ביוטין», «פפטידים ביומימטיים 8 סוגים». Английская версия совпадает.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL SPRAY</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[5] (нажатий на нанесение, на сколько хватает 15 мл)</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>«Сколько нажатий нужно на одно нанесение и на сколько хватает 15 мл? В каталоге этого нет, поэтому на странице пишем только «15 מ״ל, ежедневно, без смывания»»</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm.com: «פעם ביום, … מומלץ בערב, למשך חודשיים.» / «Once a day, … Recommended for evening use, for a duration of two months.»</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/site/sources/mitoderm-com/products-he.json и products-en.json → solution.hair.bundleText2</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Частота (раз в день, лучше вечером) и курс (два месяца) есть на mitoderm.com — их можно писать на экранах 5–6. Заказчику оставить только вопрос о числе нажатий на одно нанесение.</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Частично подтверждено. Вопрос 6 истории: «Сколько нажатий на одно нанесение и на сколько хватает 15 мл?» На mitoderm.com: «פעם ביום… מומלץ בערב, למשך חודשיים» — раз в день, лучше вечером, курс два месяца. Числа нажатий нет ни в одном источнике. Находка это и говорит и не утверждает, что 15 мл точно хватает на два месяца.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL SPRAY</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[0] (студийный пакшот) + assets: коробка «Фасад есть только на site/img/exosignal-spray.png», флакон «needs photo»</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>«Студийного пакшота EXOSIGNAL SPRAY нет… Пришлите его в чат или положите в Drive /products»; assets: «Фасад есть только на site/img/exosignal-spray.png (400×300…)»</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>«| 2, 3, 21 | 93:8081, 93:8083, 104:8121 | EXOSIGNAL SPRAY HOME | чёрная коробка с золотом + матовый флакон с золотой крышкой (белый фон) | пакшот спрея (замена слабого 49:6) |» и «| 33, 34, 41, 43, 59, 65 | 113:8141 … 113:8185 | EXOSIGNAL SPRAY HOME | матовый флакон, чёрная коробка; 65 — интерьерная сцена | пакшот, сцена |»</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/site/photo-catalog.md → строки 2, 3, 21 и 33, 34, 41, 43, 59, 65</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Фото заказчика (коробка + матовый флакон с золотым колпачком) уже есть в Figma: 93:8081, 93:8083, 104:8121 на белом фоне и 113:8141…113:8185. Фасад коробки и этикетку флакона брать с них, а не с exosignal-spray.png. У заказчика просить только то, чего на этих снимках не окажется после проверки: например, распылитель без колпачка, оборот флакона, бок и верх коробки.</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. В photo-catalog.md есть строки «2, 3, 21 | 93:8081, 93:8083, 104:8121 | EXOSIGNAL SPRAY HOME | чёрная коробка с золотом + матовый флакон с золотой крышкой (белый фон) | пакшот спрея» и «33, 34, 41, 43, 59, 65 | 113:8141 … 113:8185 | … матовый флакон, чёрная коробка». Сборщик тоже относит их к спрею (PHOTOS). А история пишет, что студийного пакшота нет, просит прислать его в чат или Drive и берёт фасад коробки со скриншота exosignal-spray.png 400×300.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL SPRAY</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[3] (фото с человеком exosignal-spray-hand.jpg в публичном репозитории)</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>«…это фото с человеком, и оно уже лежит в публичном репозитории… Убрать его из репозитория и хранить копию только локально?»</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>«Сами фото в репозиторий не кладутся: на части из них люди, репозиторий публичный.»; «**«люди»** — фото с людьми: в публичные файлы и рендеры не идёт, только в Figma и только с согласия заказчика.»</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/site/photo-catalog.md → вводный абзац; файл в git: mitoderm-catalog/site/img/exosignal-spray-hand.jpg (на фото щека, волосы и рука)</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Вопрос не задавать: решение заказчика уже есть. Убрать site/img/exosignal-spray-hand.jpg из репозитория, копию держать локально или в Figma. Ссылки в packaging-text.json/.md и story3d.json перевести на фото 93:8081 / 93:8083 / 104:8121, этикетку брать с них.</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. Файл mitoderm-catalog/site/img/exosignal-spray-hand.jpg лежит в git (git ls-files). На нём щека, шея, волосы и рука человека — проверено просмотром. Правило заказчика уже есть: photo-catalog.md — «Сами фото в репозиторий не кладутся: на части из них люди, репозиторий публичный», «люди… в публичные файлы и рендеры не идёт»; CLAUDE.md проекта — «Не в репозиторий: … фото с людьми». В репозитории на файл ссылаются только тексты: packaging-text.json/.md и story3d.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>EXOTECH GEL</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>b4.line + b4.label4 (с чем и когда применять)</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>«…משתלב עם V-TECH, EXO-NAD וסדרת BIOSPICULE™.» / «Works with V-TECH, EXO-NAD and the BIOSPICULE™ line.»; экран 2: «לאחר טיפול בקליניקה» / «After in-clinic treatments»</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Протокол (домашний протокол поддержки): «ניתן להשתמש באקסוטק גל לשימור התוצאה של האקסוזומים מיד לאחר סדרת ביומיקרונידלינג» / «EXOTECH GEL can be used to preserve the exosome results immediately after a biomicroneedling course.»; протокол BIOSPICULE MICRO BOOST 10% + V-TECH: «לבית ניתן להמליץ את הסדרה הביתית של ביוספיקול לחידוש , אקסוטק גל ללחות מיטבית וקרם רקברי להזנה ולחות אינטנסיבית.»</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/protocols/src/content.he.mjs / content.en.mjs → protocol 'exocell-mask' → home.maintain; protocol 'biospicule-vtech' → aside</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Добавить факт протокола дословно. Например, b4.line: «…בוקר וערב. ניתן להשתמש באקסוטק גל לשימור התוצאה של האקסוזומים מיד לאחר סדרת ביומיקרונידלינג.» По желанию добавить из протокола BIOSPICULE MICRO BOOST 10% + V-TECH: «אקסוטק גל ללחות מיטבית» в домашнем уходе после процедуры.</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждено. Протокол exocell-mask → home.maintain: «ניתן להשתמש באקסוטק גל לשימור התוצאה של האקסוזומים מיד לאחר סדרת ביומיקרונידלינג». Протокол biospicule-vtech, aside: «לבית ניתן להמליץ את הסדרה הביתית של ביוספיקול לחידוש , אקסוטק גל ללחות מיטבית…». В истории есть только общее «לאחר טיפול בקליניקה» и «משתלב עם V-TECH, EXO-NAD וסדרת BIOSPICULE™». Протокольного момента применения — сразу после курса биомикронидлинга, чтобы сохранить результат экзосом — нет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>EXOTECH GEL</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[2] (фото куба и сферы в высоком разрешении, другие грани; объём 30 мл)</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>«Есть ли исходные фото куба и сферы в высоком разрешении…? И что напечатано на тыльной, правой и нижней гранях куба…? Объём 30 ml на видимых сторонах не виден, сейчас он взят из каталога.»</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>photo-catalog: «| 37, 38 | 113:8153, 113:8154 | EXOTECH GEL | золотой куб-коробка «EXOTECH GEL» | 3D-коробка |»; манифест фото каталога: «EXOTECH GEL (шар + коробка, 2 ракурса) | 2 фото»; mitoderm.com: «item1»: «30 ml», «bundleText1»: «V-Tech Gel 30 ml».</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/site/photo-catalog.md → строки 37, 38; mitoderm-catalog/source-texts.md → Приложение B; site/sources/mitoderm-com/products-en.json → solution.gel</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Сначала проверить в Figma два ракурса куба заказчика (113:8153, 113:8154): разрешение и видимые грани. Объём 30 мл подтверждён каталогом и mitoderm.com. У заказчика спрашивать только то, чего на этих фото нет: вероятно, тыльную, правую и нижнюю грани куба и обратную сторону сферы.</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Частично подтверждено. В photo-catalog.md есть строка «37, 38 | 113:8153, 113:8154 | EXOTECH GEL | золотой куб-коробка «EXOTECH GEL» | 3D-коробка», сборщик тоже относит фото 37, 38 к этой странице. История берёт куб только с protocols/print/img/exotech-gel.webp и просит у заказчика исходники. Объём 30 мл, кроме каталога, подтверждён mitoderm.com («item1»: «30 ml», «V-Tech Gel 30 ml»). Есть ли на фото 37/38 сфера, обратные грани и высокое разрешение, неизвестно, поэтому их нужно сначала проверить.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>MICRO BOOST 10%</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>b3.label2 «עד 72 שעות»; b3.line; b5.label4</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>источники расходятся</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>«...הספיקולות עשויות להמשיך לעורר את העור עד 72 שעות לאחר שהמטופלת עוזבת»</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Протокол: 'הספיקולות עשויות להישאר בשכבות החיצוניות של העור עד 72 שעות.' Русский каталог: 'Микроспикулы могут сохраняться в коже до 72 часов'. Ивритский каталог, разворот стр. 12–13: 'מיקרו-מחטים ביולוגיות נשארות בעור עד 24 שעות'.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs, протокол biospicule-vtech, строка 97; source-texts-ru-2026-09-18.md, строка 363; source-texts.md, стр. 12–13, строка 269</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>На странице MICRO BOOST 10% ничего не менять: «עד 72 שעות» совпадает с протоколом и русским каталогом, текущая формулировка b3.line подтверждена. Цифру 24 ч нигде на сайте не использовать (страница BIOSPICULE уже на 72 ч). Владельцу сообщить, что в печатном ивритском каталоге на развороте стр. 12–13 стоит «עד 24 שעות», а протокол и русский каталог говорят 72 ч: вероятно, это ошибка печати.</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Расхождение есть. Протокол (строка 97) и русский каталог (строки 323, 363) — до 72 ч, ивритский каталог (разворот стр. 12–13, строка 269) — «עד 24 שעות». По процедуре решает протокол, так что 72 ч на странице верно. Поправка: переписывать b3.line ближе к протоколу не нужно. Формулировка «עשויות להמשיך לעורר את העור עד 72 שעות» опирается на русский каталог («могут сохраняться в коже до 72 часов, продолжая механическую стимуляцию») и на product-pages («להמשך גירוי וחידוש»), и смена слов — вопрос стиля.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>MICRO BOOST 10%</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>b4.label4 «+ DERMA RECOVERY בבית»; cat.steps[2][1]; b4.line</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>ошибка</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Метка «+ DERMA RECOVERY בבית» / «+ DERMA RECOVERY at home»; cat.steps[2][1]: «V-TECH או Longevity Serum, לאחר מכן EXOCELL MASK; בבית – DERMA RECOVERY CREAM ומקדם הגנה». DERMA RECOVERY CREAM показан только как домашний шаг, SPF 30 на экране не назван.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Протокол, «סיום הטיפול»: 'EXOCELL MASK  כמסכת סיום ושיקום' · 'DERMA RECOVERY CREAM להשלמת לחות הזנה ותמיכה במחסום העורי' · 'SPF   מסנן קרינה של 30 לפחות חובה' (EN: 'DERMA RECOVERY CREAM to complete hydration and nourishment and support the skin barrier', 'SPF 30 or higher sunscreen, mandatory'). Каталог, стр. 14: 'Derma Recovery סיום טיפול ובבית – חובה לאחר הטיפול לתמיכה במחסום הלחות ולהפחתת תחושת יובש ומתיחה'.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs, протокол biospicule-vtech, after «סיום הטיפול», строки 89–91; source-texts.md, стр. 14, строка 299</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Протокол и оба каталога ставят DERMA RECOVERY CREAM в финал процедуры в клинике, после EXOCELL MASK, и делают его обязательным дома. Метку b4.label4 заменить по смыслу каталога («סיום טיפול ובבית»), например «+ DERMA RECOVERY בסיום הטיפול ובבית». В cat.steps[2][1] финиш дать в порядке протокола: EXOCELL MASK → DERMA RECOVERY CREAM → מסנן קרינה SPF 30 לפחות (חובה). Защиту не переносить в «בבית». В b4.line микроканалы оставить для V-TECH / Longevity Serum, а EXOCELL MASK назвать финишной маской: протокол «כמסכת סיום ושיקום», русский каталог «Завершение процедуры».</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Цитаты точные (content.he.mjs стр. 89–91, source-texts.md стр. 14, строка 299). Русский каталог подтверждает: «Завершение процедуры: EXOCELL MASK / DERMA RECOVERY CREAM — также обязательное домашнее применение / Солнцезащитное средство». В ивритском каталоге есть ещё «הגנה בסיום טיפול». В сюжете метка «+ DERMA RECOVERY בבית», а cat.steps[2][1] (product-pages.he.json) — «בבית – DERMA RECOVERY CREAM ומקדם הגנה»: крем и защита уходят домой, SPF 30 не назван. По протоколу и обоим каталогам это ошибка.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>MICRO BOOST 10%</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>b4.line; cat.steps[2][1] (активный продукт после MICRO BOOST)</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>«...the open micro-pathways then carry V-TECH or Longevity Serum and EXOCELL MASK» / «...מובילים פנימה את V-TECH או Longevity Serum ואת EXOCELL MASK». Есть два варианта, MITOTECH CELL BOOST не упомянут.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>'לאחר ספיגת MICRO BOOST 10% ניתן, בהתאם לפרוטוקול שנבחר, לבחור בחומרים פעילים כגון:' — ['V-TECH Serum + V-TECH Gel Mask', 'MITOTECH CELL BOOST', 'LONGEVITY SERUM']. У владельца есть и отдельный протокол 'BIOSPICULE BOOST 10% + MITOTECH CELL BOOSTER': 'באמצעות גל הביוספיקולות – יש למרוח 1.5-2 מל על אזור הפנים ומיד לאחר הספיגה להניח את הcell  booster'.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs, протокол biospicule-vtech, шаг «שילוב חומרים פעילים», строки 83–84; протокол cell-booster, строка 109</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>В шаге 3 и b4.line перечислить варианты из протокола: «V-TECH Serum + V-TECH Gel Mask · MITOTECH CELL BOOSTER · LONGEVITY SERUM». Название брать по глоссарию, в протоколе оно написано «MITOTECH CELL BOOST». V-TECH давать парой «сыворотка + гель-маска». MITOTECH CELL BOOSTER — только текстом, без 3D: пакшота нет, на главной он идёт карточкой «בקרוב». Ссылку вести на эту карточку, а не на страницу: страницы нет.</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Цитаты точные: строки 83–84 (три варианта) и строка 109 (протокол BIOSPICULE BOOST 10% + MITOTECH CELL BOOSTER). В b4.line сюжета названы только «V-TECH או Longevity Serum ואת EXOCELL MASK», V-TECH одним словом. Отдельный протокол владельца MICRO BOOST + CELL BOOSTER — одна из двух официальных связок MICRO BOOST, на странице её нет. Список в протоколе открытый («כגון»), но вторая связка — отдельный протокол владельца. Средство описано в PLAN как новое, пакшота нет, на главной оно карточкой «скоро».</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>MICRO BOOST 10%</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Курс и частота процедур (нет ни на одном экране)</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>На экранах 5–7 не сказано, сколько процедур в курсе и с каким интервалом.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>'ניתן לבצע סדרה של 4–3 טיפולים, במרווח של 4 שבועות בין טיפול לטיפול.' · 'לאחר השלמת הסדרה ניתן לבצע טיפול תחזוקה בהתאם להערכת מצב העור, מטרות הטיפול ותגובת המטופל/ת.' (EN: 'A course of 3-4 treatments, 4 weeks apart.')</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs, протокол biospicule-vtech, aside «סדרת טיפולים», строки 69–70</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>На экран 5 добавить строку из протокола: «סדרה של 4–3 טיפולים, במרווח של 4 שבועות בין טיפול לטיפול; לאחר מכן ניתן לבצע טיפול תחזוקה בהתאם להערכת מצב העור». Это может быть отдельная строка или описание шага, раскрываемое тапом. Частоту V-TECH («каждые 14 дней», курс 4–6) сюда не переносить: у связки с MICRO BOOST интервал 4 недели.</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Цитата точная (строки 69–70, EN строка 68). Ни в одном тексте сюжета MICRO BOOST (экраны 1–7, inside) нет числа процедур и интервала. Для профессионального средства это ключевой параметр протокола, а протоколы владельца решают по частоте и длине курса.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>MICRO BOOST 10%</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Домашний уход после процедуры (b4.label4, cat.cta[1] на экране 7)</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Из домашнего ухода назван только DERMA RECOVERY CREAM.</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>'לבית ניתן להמליץ את הסדרה הביתית של ביוספיקול לחידוש , אקסוטק גל ללחות מיטבית וקרם רקברי להזנה ולחות אינטנסיבית.' (EN: 'For home use, recommend the BIOSPICULE home series for renewal, EXOTECH GEL for optimal hydration and DERMA RECOVERY CREAM for intensive nourishment and hydration.')</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs, протокол biospicule-vtech, aside «סדרת טיפולים», строка 71</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Домашние рекомендации после MICRO BOOST 10% дать по протоколу: домашняя серия BIOSPICULE (CELL RENEW 1.5% / CELLULAR AGE DEFENSE 2.5%) для обновления, EXOTECH GEL для увлажнения, DERMA RECOVERY CREAM для питания и увлажнения. Показать текстом со ссылками на страницы. EXOTECH GEL в 3D не показывать (другая линейка), в 3D оставить мини-коробку DERMA, как в сюжете.</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Цитата точная (строка 71, EN строка 70). На экранах 5–7 сюжета из домашнего ухода назван только DERMA RECOVERY CREAM (b4.label4, cat.steps[2][1]). Протокол рекомендует три средства. Поправка к предложению: CELL RENEW / CAD 2.5% тоже из линейки BIOSPICULE, другая линейка только у EXOTECH GEL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>MICRO BOOST 10%</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>b5.title «מזרק אחד. טיפול אחד.»; b5.line; inside.components[0].volume_dose; экран 5, шаг 1 («цифр и шкалы нет»)</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>«One syringe. One treatment.» / «3 ml ... professional dose control for one in-clinic treatment»; inside: «3 мл на одну процедуру в клинике. Количество... задаёт специалист»; доза на экранах нигде не названа.</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Протокол владельца (BIOSPICULE BOOST 10% + CELL BOOSTER): 'באמצעות גל הביוספיקולות – יש למרוח 1.5-2 מל על אזור הפנים' (EN: 'with the biospicule gel: apply 1.5-2 ml to the face'). В печатном каталоге про шприц сказано только: 'ומגיע במזרק של 3 מ״ל, המאפשר לקוסמטיקאית לשלוט בכמות החומר'. Слов «на одну процедуру» в каталоге нет, они есть только в черновике сайта product-pages kit.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs, протокол cell-booster, строка 109; source-texts.md, стр. 14, строка 280; site/product-pages.he.json, MICRO BOOST kit[0]</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Указать дозу из протокола владельца: «1.5–2 מ״ל לאזור הפנים». Её поставить в шаг 1 на экране 5 (по тапу) и в inside.volume_dose вместо «3 мл на одну процедуру»; «3 ml ℮ 0.10 fl.oz.» — это объём шприца по печати. Заголовок «מזרק אחד. טיפול אחד.» и «לטיפול אחד בקליניקה» в b5.line снять или заменить фактом печати. У владельца спросить, на сколько процедур и зон (лицо или лицо + шея + декольте) рассчитан шприц и подходит ли доза 1.5–2 мл для связки с V-TECH.</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Цитата точная (строка 109). «גל הביוספיקולות» в протоколе MITOPEN/BIOSPICULE CELL BOOSTER 10% — это MICRO BOOST 10%: в шапке протокола «10%» и картинка micro-boost-10. Печатные каталоги HE и RU говорят только про шприц 3 мл и контроль количества, слов «на одну процедуру» в них нет. Они есть только в kit сайта product-pages, а project-council уже отметил «единицу продажи — шприц 3 ml» как допущение. При 1.5–2 мл на лицо из шприца 3 мл «один шприц — одна процедура» не следует ни из одного источника. Уточнение: доза взята из протокола связки с CELL BOOSTER, в основном протоколе MICRO BOOST + V-TECH числа нет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>MICRO BOOST 10%</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[4]; b5.line «3 ml ℮ 0.10 fl. oz.»</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>«В b5.line написано «3 ml ℮ 0.10 fl. oz.» с пробелом, а на коробке «fl.oz.». Привести строку к печати?»</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>"bottom: '3 ml ℮ 0.10 fl.oz.'"</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>site/packaging-text.json, micro-boost-10 → front, строка 47</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Да, привести к печати. В b5.line (HE и EN) писать «3 ml ℮ 0.10 fl.oz.» без пробела в «fl.oz.». Вопрос 5 заказчику снять, правку внести через редактора иврита.</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>packaging-text.json, строка 47: «bottom: '3 ml ℮ 0.10 fl.oz.'». На пакшоте protocols/print/img/micro-boost-10.webp (нижняя строка в увеличении) тоже «3 ml ℮ 0.10 fl.oz.» без пробела. Источник по объёмам однозначен, вопрос заказчику не нужен.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>CELL RENEW 1.5%</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Когда начинать после процедуры в клинике (b1.line «בין הביקורים», b4.line)</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Страница продаёт средство для дома «между визитами» и называет кислоты в формуле (b2.line «חומצה סליצילית + חומצה ציטרית»). Паузы после процедуры в клинике на странице нет.</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Протокол, домашние правила после процедуры: 'אין להשתמש בחומצות, רטינואידים, בנזואיל פרוקסיד, פילינג גרגרים או תכשירים מגרים במשך 5–7 ימים, או עד שהעור חזר למצבו ולתחושתו הרגילים.' Каталог: 'Salicylic Acid + Citric Acid'.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>protocols/src/content.he.mjs, exocell-mask → home.cards «חומרים פעילים», строка 223; source-texts.md, стр. 19</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Задать владельцу вопрос до публикации: распространяется ли правило протокола «אין להשתמש בחומצות… במשך 5–7 ימים, או עד שהעור חזר למצבו ולתחושתו הרגילים» на CELL RENEW 1.5% (в составе салициловая и лимонная кислоты, спикулы) и на CAD 2.5% (спикулы, Bakuchiol)? Если да, на экран 5 (или мелко на экран 7) добавить строку: «לאחר טיפול בקליניקה – לא לפני 5–7 ימים, או עד שהעור חזר למצבו ולתחושתו הרגילים». До ответа текст не добавлять.</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Цитаты точные: строка 223 протокола (запрет на кислоты и раздражающие средства на 5–7 дней) и состав каталога (Salicylic Acid + Citric Acid). Страница позиционирует средство «בין הביקורים» (b1.line), а паузы после процедуры в клинике нет. Правило стоит в блоке домашних инструкций протокола EXOCELL MASK. Там же предлагается домашняя серия BIOSPICULE 1.5%/2.5% для поддержки, но без срока начала. Значит, распространяется ли правило на CELL RENEW, решает только владелец. Это вопрос к нему, а не готовый текст.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>CELL RENEW 1.5%</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>b6.cta / ссылка «לקליניקות: לקבלת הצעת מחיר» → шаблон ui.wa_text_price</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>ошибка</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>«...открывает WhatsApp с текстом по шаблону wa_text_price. Оба шаблона берём из proto/exocell-he-ui.json с именем CELL RENEW 1.5%»</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>"wa_text_price": "שלום, אשמח לקבל פרטים על מחירי EXOCELL MASK". В шаблоне нет подстановки {name}, есть только в "wa_text_product": "שלום, אשמח לקבל פרטים על {name}".</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>site/proto/exocell-he-ui.json, строки 16 и 18</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Если взять шаблон буквально, клиника со страницы CELL RENEW 1.5% отправит в WhatsApp вопрос о ценах EXOCELL MASK. Для ссылки «לקליניקות: לקבלת הצעת מחיר» взять ui.wa_text_product с {name} = CELL RENEW 1.5% («שלום, אשמח לקבל פרטים על {name}»), как на странице CAD 2.5%, или завести общий шаблон цены с {name}. Номер 972547621889 верный.</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>Проверено: в exocell-he-ui.json строка 16 «wa_text_price»: «שלום, אשמח לקבל פרטים על מחירי EXOCELL MASK», подстановки {name} нет, она есть только в wa_text_product (строка 18). Сюжет CELL RENEW ведёт ссылку b6.label3 на wa_text_price «с именем CELL RENEW 1.5%», но шаблон имя не принимает. В сюжете CAD 2.5% та же ссылка идёт через ui.wa_text_product с {name}. Номер 972547621889 совпадает с contacts.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>CELL RENEW 1.5%</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[0]; assets «Флакон CELL RENEW 1.5% 30 мл» (status: needs photo)</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>«Фото флакона нет, печать неизвестна»; заказчика просят прислать фото флакона и спрашивают, такой ли это airless, как у CAD 2.5%.</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>| 70, 75 | 113:8199, 113:8214 | CELL RENEW 1.5% | белый airless-флакон на полке | 3D-флакон |</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>site/photo-catalog.md, строка 42</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Фото флакона CELL RENEW 1.5% уже есть в Figma: №70 и №75 (узлы 113:8199, 113:8214), белый airless-флакон, как №9 у CAD 2.5%. Модель флакона строить по ним, assets перевести из «needs photo» в работу по Figma. У заказчика спросить только то, чего на снимках с полки не видно: вид сверху, печать крупно, цвет и прозрачность сыворотки.</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Строка 42 photo-catalog.md процитирована точно: №70 и №75 (113:8199, 113:8214) — CELL RENEW 1.5%, «белый airless-флакон на полке», назначение «3D-флакон». В сюжете сказано «Фото флакона нет» и есть просьба прислать фото. Фото заказчика уже лежат в Figma, в репозитории их нет. Сходство с флаконом CAD (№9, «белый airless-флакон») видно по описанию.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>CELL RENEW 1.5%</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[1] (фасад коробки в высоком разрешении); assets «Коробка CELL RENEW 1.5%»</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Текстура взята с protocols/print/img/cell-renew-15.webp (309×1012), заказчика просят прислать фасад от 2000 px.</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>| 10 | 93:8097 | CELL RENEW 1.5% | коробка: «BIOSPICULE SERUM», эмблема спикул, 30 ml | текстура коробки |</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>site/photo-catalog.md, строка 18</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Сначала проверить разрешение оригинала фото №10 (узел 93:8097) в Figma, он отмечен как текстура коробки. Если по высоте его хватает, брать фасад оттуда, а не из webp 309×1012. Новый фасад просить у заказчика, только если оригинал слабый. Вопрос о боковых гранях, верхе и заднике остаётся.</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Строка 18 photo-catalog.md процитирована точно: №10 (93:8097) — коробка CELL RENEW 1.5%, назначение «текстура коробки». Сюжет берёт текстуру только с protocols/print/img/cell-renew-15.webp (309×1012) и просит у заказчика фасад от 2000 px, не проверив оригинал в Figma. Ответ частичный: фото граней, верха и задника в каталоге фото нет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>CELL RENEW 1.5%</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[4] (свой солнцезащитный крем MITODERM для шага 3)</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>«есть ли у MITODERM свой солнцезащитный крем, который можно показать?»</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>В содержании каталога (все средства) солнцезащитного средства нет: '5. תכשירים משלימים לשימוש ביתי ... EXOTECH GEL • EXOSIGNAL SPRAY ... CELL RENEW 1.5% ... CELLULAR AGE DEFENSE 2.5% ... DERMA RECOVERY'. Протоколы называют только степень защиты: 'SPF   מסנן קרינה של 30 לפחות חובה' и 'יש להשתמש מדי בוקר במסנן קרינה SPF 50'.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>source-texts.md, стр. 02 (תוכן העניינים), строки 9–34; protocols/src/content.he.mjs, строки 91 и 221</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Своего солнцезащитного средства у MITODERM в источниках нет: ни в содержании каталога, ни на mitoderm.com. Вопрос «есть ли свой SPF» снять. Шаг «הגנה» показывать без упаковки, полосой дневного света, как в сюжете CAD 2.5%. Владельцу задать один общий вопрос на обе страницы: подходит ли такой показ шага.</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>В содержании каталога (стр. 02) перечислены все средства, солнцезащитного среди них нет. На mitoderm.com его тоже нет. Протоколы называют только степень защиты (строки 91 и 221, цитаты точные). Поправка: в сюжете CAD 2.5% шаг «защита» полосой света ещё ждёт подтверждения владельца («Так подходит?»), то есть «уже решено» — преувеличение.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>CELL RENEW 1.5%</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[5] (список клиник-партнёров для кнопки «איפה לקנות»); в сюжете нет экрана 8</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>«Есть ли список клиник-партнёров... (например, блок специалистов после экрана покупки)?» В сюжете 7 экранов.</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>'**Блок «Кто делает процедуру»** на каждой странице — сразу после экрана с ценой. Дизайн — со страницы специалистов в Make, данные — со списка на сайте (имя, город, телефон).' · 'В каждый сюжет добавляется экран 8 «Кто делает процедуру» с меткой פנים/קרקפת.' · '**Таблицу специалистов** заказчик пришлёт позже.'</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>PLAN.md, раздел 7, строки 80, 94, 120</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Добавить в сюжеты CELL RENEW 1.5%, CAD 2.5% и MICRO BOOST 10% экран 8 «Кто делает процедуру» сразу после экрана покупки (метка פנים, фильтр по линейке BIOSPICULE). Дизайн — со страницы специалистов, данные — из таблицы, которую заказчик пришлёт позже. Вопрос заказчику сузить до одного: «איפה לקנות» ведёт на экран 8 или на «Ask your clinic» (решение 17)?</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>PLAN.md, строки 80, 94 и 120 процитированы точно. Экран 8 «Кто делает процедуру» с меткой פנים/קרקפת полагается на каждой странице, сразу после экрана цены, таблицу заказчик пришлёт позже. Во всех трёх сюжетах по 7 экранов, экрана 8 нет. Поправка: PLAN не говорит, что «איפה לקנות» ведёт на этот блок. По решению 17 (project-council) «Where to buy» открывает «Ask your clinic», так что маршрут кнопки остаётся отдельным вопросом.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>DERMA RECOVERY CREAM</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>b0.title + b0.line</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>ошибка</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>«כל פרוטוקול מסתיים כאן.» / «Every protocol ends here.»; «…השלב המשלים, בבית.» / «The finishing step, at home.»</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Протоколы: крем наносят в клинике в конце процедуры, а после него обязателен SPF. V-TECH+MITOPEN: «בסיום DERMA RECOVERY CREAM» → «מקדם הגנה חובה»; CELL BOOSTER: «מריחת קרם לחות דרמה רקברי.» → «ומעליו מקדם הגנה 30 SPF לפחות». Каталог: «Derma Recovery סיום טיפול ובבית»</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/protocols/src/content.he.mjs стр. 52–53, 111–112; mitoderm-catalog/source-texts.md стр. 299</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Заголовок заменить на дословную строку каталога «הקרם המשלים לכל פרוטוקול טיפול» (product-pages.he.json cta[0]; EN по смыслу: «The complementary cream for every treatment protocol»). Строку исправить на «…השלב המשלים – בסיום הטיפול ובבית.» (опора на каталог: «סיום טיפול ובבית»). Не писать, что протокол заканчивается кремом: последний шаг — обязательный SPF. Новые строки на иврите отдать на вычитку.</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Тексты сюжета проверены: b0.title «כל פרוטוקול מסתיים כאן.» / «Every protocol ends here.», b0.line «…השלב המשלים, בבית.». По протоколам это неверно. Там, где крем есть, после него обязателен SPF: стр. 52–53 «בסיום DERMA RECOVERY CREAM» → «מקדם הגנה חובה», стр. 111–112 «מריחת קרם לחות דרמה רקברי.» → «ומעליו מקדם הגנה 30 SPF לפחות», стр. 90–91. В протоколах EXO-NAD и EXOSIGNAL HAIR крема нет вовсе. PLAN фиксирует финиш «EXOCELL MASK → DERMA RECOVERY → SPF». Крем наносят и в клинике, поэтому «בבית» без клиники неполно. Каталог: «Derma Recovery סיום טיפול ובבית» (source-texts.md стр. 299), а product-pages.he.json cta[0] — «הקרם המשלים לכל פרוטוקול טיפול».</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>DERMA RECOVERY CREAM</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>b4.line / b4.label1–3 (где крем стоит в протоколе)</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>«לאחר CELL RENEW 1.5% או CELLULAR AGE DEFENSE 2.5%; לאחר פרוטוקולי V-TECH, EXO-NAD ו-MICRO BOOST 10%; בוקר וערב, על עור נקי.» — EXOCELL MASK перед кремом и SPF после крема не упомянуты</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>MICRO BOOST 10% + V-TECH, «סיום הטיפול»: «EXOCELL MASK  כמסכת סיום ושיקום» → «DERMA RECOVERY CREAM להשלמת לחות הזנה ותמיכה במחסום העורי» → «SPF   מסנן קרינה של 30 לפחות חובה»; CELL BOOSTER: «בסיום ניתן להניח מסכת EXOCELL MASK» → «מריחת קרם לחות דרמה רקברי.» → «ומעליו מקדם הגנה 30 SPF לפחות»</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/protocols/src/content.he.mjs стр. 88–91, 110–112; content.en.mjs стр. 88–90, 109–111</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>В клинической ветке экрана 5 текстом, без пакшотов других линеек, показать порядок по протоколу: EXOCELL MASK (по протоколу рекомендуется) → DERMA RECOVERY CREAM → SPF 30+ (обязательно). Минимум — добавить строку на иврите дословно из протокола: «ומעליו מקדם הגנה 30 SPF לפחות». Сейчас обязательного SPF поверх крема нет ни на одном экране.</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Цитаты дословны: стр. 89–91 и 110–112. В сюжете b4.line и метки экрана 5 действительно не упоминают ни EXOCELL MASK перед кремом, ни SPF после него. SPF нет ни на одном экране. PLAN (слово заказчика 11/10) фиксирует финиш «EXOCELL MASK → DERMA RECOVERY → SPF». Поправка к предложению: EXOCELL MASK в протоколах не всегда обязательна. В V-TECH+MITOPEN — «מומלץ», в CELL BOOSTER — «ניתן», и только в MICRO BOOST 10% это просто шаг. Обязателен только SPF. По правилу о линейках другие средства показывать текстом, а не пакшотами.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>DERMA RECOVERY CREAM</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>5, 7</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>b4.label4 «חובה לאחר MICRO BOOST 10%»; b6.line «לאחר MICRO BOOST 10% הקרם חובה גם בבית.»</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>источники расходятся</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>После MICRO BOOST 10% крем обязателен и дома / «Mandatory home care after MICRO BOOST 10%»</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Протокол MICRO BOOST 10%: «לבית ניתן להמליץ את הסדרה הביתית של ביוספיקול לחידוש , אקסוטק גל ללחות מיטבית וקרם רקברי להזנה ולחות אינטנסיבית.» (EN: «For home use, recommend … DERMA RECOVERY CREAM for intensive nourishment and hydration.»). В завершении процедуры словом «חובה» помечен только SPF. Каталог: «Derma Recovery סיום טיפול ובבית – חובה לאחר הטיפול»</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/protocols/src/content.he.mjs стр. 71, 88–91; mitoderm-catalog/source-texts.md стр. 299; site/product-pages.he.json стр. 882</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Одной строкой спросить заказчика: «В протоколе MICRO BOOST 10% дома крем — ‘ניתן להמליץ’, в каталогах — ‘חובה גם בבית’. Что оставляем?» До ответа ставить формулировку протокола: заказчик назвал протоколы основными. b4.label4 → «בסיום טיפול MICRO BOOST 10%» (в клинике крем — шаг завершения после EXOCELL MASK, перед обязательным SPF). В b6.line вместо «הקרם חובה גם בבית» — рекомендация для дома с опорой на «לבית ניתן להמליץ … וקרם רקברי להזנה ולחות אינטנסיבית». Если заказчик подтвердит «חובה», вернуть каталожную строку. Новые строки на иврите отдать на вычитку.</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Цитаты точные. Протокол MICRO BOOST 10%, стр. 71: «לבית ניתן להמליץ … וקרם רקברי להזנה ולחות אינטנסיבית». В «סיום הטיפול» (стр. 88–91) словом «חובה» помечен только SPF. Сюжет: b4.label4 «חובה לאחר MICRO BOOST 10%», b6.line «לאחר MICRO BOOST 10% הקרם חובה גם בבית.» — дословно product-pages.he.json cta[1]. «Обязательно» есть и в source-texts.md стр. 299 («חובה לאחר הטיפול»), и в русском каталоге («также обязательное домашнее применение»). Противоречие реальное, но в одной части: «обязательно дома» против протокольного «можно рекомендовать». В клинике крем — штатный шаг завершения протокола, поэтому называть его там «מומלץ», как в исходном предложении, неточно. «חובה» трижды написал сам заказчик, значит решать ему.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>DERMA RECOVERY CREAM</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>questions_ru[6] — привести b5.line («1.69 fl. oz.» / «1.69 fl. oz») к печати?</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>ответ на вопрос</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Вопрос открыт: в b5.line «50 ml ℮ 1.69 fl. oz.» (EN) и «1.69 fl. oz» (HE)</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Упаковка, нижняя строка коробки и банки: «50 ml ℮ 1.69 fl.oz.»; каталог cat.kit[0]: «50 ml ℮ 1.69 fl.oz.»</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>site/packaging-text.json → derma-recovery-cream.objects[box|jar].front «bottom: '50 ml ℮ 1.69 fl.oz.'»; site/product-pages.json derma-recovery-cream.kit[0]</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>В b5.line (HE и EN) писать ровно как на коробке и банке: «50 ml ℮ 1.69 fl.oz.». Вопрос 6 у заказчика снять.</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>Проверено. В packaging-text.json → derma-recovery-cream нижняя строка и коробки, и банки: «50 ml ℮ 1.69 fl.oz.». Так же в каталоге: product-pages.json kit[0] «50 ml ℮ 1.69 fl.oz. — …» и product-pages.he.json kit[0] «…– 50 ml ℮ 1.69 fl.oz.». В сюжете b5.line: HE «1.69 fl. oz», EN «1.69 fl. oz.». Это расходится с печатью и со строкой cat.kit[0] на экране 7 того же сюжета. Ответ на questions_ru[6] уже есть в источниках, спрашивать заказчика не нужно.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>MITOPEN</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>2 (и 3)</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>b1.label3 «קרקפת» / b1.label4 «עומק לפי אינדיקציה»; action_3d_ru экрана 2: «Цифр глубины по зонам не показываем: в каталоге их нет»</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>не хватает важного</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Глубина по зонам не указана; на странице только общий диапазон 0.25–2.5 мм</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>EXOSIGNAL HAIR: «עומק עבודה: עד 0.6 מ״מ, בהתאם לאזור, למצב הקרקפת ולאבחון המקצועי.» (EN: «Working depth: up to 0.6 mm, depending on the area, scalp condition and the professional assessment.»); V-TECH (лицо): «עומק העבודה נקבע בהתאם למכשיר, לאזור המטופל, לעובי העור, למצבו ולאבחון המקצועי.»</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/protocols/src/content.he.mjs стр. 137 (exosignal-hair) и стр. 42 (vtech-mitopen); content.en.mjs стр. 136, 41</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>У метки кожи головы показать «קרקפת · עד 0.6 מ״מ» (EN: «Scalp · up to 0.6 mm»), число — в изоляции LTR. Опора дословно: «עומק עבודה: עד 0.6 מ״מ». Для лица, шеи и декольте числа не давать: глубину выбирает специалист («עומק העבודה נקבע בהתאם למכשיר, לאזור המטופל, לעובי העור, למצבו ולאבחון המקצועי.»). Пометку в action_3d_ru исправить: цифра для кожи головы есть в протоколах.</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Цитата дословна: content.he.mjs стр. 137 «עומק עבודה: עד 0.6 מ״מ, בהתאם לאזור, למצב הקרקפת ולאבחון המקצועי.», стр. 42 — для лица числа нет. В сюжете (экран 2, action_3d_ru) сказано «Цифр глубины по зонам не показываем: в каталоге их нет», а метки — «קרקפת» и «עומק לפי אינדיקציה». В каталоге этого числа и правда нет, но в основном протоколе MITOPEN + EXOSIGNAL HAIR оно есть. Для пера с диапазоном 0.25–2.5 мм потолок 0.6 мм на коже головы — существенный рабочий параметр, а не вопрос стиля.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>MITOPEN</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>b4.title / b4.line / b4.label2–3 (порядок шагов) + action_3d_ru (сначала сетка микроканалов, потом капля стекает в сетку); то же в story_one_line</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>источники расходятся</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>«הגדרה. מיקרונידלינג. החדרה.» / «בחרו עומק ומהירות בהתאם לאזור, צרו מיקרו־תעלות אחידות ולאחר מכן יישמו את V-TECH SYSTEM בפנים או את EXOSIGNAL HAIR בקרקפת.» (EN: «create uniform micro-channels, then apply V-TECH SYSTEM on the face or EXOSIGNAL HAIR on the scalp»); метки «2 · מיקרונידלינג אחיד», «3 · החדרת הפורמולה»</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Протоколы: EXOSIGNAL HAIR — «בסימולטניות עוברים ביחד עם החומר והמכשיר . לחלק את העבודה לאזורים : קודם לטפטף מעט מהחומר על אזור מסוים ואז לעשות סטמפינג» (EN: «Product and device work at the same time. Divide the work into sections: first drip a little product onto a section, then stamp.»); V-TECH — «יש ליישם את הסרום באמצעות MITOPEN / מזופן או מכשור מקצועי מתאים אחר.»; CELL BOOSTER — «לטפטף מס טיפות ביחד עם המקרונידלינג    בכל אזור בפנים -בשיטת הסטמפינג». Против: каталог product-pages.json mitopen.steps «Needle — Create uniform micro-channels…» → «Deliver — Apply V-TECH SYSTEM on the face or EXOSIGNAL HAIR on the scalp.» и mitoderm.com «After a controlled injury, the material is dripped onto the skin»</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/protocols/src/content.he.mjs стр. 138 (exosignal-hair), 41 (vtech-mitopen), 109 (cell-booster); content.en.mjs стр. 137; site/product-pages.json стр. 972–976; site/sources/mitoderm-com/products-en.json solution.main.discountLabelText2</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Побеждают протоколы. Средство не наносят на готовую сетку: его капают на участок и сразу проходят MITOPEN по нему, участок за участком. Метки: «1 · הגדרת עומק ומהירות» → «2 · טפטוף החומר על האזור» → «3 · סטמפינג עם MITOPEN, אזור אחר אזור». Заголовок, например: «הגדרה. טפטוף. סטמפינג.». b4.line, например: «בחרו עומק ומהירות בהתאם לאזור, טפטפו מעט מהחומר על אזור אחד ובצעו סטמפינג עם MITOPEN – אזור אחר אזור: V-TECH SYSTEM בפנים, EXOSIGNAL HAIR בקרקפת.». Опора на иврите дословно: «קודם לטפטף מעט מהחומר על אזור מסוים ואז לעשות סטמפינג» (EXOSIGNAL HAIR), а для лица — «יש ליישם את הסרום באמצעות MITOPEN» (V-TECH). Для лица при желании добавить: после сыворотки V-TECH Gel Mask наносят на ту же зону и массируют до впитывания, без смывания («לאחר סיום העבודה עם הסרום, יש למרוח V-TECH Gel Mask על אותו אזור.»). В 3D сначала капля падает на участок, потом перо проходит через неё; сетку раньше капли не показывать. Тот же порядок поправить в story_one_line. Новые строки на иврите отдать на вычитку.</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Цитаты проверены дословно: content.he.mjs стр. 138 («בסימולטניות עוברים ביחד עם החומר והמכשיר… קודם לטפטף מעט מהחומר על אזור מסוים ואז לעשות סטמפינג»), стр. 41 (V-TECH: «יש ליישם את הסרום באמצעות MITOPEN»), стр. 109 (CELL BOOSTER: «לטפטף מס טיפות ביחד עם המקרונידלינג… בשיטת הסטמפינג»). В сюжете действительно «צרו מיקרו־תעלות אחידות ולאחר מכן יישמו…», метки «2 · מיקרונידלינג אחיד» → «3 · החדרת הפורמולה», а в 3D капля стекает в уже готовую сетку. Порядок взят из каталога (steps) и mitoderm.com («After a controlled injury, the material is dripped»), но порядок шагов определяют протоколы. Там средство и перо работают одновременно, участок за участком. Конфликт настоящий. Одна оговорка: в протоколе V-TECH слова «капать» нет. Там сыворотку набирают в шприц 3 мл и наносят через MITOPEN. Прямо «капать, потом стемпинг» сказано в протоколах EXOSIGNAL HAIR и CELL BOOSTER (лицо).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>MITOPEN</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>b4.label4</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>источники расходятся</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>«משתלב עם V-TECH · EXOSIGNAL HAIR · MICRO BOOST 10%» / «Works with V-TECH · EXOSIGNAL HAIR · MICRO BOOST 10%»</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Протоколы: связки «MITOPEN + VTECH», «MITOPEN +MITOTECH CELL BOOSTER», «MITOPEN + EXOSIGNAL HAIR»; MICRO BOOST 10% стоит вместо пера: «BIOSPICULE BOOST 10% + VTECH», «BIOSPICULE BOOST 10% + MITOTECH CELL BOOSTER», заголовок «MITOPEN/BIOSPICULE CELL BOOSTETR 10%», EN: «Alternatively, with the biospicule gel: apply 1.5-2 ml to the face…». Каталог: «יכול לשמש כטיפול ביומיקרונידלינג כתחליף לטיפול המסורתי במיקרונידלינג!». Против: каталожные чипы MITOPEN («Works with … MICRO BOOST 10%»)</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>mitoderm-catalog/protocols/src/content.he.mjs стр. 22–26, 103; content.en.mjs стр. 108; mitoderm-catalog/source-texts.md стр. 245; site/product-pages.json стр. 1007 (mitopen.chips)</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Убрать MICRO BOOST 10% из «משתלב עם»: MITOPEN и MICRO BOOST 10% — два разных пути (микронидлинг пером или биомикронидлинг спикулами), вместе их не применяют. Метка: «משתלב עם V-TECH · EXOSIGNAL HAIR» (как в каталоге: «להחדרת חומרים: VTECH SYSTEM, EXOSIGNAL HAIR»). MITOTECH CELL BOOSTER (в протоколах есть связка «MITOPEN +MITOTECH CELL BOOSTER») добавлять только текстом, без ссылки, и только после слова заказчика: в PLAN MITOTECH отложен. Заодно убрать упоминание MICRO BOOST 10% / BIOSPICULE из colour_env и action_3d_ru экрана 5.</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Проверено. В протоколах связки только «MITOPEN + VTECH», «MITOPEN +MITOTECH CELL BOOSTER», «MITOPEN + EXOSIGNAL HAIR». MICRO BOOST 10% стоит вместо пера: заголовок «MITOPEN/BIOSPICULE…», а в стр. 109 «…או באמצעות גל הביוספיקולות» — то есть «или». В протоколе MICRO BOOST 10% (стр. 74–85) MITOPEN нет. В каталоге (source-texts.md стр. 245): «יכול לשמש כטיפול ביומיקרונידלינג כתחליף לטיפול המסורתי במיקרונידלינג!». В печатном каталоге на странице MITOPEN (source-texts.md стр. 453–466) тоже указаны только «VTECH SYSTEM, EXOSIGNAL HAIR». MICRO BOOST 10% есть лишь в чипах product-pages(.he).json. Метка сюжета «משתלב עם … MICRO BOOST 10%» противоречит протоколам. Поправка к предложению: MITOTECH по PLAN отложен до пакшота и текстов («MITOTECH (ждёт пакшот и тексты)»), поэтому без слова заказчика его не добавлять.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Site roadmap (Excel, Hebrew): the stages as of 17/10
The owner asked for the roadmap to show the changes. Stage by stage:
- MASK has been rebuilt and waits for his «ок»;
- the V-TECH HD sample, with the real box opening, waits for his edits
  and then the Mac render;
- new: Figma for the programmer, every page with the latest decisions
  and a spec;
- new: the fast-method pilot on EXOTECH GEL, Firefly frames plus Kling;
- the remaining products follow the pilot, light phone version first.
The later stages keep their reviewed Hebrew. The workbook has no
Cyrillic.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/MITODERM-3D-story.xlsx
+++ b/mitoderm-catalog/site/MITODERM-3D-story.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>סטטוס נכון ל-14/10</t>
+          <t>סטטוס נכון ל-17/10</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>התרגום לקראת סיום, חוברת העבודה בשלבי הרכבה</t>
+          <t>מוכן, עודכן ב-17/10</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>עמוד 3D לדוגמה של EXOCELL MASK: בטלפון הקופסה קטנה, ליד הכותרת; 5 שקיות עם הדפס קריא; המוצר בצבעיו האמיתיים, הטורקיז רק מסביב; פחות גלילה ריקה; כרטיסי «ראו גם»</t>
+          <t>עמוד 3D לדוגמה של EXOCELL MASK: מסכה אחת בשתי שכבות, ובמסך הערכה השכבות נפרדות, כל אחת עם שם; Rubik בכל העמוד; הטקסט מימין וה-3D משמאל; בלוק «מה באריזה» אחד</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -530,7 +530,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>נבנה מחדש לפי ההערות מ-14/10, ממתין ל«אוקיי»</t>
+          <t>נבנה מחדש ב-17/10, ממתין ל«אוקיי»</t>
         </is>
       </c>
     </row>
@@ -542,22 +542,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>רנדר HD: מעקב מסלולי קרניים (path tracing) ב-Blender Cycles במקום רינדור בדפדפן – זכוכית ונוזל עם שבירת אור, רדיד, קצוות משופעים, תאורת סטודיו; הדוגמה – האובייקט המרכזי של V-TECH והערכה, ואחרי «אוקיי» – סדרת הרנדרים</t>
+          <t>V-TECH ב-HD ‏(Blender Cycles): הקופסה נפתחת כמו בצילומים – העטיפה המוזהבת עולה, הקופסה השחורה נפתחת, 5 אמפולות ו-5 שקיות; רדיד סאטן בלי צללים כבדים; תאי אקסוזום, מולקולות PDRN וסליל DNA; תנועה גם בטלפון</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>דוגמה 2 שעות, עמוד 1–2 שעות</t>
+          <t>הדוגמה מוכנה; רינדור סופי על ה-Mac כ-3–4 שעות</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>צילומים של כל אריזה מכל הצדדים, מ-3000 px ומעלה, מידות במ״מ, צילום של אריזה פתוחה</t>
+          <t>תיקונים לדוגמה, «אוקיי», הרצת הרינדור על ה-Mac</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Blender מותקן, הטקסטורות מוכנות, הדוגמה הבאה בתור</t>
+          <t>הדוגמה פורסמה ב-17/10, ממתינה לתיקונים</t>
         </is>
       </c>
     </row>
@@ -569,22 +569,22 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>השלמת V-TECH: מסך הפרוטוקול – בקצרה «איך זה עובד», בלי מינונים; הפרוטוקול המלא – אחרי הרכישה; בלוק «מאותה סדרה / משתלב עם»; פריימים ב-HD</t>
+          <t>Figma למתכנת: כל העמודים לפי ההחלטות האחרונות (טקסט מימין, 3D משמאל, Rubik, בלוק «מה באריזה» אחד), עם מפרט: מנוע הפריימים, הנכסים, נקודות השבירה והתנועה בטלפון</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2 שעות</t>
+          <t>יום אחד</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>«אוקיי» על V-TECH ועל MASK</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>העמוד ב-Figma הורכב, 2 סבבי בדיקה</t>
+          <t>בעבודה</t>
         </is>
       </c>
     </row>
@@ -596,22 +596,22 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>שאר עמודי המוצרים, אחד אחרי השני: MICRO BOOST 10% → DERMA RECOVERY CREAM → MITOPEN → EXO-NAD → EXOSIGNAL HAIR → EXOTECH GEL → EXOSIGNAL SPRAY → CELL RENEW 1.5% → CELLULAR AGE DEFENSE 2.5% → MITOSCAN</t>
+          <t>פיילוט של השיטה המהירה על EXOTECH GEL: פריימים מרכזיים מ-Firefly (של המזמין/ה) ומעברים ב-Kling, שהופכים לפריימים לאתר באותו מנוע; השוואה ל-Blender באיכות, בזמן ובמחיר</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2–3 שעות לכל עמוד</t>
+          <t>יום אחד</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>צילומי HD של האריזות, פקשוט של הספריי, צילומים של סריקות MITOSCAN</t>
+          <t>שני פריימים מ-Firefly ‏(2400×1500, המוצר משמאל); אישור להוצאה לפני כל יצירה</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>אחרי שלב 1</t>
+          <t>הבא בתור</t>
         </is>
       </c>
     </row>
@@ -623,22 +623,22 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>דף הבית – דף בית אמיתי: מסך פתיחה כמו ב-Make → כל המוצרים ב-3D מתכנסים ומתפזרים לפי סדרות → בחירת תחום למעלה → כל סדרה פעם אחת; לחיצה על סדרה פותחת את חלון הסדרה; «אודות» למטה; עמוד כל המוצרים</t>
+          <t>שאר עמודי המוצרים בשיטה הטובה מבין השתיים – קודם גרסה קלה לטלפון, אחר כך 3D: MICRO BOOST 10% → DERMA RECOVERY CREAM → MITOPEN → EXO-NAD → EXOSIGNAL HAIR → EXOSIGNAL SPRAY → CELL RENEW 1.5% → CELLULAR AGE DEFENSE 2.5% → MITOSCAN</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>1 יום</t>
+          <t>יום עבודה לכל עמוד</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>דוגמה למסך הפתיחה מ-Make</t>
+          <t>צילומי HD של האריזות (גם פתוחות), מידות במ״מ, צילומי לפני/אחרי באישור הלקוחות</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>אחרי שלב 3</t>
+          <t>אחרי הפיילוט</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>חשבון ותוכנית נאמנות: בחירת תחום → הדגשים אישיים; הרשמה (שם, email, טלפון, תפקיד); אימות סטטוס מקצועי עבור המוצרים המקצועיים; קוד קופון, 5% על הבאת חבר/ה, מדרגות עד 15%; הפרוטוקולים של המוצרים שנרכשו – בחשבון ובדוא״ל</t>
+          <t>דף הבית – דף בית אמיתי: מסך פתיחה כמו ב-Make → כל המוצרים ב-3D מתכנסים ומתפזרים לפי סדרות → בחירת תחום למעלה → כל סדרה פעם אחת; לחיצה על סדרה פותחת את חלון הסדרה; «אודות» למטה; עמוד כל המוצרים</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>כללי התוכנית (מדרגות, מועדים), מי מאמת/ת את הסטטוס</t>
+          <t>דוגמה למסך הפתיחה מ-Make</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -677,17 +677,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>אירועי האקדמיה בדף הבית וטופס להזמנת מקומות</t>
+          <t>חשבון ותוכנית נאמנות: בחירת תחום → הדגשים אישיים; הרשמה (שם, email, טלפון, תפקיד); אימות סטטוס מקצועי עבור המוצרים המקצועיים; קוד קופון, 5% על הבאת חבר/ה, מדרגות עד 15%; הפרוטוקולים של המוצרים שנרכשו – בחשבון ובדוא״ל</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>3 שעות</t>
+          <t>1 יום</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>תאריכים, מחירים</t>
+          <t>כללי התוכנית (מדרגות, מועדים), מי מאמת/ת את הסטטוס</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -704,22 +704,22 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>עמודי שירות: נגישות, פרטיות, תנאי שימוש, פאנל ניהול</t>
+          <t>אירועי האקדמיה בדף הבית וטופס להזמנת מקומות</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2 שעות</t>
+          <t>3 שעות</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>טקסטים משפטיים</t>
+          <t>תאריכים, מחירים</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>בסוף</t>
+          <t>אחרי שלב 6</t>
         </is>
       </c>
     </row>
@@ -731,20 +731,47 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>עמודי שירות: נגישות, פרטיות, תנאי שימוש, פאנל ניהול</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2 שעות</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>טקסטים משפטיים</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>בסוף</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
           <t>התוצר הסופי – קישור אחד: מפת האתר עם כל העמודים ומסלולי המשתמש</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>2 שעות</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>בסוף, טיוטה – מוקדם יותר</t>
         </is>

</xml_diff>

<commit_message>
Developer handoff: Hebrew note, roadmap status 18/10, Figma lessons
The owner asked for the roadmap and Figma to show the current state so
the programmer can start building every page. Figma now opens on a
Hebrew start page for the programmer, and both sample pages match the
prototypes. This commit carries the repo side:
- HANDOFF-dev.he.md: build order, files, frame engine, rules, open items.
- Roadmap rows 1 and 2 and the header set to 18/10; Excel rebuilt,
  no Cyrillic.
- PLAN section 12 records what changed in Figma and how images got there.
- design-rules: Hebrew with Latin in Figma needs RLM around brackets and
  quotes, and code goes in its own LTR block.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/MITODERM-3D-story.xlsx
+++ b/mitoderm-catalog/site/MITODERM-3D-story.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>סטטוס נכון ל-17/10</t>
+          <t>סטטוס נכון ל-18/10</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>הדוגמה פורסמה ב-17/10, ממתינה לתיקונים</t>
+          <t>הדוגמה פורסמה ב-17/10; ב-18/10 נוספו מולקולות PDRN וסליל DNA; ממתינה לתיקונים</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>בעבודה</t>
+          <t>18/10: ב-Figma יש עמוד התחלה למתכנת, ועמודי V-TECH ו-MASK עודכנו; שאר העמודים — לפי התבנית</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EXOTECH GEL story: the jar unscrews into two gold halves
The owner said how the jar opens. The story had the lid lift straight up
with no turn, because that answer was missing. Now the upper half turns
about a quarter turn as it lifts (screens 2→3) and screws back on as it
closes (4→5). The Russian source, its snapshot and the reviewed Hebrew
change together, so the Hebrew workbook still has no Russian in it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/MITODERM-3D-story.xlsx
+++ b/mitoderm-catalog/site/MITODERM-3D-story.xlsx
@@ -7987,7 +7987,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>המצלמה יורדת לגובה התפר. המכסה – חצי הכדור העליון עם הכיתוב השלם 'EXOTECH / GEL' – מתרומם ישר למעלה בכמה מילימטרים: בלי סיבוב ביחס לבסיס, בלי הטיה לאחור. הסדק הצר לאורך קו המשווה מתמלא בזוהר זהוב חם, ולכן לא נראים לא פנים הצנצנת ולא הצד התחתון של המכסה (שאלה 1). הבסיס הזהוב החלק נשאר במקומו.</t>
+          <t>המצלמה יורדת לגובה התפר. המכסה – חצי הכדור העליון עם הכיתוב השלם 'EXOTECH / GEL' – נפתח בהברגה (תשובת המזמין/ה, 18/10: הכדור מתחלק לשני חצאים): מסתובב סביב הציר האנכי כרבע סיבוב ומתרומם בכמה מילימטרים, בלי הטיה לאחור. הסדק הצר לאורך קו המשווה מתמלא בזוהר זהוב חם, ולכן לא נראים לא פנים הצנצנת ולא הצד התחתון של המכסה (מראה הג׳ל – שאלה 2). הבסיס הזהוב החלק נשאר במקומו.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8059,7 +8059,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>המכסה עם הכיתוב השלם 'EXOTECH / GEL' מרחף מעל הבסיס, והסדק הצר זוהר בזהב חם. מהסדק עולות בזו אחר זו חמש טיפות ג׳ל שקופות – חמשת הרכיבים הפעילים מ-b2.line. ארבע טיפות נקיות, בלי מתכת, והן נבדלות בגודל, בצורה ובשבירת האור. ניצוצות זהב ונחושת מנצנצים רק בטיפת הפפטידים (b2.label3), כמו בהרכב. הטיפות חגות לאט סביב הכדור בגבהים שונים. ארבע טיפות מקושרות לארבעת הצ׳יפים של b2: ריחוף או הקשה על צ׳יפ מדגישים את הטיפה שלו בהילה בהירה (מיקרו-אינטראקציה מהסטוריבורד האנגלי של בלוק 2). הטיפה החמישית, cat.ingredients[4] (פוליסכרידים ממקור חלזון), מודגשת בריחוף מעל המשפט.</t>
+          <t>החצי העליון של הכדור, אחרי שנפתח בהברגה, מרחף עם הכיתוב השלם 'EXOTECH / GEL' מעל החצי התחתון, והסדק הצר זוהר בזהב חם. מהסדק עולות בזו אחר זו חמש טיפות ג׳ל שקופות – חמשת הרכיבים הפעילים מ-b2.line. ארבע טיפות נקיות, בלי מתכת, והן נבדלות בגודל, בצורה ובשבירת האור. ניצוצות זהב ונחושת מנצנצים רק בטיפת הפפטידים (b2.label3), כמו בהרכב. הטיפות חגות לאט סביב הכדור בגבהים שונים. ארבע טיפות מקושרות לארבעת הצ׳יפים של b2: ריחוף או הקשה על צ׳יפ מדגישים את הטיפה שלו בהילה בהירה (מיקרו-אינטראקציה מהסטוריבורד האנגלי של בלוק 2). הטיפה החמישית, cat.ingredients[4] (פוליסכרידים ממקור חלזון), מודגשת בריחוף מעל המשפט.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -8141,7 +8141,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>הרצועה אינה חוזרת לצנצנת. היא עפה אל המצלמה ומתמוססת על פני כל הפריים באדוות אור זהובות וחמות: הג׳ל נספג בעור הצופה (הדימוי «לעסות עד לספיגה» מתוך b4.line). במקביל המכסה יורד ישר למטה אל הבסיס, בלי סיבוב, וזוהר הסדק כבה – הצנצנת סגורה.</t>
+          <t>הרצועה אינה חוזרת לצנצנת. היא עפה אל המצלמה ומתמוססת על פני כל הפריים באדוות אור זהובות וחמות: הג׳ל נספג בעור הצופה (הדימוי «לעסות עד לספיגה» מתוך b4.line). במקביל החצי העליון יורד אל החצי התחתון ונסגר בהברגה (רבע סיבוב), וזוהר הסדק כבה – הצנצנת סגורה.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24566,7 +24566,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>איך נפתח הכדור? המכסה – חצי הכדור העליון עם הכיתוב כולו 'EXOTECH / GEL', התפר – קו המשווה מתחת ל-'GEL'. הוא נפתח בהברגה או פשוט מורם? נדרשים צילומים של הצנצנת הפתוחה מלמעלה ובזווית שלושה רבעים, וצילום של המכסה מלמטה. בינתיים המכסה מתרומם ישר למעלה בכמה מילימטרים, הסדק מכוסה בזוהר, והפנים אינם נראים.</t>
+          <t>איך נפתח הכדור? המכסה – חצי הכדור העליון עם הכיתוב כולו 'EXOTECH / GEL', התפר – קו המשווה מתחת ל-'GEL'. הוא נפתח בהברגה או פשוט מורם? נדרשים צילומים של הצנצנת הפתוחה מלמעלה ובזווית שלושה רבעים, וצילום של המכסה מלמטה. בינתיים המכסה מתרומם ישר למעלה בכמה מילימטרים, הסדק מכוסה בזוהר, והפנים אינם נראים. תשובת המזמין/ה (18/10): נפתח בהברגה – הכדור הזהוב מתחלק לשני חצאים.</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
EXOTECH GEL story: the gel is white like cream
The owner said the gel is white, like a cream. The story had made the
droplets, the ribbon and the ring film clear and glass-like, because the
colour was not yet known. They are now an opaque white cream with soft
subsurface scattering and glossy highlights, and the ribbon reads as
light because it is thin and rises. The Russian source, its snapshot and
the reviewed Hebrew change together, and the Hebrew workbook still has
no Russian in it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/MITODERM-3D-story.xlsx
+++ b/mitoderm-catalog/site/MITODERM-3D-story.xlsx
@@ -7987,7 +7987,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>המצלמה יורדת לגובה התפר. המכסה – חצי הכדור העליון עם הכיתוב השלם 'EXOTECH / GEL' – נפתח בהברגה (תשובת המזמין/ה, 18/10: הכדור מתחלק לשני חצאים): מסתובב סביב הציר האנכי כרבע סיבוב ומתרומם בכמה מילימטרים, בלי הטיה לאחור. הסדק הצר לאורך קו המשווה מתמלא בזוהר זהוב חם, ולכן לא נראים לא פנים הצנצנת ולא הצד התחתון של המכסה (מראה הג׳ל – שאלה 2). הבסיס הזהוב החלק נשאר במקומו.</t>
+          <t>המצלמה יורדת לגובה התפר. המכסה – חצי הכדור העליון עם הכיתוב השלם 'EXOTECH / GEL' – נפתח בהברגה (תשובת המזמין/ה, 18/10: הכדור מתחלק לשני חצאים): מסתובב סביב הציר האנכי כרבע סיבוב ומתרומם בכמה מילימטרים, בלי הטיה לאחור. הסדק הצר לאורך קו המשווה מתמלא בזוהר זהוב חם, ולכן לא נראים לא פנים הצנצנת ולא הצד התחתון של המכסה. הבסיס הזהוב החלק נשאר במקומו.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8059,7 +8059,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>החצי העליון של הכדור, אחרי שנפתח בהברגה, מרחף עם הכיתוב השלם 'EXOTECH / GEL' מעל החצי התחתון, והסדק הצר זוהר בזהב חם. מהסדק עולות בזו אחר זו חמש טיפות ג׳ל שקופות – חמשת הרכיבים הפעילים מ-b2.line. ארבע טיפות נקיות, בלי מתכת, והן נבדלות בגודל, בצורה ובשבירת האור. ניצוצות זהב ונחושת מנצנצים רק בטיפת הפפטידים (b2.label3), כמו בהרכב. הטיפות חגות לאט סביב הכדור בגבהים שונים. ארבע טיפות מקושרות לארבעת הצ׳יפים של b2: ריחוף או הקשה על צ׳יפ מדגישים את הטיפה שלו בהילה בהירה (מיקרו-אינטראקציה מהסטוריבורד האנגלי של בלוק 2). הטיפה החמישית, cat.ingredients[4] (פוליסכרידים ממקור חלזון), מודגשת בריחוף מעל המשפט.</t>
+          <t>החצי העליון של הכדור, אחרי שנפתח בהברגה, מרחף עם הכיתוב השלם 'EXOTECH / GEL' מעל החצי התחתון, והסדק הצר זוהר בזהב חם. מהסדק עולות בזו אחר זו חמש טיפות של ג׳ל לבן כמו קרם (תשובת המזמין/ה, 18/10) – חמשת הרכיבים הפעילים מ-b2.line. ארבע טיפות בלי מתכת, והן נבדלות בגודל, בצורה ובברק. ניצוצות זהב ונחושת מנצנצים רק בטיפת הפפטידים (b2.label3), כמו בהרכב. הטיפות חגות לאט סביב הכדור בגבהים שונים. ארבע טיפות מקושרות לארבעת הצ׳יפים של b2: ריחוף או הקשה על צ׳יפ מדגישים את הטיפה שלו בהילה בהירה (מיקרו-אינטראקציה מהסטוריבורד האנגלי של בלוק 2). הטיפה החמישית, cat.ingredients[4] (פוליסכרידים ממקור חלזון), מודגשת בריחוף מעל המשפט.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -8136,7 +8136,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>הטיפה הגדולה אינה נופלת, אלא נמתחת למעלה לרצועה שקופה ודקה – שכבת ג׳ל דקה. הרצועה מתנופפת כמו משי, לוכדת ברקים חמים, ודרכה נראה הכדור: השקיפות והעלייה למעלה מבטאות את «אף פעם לא מכביד» (b3.title). הסמן «נושף» קלות על הרצועה, וממנו יוצא גל. בזמן שהרצועה נפרשת, מופיעות בזו אחר זו ארבע התוויות של b3. זו «סצנת המראה» של בלוק 3: אין אנשים בפריים, העור הוא הצופה עצמו (ראו המעבר). פריים עם אדם – רק אחרי התשובה לשאלה 5.</t>
+          <t>הטיפה הגדולה אינה נופלת, אלא נמתחת למעלה לרצועה דקה ולבנה כמו קרם – שכבת ג׳ל דקה. הרצועה מתנופפת כמו משי, לוכדת ברקים חמים, ובשוליים היא דקה יותר וזוהרת: הדקות והעלייה למעלה מבטאות את «אף פעם לא מכביד» (b3.title). הסמן «נושף» קלות על הרצועה, וממנו יוצא גל. בזמן שהרצועה נפרשת, מופיעות בזו אחר זו ארבע התוויות של b3. זו «סצנת המראה» של בלוק 3: אין אנשים בפריים, העור הוא הצופה עצמו (ראו המעבר). פריים עם אדם – רק אחרי התשובה לשאלה 5.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -8213,7 +8213,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>הכדור הסגור עומד במרכז החצי הימני. הגלילה מעבירה אותו דרך שלושה שלבים, בסנכרון עם התוויות של b4. «1 · ניקוי»: על פני הזהב עובר משמאל לימין ברק בהיר ונקי. «2 · מריחת שכבה דקה»: סביב הכדור מופיעה לרגע טבעת-שכבה שקופה ודקה, ונספגת. «3 · בוקר וערב»: הסופטבוקס הראשי של מפת הסטודיו מקיף את הכדור בקשת – בבוקר אור בגוון קרם-זהב מלמעלה מימין, בערב אור ענבר נמוך משמאל; גבול האור והצל מחליק על פני הכדור. תווית 4 «משתלב עם V-TECH · EXO-NAD · BIOSPICULE™» – טקסט בלבד: אריזות של מוצרים אחרים לא מציגים, והירוק של BIOSPICULE אינו מופיע בדף. הכפתור b4.cta – ghost, והוא גולל אל פרטי הקשר במסך 7 (b6.label4).</t>
+          <t>הכדור הסגור עומד במרכז החצי הימני. הגלילה מעבירה אותו דרך שלושה שלבים, בסנכרון עם התוויות של b4. «1 · ניקוי»: על פני הזהב עובר משמאל לימין ברק בהיר ונקי. «2 · מריחת שכבה דקה»: סביב הכדור מופיעה לרגע טבעת-שכבה דקה ולבנה כמו קרם, ונספגת. «3 · בוקר וערב»: הסופטבוקס הראשי של מפת הסטודיו מקיף את הכדור בקשת – בבוקר אור בגוון קרם-זהב מלמעלה מימין, בערב אור ענבר נמוך משמאל; גבול האור והצל מחליק על פני הכדור. תווית 4 «משתלב עם V-TECH · EXO-NAD · BIOSPICULE™» – טקסט בלבד: אריזות של מוצרים אחרים לא מציגים, והירוק של BIOSPICULE אינו מופיע בדף. הכפתור b4.cta – ghost, והוא גולל אל פרטי הקשר במסך 7 (b6.label4).</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -16837,7 +16837,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>ללא פקשוט: פרופיל טיפה פרוצדורלי, חומר שקוף שובר אור (transmission). ארבע טיפות ללא מתכת, נבדלות בגודל, בצורה ובשבירת האור. ניצוצות זהב ונחושת – רק בטיפת הפפטידים. הצבע והשקיפות של הג׳ל – לפי צילום (שאלה 2).</t>
+          <t>ללא פקשוט: פרופיל טיפה פרוצדורלי, חומר לבן כמו קרם, אטום, עם פיזור רך מתחת לפני השטח וברקים מבריקים (תשובת המזמין/ה, 18/10: הג׳ל לבן כמו קרם). ארבע טיפות ללא מתכת, נבדלות בגודל, בצורה ובברק. ניצוצות זהב ונחושת – רק בטיפת הפפטידים.</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -16864,7 +16864,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>ללא פקשוט: משטח גלי דק מאותו חומר של הג׳ל. במעבר 4→5 הוא עף אל המצלמה ומתמוסס באדוות אור. הצבע – לפי צילום הג׳ל (שאלה 2).</t>
+          <t>ללא פקשוט: משטח גלי דק מאותו חומר של הג׳ל. במעבר 4→5 הוא עף אל המצלמה ומתמוסס באדוות אור. הצבע – לבן כמו קרם (תשובת המזמין/ה, 18/10).</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -24579,7 +24579,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>באיזה צבע הג׳ל ועד כמה הוא שקוף? נדרש צילום של הג׳ל בצנצנת פתוחה או על האצבע. בינתיים הטיפות והשכבה הדקה שקופות בגוון ניטרלי, עם ברקים חמים.</t>
+          <t>באיזה צבע הג׳ל ועד כמה הוא שקוף? נדרש צילום של הג׳ל בצנצנת פתוחה או על האצבע. בינתיים הטיפות והשכבה הדקה שקופות בגוון ניטרלי, עם ברקים חמים. תשובת המזמין/ה (18/10): לבן כמו קרם.</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Roadmap status as of 18/10 evening, in Excel and Figma
The roadmap is what the owner and the programmer read for status, and
it still said "next" for the EXOTECH pilot and "two Firefly frames".
Now: the programmer builds in React; the Kling-to-frames tool is ready;
the EXOTECH GEL draft waits for review; the owner owes six Firefly
frames (left half, 10% margin, pure black, light along the box's black
edges); the page builder fits any product. Same five cells in the
Figma copy on page 00. Excel rebuilt with no Cyrillic.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/MITODERM-3D-story.xlsx
+++ b/mitoderm-catalog/site/MITODERM-3D-story.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מפת דרכים" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סקירה כללית" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מסכים" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מה בפנים" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נכסי 3D" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מחרוזות חדשות" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="טופס" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mitoderm.com" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="שאלות" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הצלבה מול המקורות" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="מפת דרכים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="סקירה כללית" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="מסכים" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="מה בפנים" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="נכסי 3D" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="מחרוזות חדשות" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="טופס" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="mitoderm.com" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="שאלות" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="הצלבה מול המקורות" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -476,7 +476,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>סטטוס נכון ל-18/10</t>
+          <t>סטטוס נכון ל-18/10, ערב</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>18/10: ב-Figma יש עמוד התחלה למתכנת, ועמודי V-TECH ו-MASK עודכנו; שאר העמודים — לפי התבנית</t>
+          <t>18/10: ב-Figma יש עמוד התחלה למתכנת, ועמודי V-TECH ו-MASK עודכנו; שאר העמודים — לפי התבנית; המתכנת בונה ב-React</t>
         </is>
       </c>
     </row>
@@ -606,12 +606,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>שני פריימים מ-Firefly ‏(2400×1500, המוצר משמאל); אישור להוצאה לפני כל יצירה</t>
+          <t>שישה פריימים מ-Firefly ‏(2400×1500, המוצר בחצי השמאלי ולפחות 10% מהשוליים, רקע שחור נקי, קו אור דק לאורך הקצוות של הפאות השחורות של הקופסה); אישור להוצאה לפני כל יצירה</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>הבא בתור</t>
+          <t>18/10: הכלי שהופך סרטוני Kling לפריימים לאתר מוכן ונבדק; טיוטת עמוד EXOTECH GEL על התבנית (תמונות זמניות מתמונת המוצר) ממתינה לבדיקה; ממתינים לשישה פריימים מ-Firefly</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>אחרי הפיילוט</t>
+          <t>אחרי הפיילוט; בונה העמודים כבר מתאים לכל מוצר, והדוגמה היא טיוטת EXOTECH GEL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roadmap 23/10 in Hebrew; handoff lists all 12 product pages
The roadmap sheet in the workbook and the developer handoff now say
where each stage stands after the product page series, and the handoff
links the DERMA RECOVERY CREAM page published today. The Russian source
rows 5-9 were off by one row; fixed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/MITODERM-3D-story.xlsx
+++ b/mitoderm-catalog/site/MITODERM-3D-story.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -477,7 +477,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>סטטוס נכון ל-18/10, ערב</t>
+          <t>סטטוס נכון ל-23/10</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>מוכן, עודכן ב-17/10</t>
+          <t>הושלם; מפת הדרכים עודכנה ב-23/10</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>נבנה מחדש ב-17/10, ממתין ל«אוקיי»</t>
+          <t>19–21/10: בטלפון התנועה חלקה והחדות מלאה, כל התמונות ב-HD; העמוד פורסם ונמצא ב-site/public; ממתין ל«אוקיי»</t>
         </is>
       </c>
     </row>
@@ -543,22 +543,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>V-TECH ב-HD ‏(Blender Cycles): הקופסה נפתחת כמו בצילומים – העטיפה המוזהבת עולה, הקופסה השחורה נפתחת, 5 אמפולות ו-5 שקיות; רדיד סאטן בלי צללים כבדים; תאי אקסוזום, מולקולות PDRN וסליל DNA; תנועה גם בטלפון</t>
+          <t>‏V-TECH ב-HD ‏(‏Blender Cycles‏)‏: הקופסה נפתחת כמו בצילומים – העטיפה המוזהבת עולה, הקופסה השחורה נפתחת, 5 אמפולות ו-5 שקיות; רדיד סאטן בלי צללים כבדים; תאי אקסוזום, מולקולות PDRN וסליל DNA; תנועה גם בטלפון</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>הדוגמה מוכנה; רינדור סופי על ה-Mac כ-3–4 שעות</t>
+          <t>הפריימים ברוחב 2400 מוכנים; רמת 3840 — רינדור על ה-Mac</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>תיקונים לדוגמה, «אוקיי», הרצת הרינדור על ה-Mac</t>
+          <t>תיקונים לעמוד; לא חובה: הרצת render_mac.sh על ה-Mac לרמת 3840</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>הדוגמה פורסמה ב-17/10; ב-18/10 נוספו מולקולות PDRN וסליל DNA; ממתינה לתיקונים</t>
+          <t>21/10: ‏200 פריימים ברוחב 2400 פיקסלים עברו רינדור בענן, והעמוד ב-HD פורסם (עבר את כל 55 הבדיקות); פריים ניסיון ברוחב 3840 נראה חד יותר באופן ניכר במסך ה-MacBook</t>
         </is>
       </c>
     </row>
@@ -570,22 +570,22 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Figma למתכנת: כל העמודים לפי ההחלטות האחרונות (טקסט מימין, 3D משמאל, Rubik, בלוק «מה באריזה» אחד), עם מפרט: מנוע הפריימים, הנכסים, נקודות השבירה והתנועה בטלפון</t>
+          <t>‏Figma למתכנת: כל העמודים לפי ההחלטות האחרונות (טקסט מימין, 3D משמאל, Rubik, בלוק «מה באריזה» אחד), עם מפרט: מנוע הפריימים, הנכסים, נקודות השבירה והתנועה בטלפון</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>יום אחד</t>
+          <t>1 יום</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>«אוקיי» על V-TECH ועל MASK</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>18/10: ב-Figma יש עמוד התחלה למתכנת, ועמודי V-TECH ו-MASK עודכנו; שאר העמודים — לפי התבנית; המתכנת בונה ב-React</t>
+          <t>18/10: ב-Figma יש עמוד התחלה למתכנת ועמודי V-TECH ו-MASK; מ-22/10 העמודים החיים (הקישורים ב-HANDOFF, התיקייה site/public‏)‏ והטקסטים ב-Excel הם מקור האמת לבנייה; המתכנת בונה ב-React</t>
         </is>
       </c>
     </row>
@@ -597,22 +597,22 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>פיילוט של השיטה המהירה על EXOTECH GEL: פריימים מרכזיים מ-Firefly (של המזמין/ה) ומעברים ב-Kling, שהופכים לפריימים לאתר באותו מנוע; השוואה ל-Blender באיכות, בזמן ובמחיר</t>
+          <t>בחירת השיטה לעמודי המוצרים: פיילוט על EXOTECH GEL — סצנה חיה ב-three.js מול פריימים מ-Firefly ומ-Kling ומול רינדור ב-Blender</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>יום אחד</t>
+          <t>1 יום</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>שישה פריימים מ-Firefly ‏(2400×1500, המוצר בחצי השמאלי ולפחות 10% מהשוליים, רקע שחור נקי, קו אור דק לאורך הקצוות של הפאות השחורות של הקופסה); אישור להוצאה לפני כל יצירה</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>18/10: הכלי שהופך סרטוני Kling לפריימים לאתר מוכן ונבדק; טיוטת עמוד EXOTECH GEL על התבנית (תמונות זמניות מתמונת המוצר) ממתינה לבדיקה; ממתינים לשישה פריימים מ-Firefly</t>
+          <t>הושלם ב-19–21/10: עמוד EXOTECH GEL ב-three.js אושר כדוגמה; לא היה צורך ב-Firefly או ב-Kling, ולא היו הוצאות</t>
         </is>
       </c>
     </row>
@@ -624,61 +624,61 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>שאר עמודי המוצרים בשיטה הטובה מבין השתיים – קודם גרסה קלה לטלפון, אחר כך 3D: MICRO BOOST 10% → DERMA RECOVERY CREAM → MITOPEN → EXO-NAD → EXOSIGNAL HAIR → EXOSIGNAL SPRAY → CELL RENEW 1.5% → CELLULAR AGE DEFENSE 2.5% → MITOSCAN</t>
+          <t>שאר עמודי המוצרים ב-three.js לפי הדוגמה של EXOTECH GEL, אחד אחרי השני: EXOSIGNAL HAIR ‏← EXOSIGNAL SPRAY ‏← EXO-NAD ‏← MICRO BOOST 10% ‏← CELLULAR AGE DEFENSE 2.5% ‏← CELL RENEW 1.5% ‏← MITOPEN ‏← MITOSCAN ‏← DERMA RECOVERY CREAM. ב-3D רק מה שקיים באמת: המוצרים והאריזות האמיתיים, חלקיקים של הרכיבים האמיתיים וזוהר רך בצבע הסדרה</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>יום עבודה לכל עמוד</t>
+          <t>2–4 שעות לכל עמוד (בנייה, שתי בדיקות, תיקונים)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>צילומי HD של האריזות (גם פתוחות), מידות במ״מ, צילומי לפני/אחרי באישור הלקוחות</t>
+          <t>‏BIOSPICULE: ההדפסה שעל צידי הקופסאות, כקבצים (פריסת הקופסה או צילום חזיתי של כל צד), ומידות במ״מ; EXO-NAD: הצילומים כקבצים בגודל מלא; EXOSIGNAL SPRAY: פקשוט סטודיו; תשובות לשאלות: האם ב-HAIR יש PDRN בריכוז 2%; האם להשאיר את סליל ה-DNA ומולקולות ה-PDRN ב-V-TECH, ב-GEL וב-HAIR; האם הזהב נמצא ב-pH Normalizer או בפילינג של EXO-NAD</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>אחרי הפיילוט; בונה העמודים כבר מתאים לכל מוצר, והדוגמה היא טיוטת EXOTECH GEL</t>
+          <t>23/10: פורסמו 11 מתוך 12 העמודים, והם נמצאים ב-site/public ‏(‏הקישורים ב-HANDOFF‏)‏; בעמוד DERMA RECOVERY CREAM נעשים התיקונים האחרונים אחרי הבדיקה; כשיגיעו הקבצים של BIOSPICULE, ההדפסה על צידי ארבע הקופסאות תתווסף לעמודים, באותם קישורים</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4א</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>דף הבית – דף בית אמיתי: מסך פתיחה כמו ב-Make → כל המוצרים ב-3D מתכנסים ומתפזרים לפי סדרות → בחירת תחום למעלה → כל סדרה פעם אחת; לחיצה על סדרה פותחת את חלון הסדרה; «אודות» למטה; עמוד כל המוצרים</t>
+          <t>כתובת משותפת לאתר: אחסון התיקייה site/public ‏(‏כל העמודים ודף הפתיחה‏)‏ ב-Vercel או ב-GitHub Pages — קישורים ישירים, בלי הצ׳אט, זמינים מיד למתכנת ולצוות</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>1 יום</t>
+          <t>30 דקות</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>דוגמה למסך הפתיחה מ-Make</t>
+          <t>פעולה אחת: לתת לאפליקציה של Vercel גישה למאגר GregoryDich או להפעיל את GitHub Pages</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>אחרי שלב 4</t>
+          <t>האתר בנוי ומתעדכן עם כל עמוד חדש; ממתין לגישה — שירותי האחסון החיצוניים חסומים מסביבת העבודה בענן</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>חשבון ותוכנית נאמנות: בחירת תחום → הדגשים אישיים; הרשמה (שם, email, טלפון, תפקיד); אימות סטטוס מקצועי עבור המוצרים המקצועיים; קוד קופון, 5% על הבאת חבר/ה, מדרגות עד 15%; הפרוטוקולים של המוצרים שנרכשו – בחשבון ובדוא״ל</t>
+          <t>דף הבית – דף בית אמיתי: מסך פתיחה כמו ב-Make ← כל המוצרים ב-3D מתכנסים ומתפזרים לפי סדרות ← בחירת תחום למעלה ← כל סדרה פעם אחת; לחיצה על סדרה פותחת את חלון הסדרה; «אודות» למטה; עמוד כל המוצרים</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -688,91 +688,118 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>כללי התוכנית (מדרגות, מועדים), מי מאמת/ת את הסטטוס</t>
+          <t>דוגמה למסך הפתיחה מ-Make</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>אחרי שלב 5</t>
+          <t>השלב הבא — אחרי העמוד של DERMA RECOVERY CREAM</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>אירועי האקדמיה בדף הבית וטופס להזמנת מקומות</t>
+          <t>חשבון ותוכנית נאמנות: בחירת תחום ← הדגשים אישיים; הרשמה (שם, email, טלפון, תפקיד); אימות סטטוס מקצועי עבור המוצרים המקצועיים; קוד קופון, 5% על הבאת חבר/ה, מדרגות עד 15%; הפרוטוקולים של המוצרים שנרכשו – בחשבון ובדוא״ל</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>3 שעות</t>
+          <t>1 יום</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>תאריכים, מחירים</t>
+          <t>כללי התוכנית (מדרגות, מועדים), מי מאמת/ת את הסטטוס</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>אחרי שלב 6</t>
+          <t>אחרי שלב 5</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>עמודי שירות: נגישות, פרטיות, תנאי שימוש, פאנל ניהול</t>
+          <t>אירועי האקדמיה בדף הבית וטופס להזמנת מקומות</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2 שעות</t>
+          <t>3 שעות</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>טקסטים משפטיים</t>
+          <t>תאריכים, מחירים</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>בסוף</t>
+          <t>אחרי שלב 6</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>עמודי שירות: נגישות, פרטיות, תנאי שימוש, פאנל ניהול</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2 שעות</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>טקסטים משפטיים</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>בסוף</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>התוצר הסופי – קישור אחד: מפת האתר עם כל העמודים ומסלולי המשתמש</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>2 שעות</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>בסוף, טיוטה – מוקדם יותר</t>
         </is>

</xml_diff>

<commit_message>
Roadmap: all 12 product pages published, home page is next
The two status cells were written while DERMA RECOVERY CREAM was still
in its review fixes; it has shipped since.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/MITODERM-3D-story.xlsx
+++ b/mitoderm-catalog/site/MITODERM-3D-story.xlsx
@@ -639,7 +639,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>23/10: פורסמו 11 מתוך 12 העמודים, והם נמצאים ב-site/public ‏(‏הקישורים ב-HANDOFF‏)‏; בעמוד DERMA RECOVERY CREAM נעשים התיקונים האחרונים אחרי הבדיקה; כשיגיעו הקבצים של BIOSPICULE, ההדפסה על צידי ארבע הקופסאות תתווסף לעמודים, באותם קישורים</t>
+          <t>23/10: כל 12 העמודים פורסמו, והם נמצאים ב-site/public ‏(‏הקישורים ב-HANDOFF‏)‏; כשיגיעו הקבצים של BIOSPICULE, ההדפסה על צידי ארבע הקופסאות תתווסף לעמודים, באותם קישורים</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>השלב הבא — אחרי העמוד של DERMA RECOVERY CREAM</t>
+          <t>השלב הבא</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roadmap: MASK approved; stage 10, the React version for Vercel
The owner approved the EXOCELL MASK page on 23/10 and asked for a React
version of the whole design, deployed on Vercel, once the design is done.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kxi7WWH4xGLi2AcFRd4q2
</commit_message>
<xml_diff>
--- a/mitoderm-catalog/site/MITODERM-3D-story.xlsx
+++ b/mitoderm-catalog/site/MITODERM-3D-story.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -526,12 +526,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>«אוקיי» על העמוד</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>19–21/10: בטלפון התנועה חלקה והחדות מלאה, כל התמונות ב-HD; העמוד פורסם ונמצא ב-site/public; ממתין ל«אוקיי»</t>
+          <t>23/10: התקבל ‏«‏אוקיי‏»‏ — הדוגמה אושרה; העמוד פורסם ונמצא ב-site/public</t>
         </is>
       </c>
     </row>
@@ -802,6 +802,33 @@
       <c r="E13" s="2" t="inlineStr">
         <is>
           <t>בסוף, טיוטה – מוקדם יותר</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>גרסת React ל-Vercel: כל העיצוב של האתר — כל העמודים, מנוע הפריימים וסצנות ה-three.js — כאפליקציית React עם פריסה ב-Vercel, כדי שהמתכנת והצוות ימשיכו מקוד מוכן</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2–3 ימים</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>גישה של Vercel למאגר GregoryDich ‏(‏אותה פעולה כמו בשלב 4א‏)‏</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>אחרי העיצוב של כל העמודים; הבסיס כבר קיים: המנוע ב-React ‏(‏proto/react: ה-hook‏ useFrameStory, ‏StoryPage ודמו‏)‏</t>
         </is>
       </c>
     </row>

</xml_diff>